<commit_message>
🤖 Daily job update — 2026-05-20
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49,7 +49,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +81,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -108,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -141,6 +146,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -508,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1286,8 +1303,1394 @@
       </c>
       <c r="M12" s="2" t="inlineStr"/>
     </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>4401686051</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Front End Software Engineer</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Saronic Technologies</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, react, node, aws, api, Location: Austin, TX, Title match: Front End Software Engineer</t>
+        </is>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M13" s="12" t="inlineStr"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>4309696652</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Rhode Island, United States</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, full stack, c++, Title match: Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M14" s="13" t="inlineStr"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>4309804319</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Colorado, United States</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, full stack, c++, Title match: Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L15" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M15" s="12" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>4410271532</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Associate Developer</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>HealthStream</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>Nashville, TN</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Very Low</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Skills: aws, api, c, ci/cd</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M16" s="13" t="inlineStr"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>4304445726</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Oregon, United States</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, c++, c, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M17" s="12" t="inlineStr"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>4342036151</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Modern Treasury</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Skills: react, aws, rest, api, git, full-stack, Title match: Software Engineer</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="inlineStr"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>4304441843</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Idaho, United States</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, c++, c, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>4408047047</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Computer Sciences - Graduates - AI Training - Las Vegas, US</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Prolific</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Las Vegas, NV</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>Very Low</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>Temporary</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Skills: aws, c, llm, algorithms</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M20" s="13" t="inlineStr"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>4304444837</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>New Jersey, United States</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, c++, c, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L21" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M21" s="12" t="inlineStr"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>4405641326</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Full-stack Engineer</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>PartnerTap</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Skills: javascript, react, rest, api, html, css, Location: Seattle, WA</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L22" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M22" s="13" t="inlineStr"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>4341020900</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>PlanIT Group, LLC</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>Contract</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, react, node, api, html, Title match: Software Engineer</t>
+        </is>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L23" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M23" s="12" t="inlineStr"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>4304450637</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>New York, United States</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, c++, c, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M24" s="13" t="inlineStr"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>4304451654</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Utah, United States</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, c++, c, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K25" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M25" s="12" t="inlineStr"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>4413745880</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Crate &amp; Barrel</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>Northbrook, IL</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, git, sql, c++, c, Title match: Software Engineer</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M26" s="13" t="inlineStr"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>4304438841</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Connecticut, United States</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, c++, c, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K27" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M27" s="12" t="inlineStr"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>4393215930</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>Transcend</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>California, United States</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Skills: react, node, aws, rest, api, sql, Title match: Software Engineer</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="inlineStr"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>4304445723</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>Illinois, United States</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, c++, c, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K29" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M29" s="12" t="inlineStr"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>4396380649</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Full-Stack Developer Intern, Music &amp; Audio</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Melotech</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Skills: node, api, full stack, full-stack, backend, frontend, Title match: Full-Stack Developer Intern, Music &amp; Audio</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L30" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M30" s="13" t="inlineStr"/>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>4304454025</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Washington, DC</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>72%</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J31" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, c++, c, Location: Washington, DC, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K31" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L31" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M31" s="12" t="inlineStr"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>4309802287</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>New Jersey, United States</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H32" s="13" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, full stack, c++, Title match: Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L32" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M32" s="13" t="inlineStr"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>4309694880</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>New York, United States</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, full stack, c++, Title match: Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K33" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L33" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M33" s="12" t="inlineStr"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>4411274012</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Junior UI Developer</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>General Dynamics Information Technology</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>Very Low</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Skills: react, git, c, agile</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L34" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M34" s="13" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M12"/>
+  <autoFilter ref="A1:M34"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -1300,6 +2703,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-05-21
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49,7 +49,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -86,6 +86,11 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCC99"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -113,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -158,6 +163,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -525,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -611,12 +628,12 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>4406952064</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -626,12 +643,12 @@
           <t>DevSecOps Intern</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="13" t="inlineStr">
         <is>
           <t>Modern Technology Solutions, Inc. (MTSI)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="13" t="inlineStr">
         <is>
           <t>Huntsville, AL</t>
         </is>
@@ -646,12 +663,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="13" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="13" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -666,20 +683,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="L2" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M2" s="13" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>4405630173</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -689,12 +706,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>DLRdmv®</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>Dallas, TX</t>
         </is>
@@ -709,12 +726,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="12" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="12" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -729,20 +746,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M3" s="7" t="inlineStr"/>
+      <c r="L3" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M3" s="12" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>4287414862</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -752,12 +769,12 @@
           <t>[Online Assessment]Software Development Engineer Intern (Network Automation)- 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>ByteDance</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -772,12 +789,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="13" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="13" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -792,20 +809,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M4" s="13" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>4309805269</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -815,12 +832,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Delaware, United States</t>
         </is>
@@ -835,12 +852,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>81</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="12" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -855,20 +872,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr"/>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M5" s="12" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>4371812987</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -878,12 +895,12 @@
           <t>Software Development Engineer Fall Intern - Military Veteran</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -898,12 +915,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="13" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -918,20 +935,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M6" s="13" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>4274682122</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -941,12 +958,12 @@
           <t>Software Engineer Intern (Data Ecosystem) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -961,12 +978,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="12" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -981,20 +998,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M7" s="7" t="inlineStr"/>
+      <c r="L7" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M7" s="12" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>4283848614</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1004,12 +1021,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Fall (BS/ MS)</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1024,12 +1041,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="13" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1044,20 +1061,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr"/>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>4411790844</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1067,12 +1084,12 @@
           <t>Software Engineer Intern (Infrastructure Automation) - Fall 2026</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Bellevue, WA</t>
         </is>
@@ -1087,12 +1104,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="12" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1107,20 +1124,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M9" s="7" t="inlineStr"/>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M9" s="12" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>4332425058</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1130,12 +1147,12 @@
           <t>Software Development Engineer Internship - Fall 2026 (US)</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1150,12 +1167,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="13" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="13" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1170,20 +1187,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M10" s="13" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>4323643644</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1193,12 +1210,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1213,12 +1230,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1233,20 +1250,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M11" s="7" t="inlineStr"/>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M11" s="12" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>4320849104</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1256,12 +1273,12 @@
           <t>Software Engineer Intern (Commerce Ads) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1276,12 +1293,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="13" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="13" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1296,12 +1313,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M12" s="13" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
@@ -2689,8 +2706,197 @@
       </c>
       <c r="M34" s="13" t="inlineStr"/>
     </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>4264562292</t>
+        </is>
+      </c>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Cymertek Corporation</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>San Antonio, TX</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="I35" s="16" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J35" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, aws, docker, git, sql, full stack, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L35" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M35" s="16" t="inlineStr"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>4417482675</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Software Developer I</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>El Paso Water</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>El Paso, TX</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H36" s="17" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="I36" s="17" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, rest, c, Title match: Software Developer I</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L36" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M36" s="17" t="inlineStr"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>4416508200</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Software Development Engineer in Test Intern (Global E-Commerce) - 2026 Summer (BS/MS)</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>68%</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="I37" s="16" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>Skills: aws, rest, api, c, express, agile, Location: Seattle, WA, Title match: Software Development Engineer in Test Intern (Global E-Commerce) - 2026 Summer (BS/MS)</t>
+        </is>
+      </c>
+      <c r="K37" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L37" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M37" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M34"/>
+  <autoFilter ref="A1:M37"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -2725,6 +2931,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-05-22
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -176,6 +176,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -542,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -628,12 +634,12 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>4406952064</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -643,12 +649,12 @@
           <t>DevSecOps Intern</t>
         </is>
       </c>
-      <c r="D2" s="13" t="inlineStr">
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>Modern Technology Solutions, Inc. (MTSI)</t>
         </is>
       </c>
-      <c r="E2" s="13" t="inlineStr">
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>Huntsville, AL</t>
         </is>
@@ -663,12 +669,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H2" s="13" t="inlineStr">
+      <c r="H2" s="17" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="I2" s="13" t="inlineStr">
+      <c r="I2" s="17" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -683,20 +689,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L2" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M2" s="13" t="inlineStr"/>
+      <c r="L2" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M2" s="17" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>4405630173</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -706,12 +712,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>DLRdmv®</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>Dallas, TX</t>
         </is>
@@ -726,12 +732,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H3" s="12" t="inlineStr">
+      <c r="H3" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I3" s="12" t="inlineStr">
+      <c r="I3" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -746,20 +752,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L3" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M3" s="12" t="inlineStr"/>
+      <c r="L3" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M3" s="16" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>4287414862</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -769,12 +775,12 @@
           <t>[Online Assessment]Software Development Engineer Intern (Network Automation)- 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>ByteDance</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -789,12 +795,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="13" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I4" s="13" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -809,20 +815,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L4" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M4" s="13" t="inlineStr"/>
+      <c r="L4" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M4" s="17" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>4309805269</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -832,12 +838,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Delaware, United States</t>
         </is>
@@ -852,12 +858,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>81</t>
         </is>
       </c>
-      <c r="I5" s="12" t="inlineStr">
+      <c r="I5" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -872,20 +878,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L5" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M5" s="12" t="inlineStr"/>
+      <c r="L5" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M5" s="16" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>4371812987</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -895,12 +901,12 @@
           <t>Software Development Engineer Fall Intern - Military Veteran</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -915,12 +921,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H6" s="13" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="I6" s="13" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -935,20 +941,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L6" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M6" s="13" t="inlineStr"/>
+      <c r="L6" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M6" s="17" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>4274682122</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -958,12 +964,12 @@
           <t>Software Engineer Intern (Data Ecosystem) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -978,12 +984,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I7" s="12" t="inlineStr">
+      <c r="I7" s="16" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -998,20 +1004,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L7" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M7" s="12" t="inlineStr"/>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M7" s="16" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>4283848614</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1021,12 +1027,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Fall (BS/ MS)</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1041,12 +1047,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H8" s="13" t="inlineStr">
+      <c r="H8" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I8" s="13" t="inlineStr">
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1061,20 +1067,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L8" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M8" s="13" t="inlineStr"/>
+      <c r="L8" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>4411790844</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1084,12 +1090,12 @@
           <t>Software Engineer Intern (Infrastructure Automation) - Fall 2026</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Bellevue, WA</t>
         </is>
@@ -1104,12 +1110,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H9" s="12" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I9" s="12" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1124,20 +1130,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L9" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M9" s="12" t="inlineStr"/>
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M9" s="16" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>4332425058</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1147,12 +1153,12 @@
           <t>Software Development Engineer Internship - Fall 2026 (US)</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1167,12 +1173,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H10" s="13" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I10" s="13" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1187,20 +1193,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L10" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M10" s="13" t="inlineStr"/>
+      <c r="L10" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M10" s="17" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>4323643644</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1210,12 +1216,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1230,12 +1236,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I11" s="12" t="inlineStr">
+      <c r="I11" s="16" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1250,20 +1256,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L11" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M11" s="12" t="inlineStr"/>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M11" s="16" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>4320849104</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1273,12 +1279,12 @@
           <t>Software Engineer Intern (Commerce Ads) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1293,12 +1299,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H12" s="13" t="inlineStr">
+      <c r="H12" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I12" s="13" t="inlineStr">
+      <c r="I12" s="17" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1313,20 +1319,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L12" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M12" s="13" t="inlineStr"/>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>4401686051</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1336,12 +1342,12 @@
           <t>Front End Software Engineer</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Saronic Technologies</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
@@ -1356,12 +1362,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H13" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I13" s="12" t="inlineStr">
+      <c r="I13" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1376,20 +1382,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L13" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M13" s="12" t="inlineStr"/>
+      <c r="L13" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M13" s="16" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>4309696652</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1399,12 +1405,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>Rhode Island, United States</t>
         </is>
@@ -1419,12 +1425,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H14" s="13" t="inlineStr">
+      <c r="H14" s="17" t="inlineStr">
         <is>
           <t>114</t>
         </is>
       </c>
-      <c r="I14" s="13" t="inlineStr">
+      <c r="I14" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1439,20 +1445,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L14" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M14" s="13" t="inlineStr"/>
+      <c r="L14" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>4309804319</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1462,12 +1468,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>Colorado, United States</t>
         </is>
@@ -1482,12 +1488,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="I15" s="12" t="inlineStr">
+      <c r="I15" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1502,20 +1508,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L15" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M15" s="12" t="inlineStr"/>
+      <c r="L15" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M15" s="16" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>4410271532</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1525,12 +1531,12 @@
           <t>Associate Developer</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>HealthStream</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E16" s="17" t="inlineStr">
         <is>
           <t>Nashville, TN</t>
         </is>
@@ -1545,12 +1551,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H16" s="13" t="inlineStr">
+      <c r="H16" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I16" s="13" t="inlineStr">
+      <c r="I16" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1565,20 +1571,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L16" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M16" s="13" t="inlineStr"/>
+      <c r="L16" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M16" s="17" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>4304445726</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1588,12 +1594,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>Oregon, United States</t>
         </is>
@@ -1608,12 +1614,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>115</t>
         </is>
       </c>
-      <c r="I17" s="12" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1628,20 +1634,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L17" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M17" s="12" t="inlineStr"/>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M17" s="16" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>4342036151</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1651,12 +1657,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>Modern Treasury</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -1671,12 +1677,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H18" s="13" t="inlineStr">
+      <c r="H18" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I18" s="13" t="inlineStr">
+      <c r="I18" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1691,20 +1697,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L18" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M18" s="13" t="inlineStr"/>
+      <c r="L18" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>4304441843</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1714,12 +1720,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr">
         <is>
           <t>Idaho, United States</t>
         </is>
@@ -1734,12 +1740,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H19" s="12" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>157</t>
         </is>
       </c>
-      <c r="I19" s="12" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1754,20 +1760,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L19" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M19" s="12" t="inlineStr"/>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M19" s="16" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>4408047047</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1777,12 +1783,12 @@
           <t>Computer Sciences - Graduates - AI Training - Las Vegas, US</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>Prolific</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>Las Vegas, NV</t>
         </is>
@@ -1797,12 +1803,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H20" s="13" t="inlineStr">
+      <c r="H20" s="17" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="I20" s="13" t="inlineStr">
+      <c r="I20" s="17" t="inlineStr">
         <is>
           <t>Temporary</t>
         </is>
@@ -1817,20 +1823,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L20" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M20" s="13" t="inlineStr"/>
+      <c r="L20" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>4304444837</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1840,12 +1846,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -1860,12 +1866,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H21" s="12" t="inlineStr">
+      <c r="H21" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I21" s="12" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1880,20 +1886,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L21" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M21" s="12" t="inlineStr"/>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M21" s="16" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>4405641326</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1903,12 +1909,12 @@
           <t>Full-stack Engineer</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>PartnerTap</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="E22" s="17" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1923,12 +1929,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H22" s="13" t="inlineStr">
+      <c r="H22" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr">
+      <c r="I22" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1943,20 +1949,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L22" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M22" s="13" t="inlineStr"/>
+      <c r="L22" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>4341020900</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1966,12 +1972,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>PlanIT Group, LLC</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -1986,12 +1992,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H23" s="12" t="inlineStr">
+      <c r="H23" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I23" s="12" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
@@ -2006,20 +2012,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L23" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M23" s="12" t="inlineStr"/>
+      <c r="L23" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M23" s="16" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>4304450637</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2029,12 +2035,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2049,12 +2055,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H24" s="13" t="inlineStr">
+      <c r="H24" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I24" s="13" t="inlineStr">
+      <c r="I24" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2069,20 +2075,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L24" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M24" s="13" t="inlineStr"/>
+      <c r="L24" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M24" s="17" t="inlineStr"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>4304451654</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2092,12 +2098,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E25" s="16" t="inlineStr">
         <is>
           <t>Utah, United States</t>
         </is>
@@ -2112,12 +2118,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H25" s="12" t="inlineStr">
+      <c r="H25" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I25" s="12" t="inlineStr">
+      <c r="I25" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2132,20 +2138,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L25" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M25" s="12" t="inlineStr"/>
+      <c r="L25" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M25" s="16" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>4413745880</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2155,12 +2161,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>Crate &amp; Barrel</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E26" s="17" t="inlineStr">
         <is>
           <t>Northbrook, IL</t>
         </is>
@@ -2175,12 +2181,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H26" s="13" t="inlineStr">
+      <c r="H26" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I26" s="13" t="inlineStr">
+      <c r="I26" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2195,20 +2201,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L26" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M26" s="13" t="inlineStr"/>
+      <c r="L26" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M26" s="17" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>4304438841</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2218,12 +2224,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>Connecticut, United States</t>
         </is>
@@ -2238,12 +2244,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H27" s="12" t="inlineStr">
+      <c r="H27" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I27" s="12" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2258,20 +2264,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L27" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M27" s="12" t="inlineStr"/>
+      <c r="L27" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M27" s="16" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>4393215930</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2281,12 +2287,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>Transcend</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>California, United States</t>
         </is>
@@ -2301,12 +2307,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H28" s="13" t="inlineStr">
+      <c r="H28" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I28" s="13" t="inlineStr">
+      <c r="I28" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2321,20 +2327,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L28" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M28" s="13" t="inlineStr"/>
+      <c r="L28" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M28" s="17" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>4304445723</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2344,12 +2350,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D29" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>Illinois, United States</t>
         </is>
@@ -2364,12 +2370,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H29" s="12" t="inlineStr">
+      <c r="H29" s="16" t="inlineStr">
         <is>
           <t>198</t>
         </is>
       </c>
-      <c r="I29" s="12" t="inlineStr">
+      <c r="I29" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2384,20 +2390,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L29" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M29" s="12" t="inlineStr"/>
+      <c r="L29" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M29" s="16" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>4396380649</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2407,12 +2413,12 @@
           <t>Full-Stack Developer Intern, Music &amp; Audio</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>Melotech</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
+      <c r="E30" s="17" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -2427,12 +2433,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H30" s="13" t="inlineStr">
+      <c r="H30" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I30" s="13" t="inlineStr">
+      <c r="I30" s="17" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -2447,20 +2453,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L30" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M30" s="13" t="inlineStr"/>
+      <c r="L30" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M30" s="17" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>4304454025</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2470,12 +2476,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="E31" s="16" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -2490,12 +2496,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H31" s="12" t="inlineStr">
+      <c r="H31" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I31" s="12" t="inlineStr">
+      <c r="I31" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2510,20 +2516,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L31" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M31" s="12" t="inlineStr"/>
+      <c r="L31" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M31" s="16" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>4309802287</t>
         </is>
       </c>
-      <c r="B32" s="13" t="inlineStr">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2533,12 +2539,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D32" s="13" t="inlineStr">
+      <c r="D32" s="17" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="E32" s="17" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -2553,12 +2559,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H32" s="13" t="inlineStr">
+      <c r="H32" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I32" s="13" t="inlineStr">
+      <c r="I32" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2573,20 +2579,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L32" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M32" s="13" t="inlineStr"/>
+      <c r="L32" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M32" s="17" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="12" t="inlineStr">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>4309694880</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2596,12 +2602,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D33" s="16" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E33" s="12" t="inlineStr">
+      <c r="E33" s="16" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2616,12 +2622,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H33" s="12" t="inlineStr">
+      <c r="H33" s="16" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I33" s="12" t="inlineStr">
+      <c r="I33" s="16" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2636,20 +2642,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L33" s="12" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M33" s="12" t="inlineStr"/>
+      <c r="L33" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M33" s="16" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>4411274012</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2659,12 +2665,12 @@
           <t>Junior UI Developer</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D34" s="17" t="inlineStr">
         <is>
           <t>General Dynamics Information Technology</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr">
+      <c r="E34" s="17" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -2679,12 +2685,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H34" s="13" t="inlineStr">
+      <c r="H34" s="17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I34" s="13" t="inlineStr">
+      <c r="I34" s="17" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2699,12 +2705,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L34" s="13" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M34" s="13" t="inlineStr"/>
+      <c r="L34" s="17" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M34" s="17" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="16" t="inlineStr">
@@ -2895,8 +2901,134 @@
       </c>
       <c r="M37" s="16" t="inlineStr"/>
     </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>4309809191</t>
+        </is>
+      </c>
+      <c r="B38" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D38" s="20" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E38" s="20" t="inlineStr">
+        <is>
+          <t>Ohio, United States</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H38" s="20" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="I38" s="20" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, full stack, c++, Title match: Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L38" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M38" s="20" t="inlineStr"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>3986118096</t>
+        </is>
+      </c>
+      <c r="B39" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="E39" s="21" t="inlineStr">
+        <is>
+          <t>Irving, TX</t>
+        </is>
+      </c>
+      <c r="F39" s="18" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="G39" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H39" s="21" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I39" s="21" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J39" s="8" t="inlineStr">
+        <is>
+          <t>Skills: rest, api, machine learning, c, Title match: Software Engineer</t>
+        </is>
+      </c>
+      <c r="K39" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L39" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M39" s="21" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M37"/>
+  <autoFilter ref="A1:M39"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -2934,6 +3066,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-05-25
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -176,6 +176,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -548,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -634,12 +640,12 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>4406952064</t>
         </is>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -649,12 +655,12 @@
           <t>DevSecOps Intern</t>
         </is>
       </c>
-      <c r="D2" s="17" t="inlineStr">
+      <c r="D2" s="20" t="inlineStr">
         <is>
           <t>Modern Technology Solutions, Inc. (MTSI)</t>
         </is>
       </c>
-      <c r="E2" s="17" t="inlineStr">
+      <c r="E2" s="20" t="inlineStr">
         <is>
           <t>Huntsville, AL</t>
         </is>
@@ -669,12 +675,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H2" s="17" t="inlineStr">
+      <c r="H2" s="20" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="I2" s="17" t="inlineStr">
+      <c r="I2" s="20" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -689,20 +695,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L2" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M2" s="17" t="inlineStr"/>
+      <c r="L2" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M2" s="20" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>4405630173</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -712,12 +718,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>DLRdmv®</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>Dallas, TX</t>
         </is>
@@ -732,12 +738,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H3" s="16" t="inlineStr">
+      <c r="H3" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I3" s="16" t="inlineStr">
+      <c r="I3" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -752,20 +758,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L3" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M3" s="16" t="inlineStr"/>
+      <c r="L3" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M3" s="21" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>4287414862</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -775,12 +781,12 @@
           <t>[Online Assessment]Software Development Engineer Intern (Network Automation)- 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>ByteDance</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -795,12 +801,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H4" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I4" s="17" t="inlineStr">
+      <c r="I4" s="20" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -815,20 +821,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L4" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M4" s="17" t="inlineStr"/>
+      <c r="L4" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M4" s="20" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>4309805269</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -838,12 +844,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>Delaware, United States</t>
         </is>
@@ -858,12 +864,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" s="16" t="inlineStr">
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>81</t>
         </is>
       </c>
-      <c r="I5" s="16" t="inlineStr">
+      <c r="I5" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -878,20 +884,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L5" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M5" s="16" t="inlineStr"/>
+      <c r="L5" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M5" s="21" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>4371812987</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -901,12 +907,12 @@
           <t>Software Development Engineer Fall Intern - Military Veteran</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -921,12 +927,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H6" s="17" t="inlineStr">
+      <c r="H6" s="20" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="I6" s="17" t="inlineStr">
+      <c r="I6" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -941,20 +947,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L6" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M6" s="17" t="inlineStr"/>
+      <c r="L6" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M6" s="20" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>4274682122</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -964,12 +970,12 @@
           <t>Software Engineer Intern (Data Ecosystem) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -984,12 +990,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I7" s="16" t="inlineStr">
+      <c r="I7" s="21" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1004,20 +1010,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L7" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M7" s="16" t="inlineStr"/>
+      <c r="L7" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M7" s="21" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>4283848614</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1027,12 +1033,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Fall (BS/ MS)</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1047,12 +1053,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="H8" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I8" s="17" t="inlineStr">
+      <c r="I8" s="20" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1067,20 +1073,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L8" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M8" s="17" t="inlineStr"/>
+      <c r="L8" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M8" s="20" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>4411790844</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1090,12 +1096,12 @@
           <t>Software Engineer Intern (Infrastructure Automation) - Fall 2026</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>Bellevue, WA</t>
         </is>
@@ -1110,12 +1116,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H9" s="16" t="inlineStr">
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I9" s="16" t="inlineStr">
+      <c r="I9" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1130,20 +1136,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L9" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M9" s="16" t="inlineStr"/>
+      <c r="L9" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M9" s="21" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>4332425058</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1153,12 +1159,12 @@
           <t>Software Development Engineer Internship - Fall 2026 (US)</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1173,12 +1179,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="H10" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I10" s="17" t="inlineStr">
+      <c r="I10" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1193,20 +1199,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L10" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M10" s="17" t="inlineStr"/>
+      <c r="L10" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M10" s="20" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>4323643644</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1216,12 +1222,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1236,12 +1242,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H11" s="16" t="inlineStr">
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I11" s="16" t="inlineStr">
+      <c r="I11" s="21" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1256,20 +1262,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L11" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M11" s="16" t="inlineStr"/>
+      <c r="L11" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M11" s="21" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>4320849104</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1279,12 +1285,12 @@
           <t>Software Engineer Intern (Commerce Ads) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr">
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1299,12 +1305,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="H12" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I12" s="17" t="inlineStr">
+      <c r="I12" s="20" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1319,20 +1325,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L12" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M12" s="17" t="inlineStr"/>
+      <c r="L12" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M12" s="20" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>4401686051</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1342,12 +1348,12 @@
           <t>Front End Software Engineer</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>Saronic Technologies</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
@@ -1362,12 +1368,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H13" s="16" t="inlineStr">
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I13" s="16" t="inlineStr">
+      <c r="I13" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1382,20 +1388,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L13" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M13" s="16" t="inlineStr"/>
+      <c r="L13" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M13" s="21" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>4309696652</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1405,12 +1411,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>Rhode Island, United States</t>
         </is>
@@ -1425,12 +1431,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H14" s="17" t="inlineStr">
+      <c r="H14" s="20" t="inlineStr">
         <is>
           <t>114</t>
         </is>
       </c>
-      <c r="I14" s="17" t="inlineStr">
+      <c r="I14" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1445,20 +1451,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L14" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M14" s="17" t="inlineStr"/>
+      <c r="L14" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M14" s="20" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>4309804319</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1468,12 +1474,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>Colorado, United States</t>
         </is>
@@ -1488,12 +1494,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H15" s="16" t="inlineStr">
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="I15" s="16" t="inlineStr">
+      <c r="I15" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1508,20 +1514,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L15" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M15" s="16" t="inlineStr"/>
+      <c r="L15" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M15" s="21" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>4410271532</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1531,12 +1537,12 @@
           <t>Associate Developer</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>HealthStream</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr">
+      <c r="E16" s="20" t="inlineStr">
         <is>
           <t>Nashville, TN</t>
         </is>
@@ -1551,12 +1557,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H16" s="17" t="inlineStr">
+      <c r="H16" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I16" s="17" t="inlineStr">
+      <c r="I16" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1571,20 +1577,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L16" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M16" s="17" t="inlineStr"/>
+      <c r="L16" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M16" s="20" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>4304445726</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1594,12 +1600,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>Oregon, United States</t>
         </is>
@@ -1614,12 +1620,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H17" s="16" t="inlineStr">
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>115</t>
         </is>
       </c>
-      <c r="I17" s="16" t="inlineStr">
+      <c r="I17" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1634,20 +1640,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L17" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M17" s="16" t="inlineStr"/>
+      <c r="L17" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M17" s="21" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>4342036151</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1657,12 +1663,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>Modern Treasury</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -1677,12 +1683,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H18" s="17" t="inlineStr">
+      <c r="H18" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I18" s="17" t="inlineStr">
+      <c r="I18" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1697,20 +1703,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L18" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M18" s="17" t="inlineStr"/>
+      <c r="L18" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M18" s="20" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>4304441843</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1720,12 +1726,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>Idaho, United States</t>
         </is>
@@ -1740,12 +1746,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H19" s="16" t="inlineStr">
+      <c r="H19" s="21" t="inlineStr">
         <is>
           <t>157</t>
         </is>
       </c>
-      <c r="I19" s="16" t="inlineStr">
+      <c r="I19" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1760,20 +1766,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L19" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M19" s="16" t="inlineStr"/>
+      <c r="L19" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M19" s="21" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>4408047047</t>
         </is>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1783,12 +1789,12 @@
           <t>Computer Sciences - Graduates - AI Training - Las Vegas, US</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>Prolific</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="E20" s="20" t="inlineStr">
         <is>
           <t>Las Vegas, NV</t>
         </is>
@@ -1803,12 +1809,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H20" s="17" t="inlineStr">
+      <c r="H20" s="20" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="I20" s="17" t="inlineStr">
+      <c r="I20" s="20" t="inlineStr">
         <is>
           <t>Temporary</t>
         </is>
@@ -1823,20 +1829,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L20" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M20" s="17" t="inlineStr"/>
+      <c r="L20" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M20" s="20" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>4304444837</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1846,12 +1852,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -1866,12 +1872,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H21" s="16" t="inlineStr">
+      <c r="H21" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I21" s="16" t="inlineStr">
+      <c r="I21" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1886,20 +1892,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L21" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M21" s="16" t="inlineStr"/>
+      <c r="L21" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M21" s="21" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>4405641326</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1909,12 +1915,12 @@
           <t>Full-stack Engineer</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>PartnerTap</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1929,12 +1935,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
+      <c r="H22" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I22" s="17" t="inlineStr">
+      <c r="I22" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1949,20 +1955,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L22" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M22" s="17" t="inlineStr"/>
+      <c r="L22" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M22" s="20" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>4341020900</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1972,12 +1978,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>PlanIT Group, LLC</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -1992,12 +1998,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H23" s="16" t="inlineStr">
+      <c r="H23" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I23" s="16" t="inlineStr">
+      <c r="I23" s="21" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
@@ -2012,20 +2018,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L23" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M23" s="16" t="inlineStr"/>
+      <c r="L23" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M23" s="21" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>4304450637</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2035,12 +2041,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr">
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2055,12 +2061,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H24" s="17" t="inlineStr">
+      <c r="H24" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I24" s="17" t="inlineStr">
+      <c r="I24" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2075,20 +2081,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L24" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M24" s="17" t="inlineStr"/>
+      <c r="L24" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M24" s="20" t="inlineStr"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>4304451654</t>
         </is>
       </c>
-      <c r="B25" s="16" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2098,12 +2104,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>Utah, United States</t>
         </is>
@@ -2118,12 +2124,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H25" s="16" t="inlineStr">
+      <c r="H25" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I25" s="16" t="inlineStr">
+      <c r="I25" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2138,20 +2144,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L25" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M25" s="16" t="inlineStr"/>
+      <c r="L25" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M25" s="21" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>4413745880</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2161,12 +2167,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>Crate &amp; Barrel</t>
         </is>
       </c>
-      <c r="E26" s="17" t="inlineStr">
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>Northbrook, IL</t>
         </is>
@@ -2181,12 +2187,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H26" s="17" t="inlineStr">
+      <c r="H26" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I26" s="17" t="inlineStr">
+      <c r="I26" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2201,20 +2207,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L26" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M26" s="17" t="inlineStr"/>
+      <c r="L26" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M26" s="20" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>4304438841</t>
         </is>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2224,12 +2230,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D27" s="16" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>Connecticut, United States</t>
         </is>
@@ -2244,12 +2250,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H27" s="16" t="inlineStr">
+      <c r="H27" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I27" s="16" t="inlineStr">
+      <c r="I27" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2264,20 +2270,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L27" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M27" s="16" t="inlineStr"/>
+      <c r="L27" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M27" s="21" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>4393215930</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2287,12 +2293,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>Transcend</t>
         </is>
       </c>
-      <c r="E28" s="17" t="inlineStr">
+      <c r="E28" s="20" t="inlineStr">
         <is>
           <t>California, United States</t>
         </is>
@@ -2307,12 +2313,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H28" s="17" t="inlineStr">
+      <c r="H28" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I28" s="17" t="inlineStr">
+      <c r="I28" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2327,20 +2333,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L28" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M28" s="17" t="inlineStr"/>
+      <c r="L28" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M28" s="20" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>4304445723</t>
         </is>
       </c>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2350,12 +2356,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>Illinois, United States</t>
         </is>
@@ -2370,12 +2376,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H29" s="16" t="inlineStr">
+      <c r="H29" s="21" t="inlineStr">
         <is>
           <t>198</t>
         </is>
       </c>
-      <c r="I29" s="16" t="inlineStr">
+      <c r="I29" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2390,20 +2396,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L29" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M29" s="16" t="inlineStr"/>
+      <c r="L29" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M29" s="21" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="17" t="inlineStr">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>4396380649</t>
         </is>
       </c>
-      <c r="B30" s="17" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2413,12 +2419,12 @@
           <t>Full-Stack Developer Intern, Music &amp; Audio</t>
         </is>
       </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>Melotech</t>
         </is>
       </c>
-      <c r="E30" s="17" t="inlineStr">
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -2433,12 +2439,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H30" s="17" t="inlineStr">
+      <c r="H30" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I30" s="17" t="inlineStr">
+      <c r="I30" s="20" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -2453,20 +2459,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L30" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M30" s="17" t="inlineStr"/>
+      <c r="L30" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M30" s="20" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>4304454025</t>
         </is>
       </c>
-      <c r="B31" s="16" t="inlineStr">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2476,12 +2482,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D31" s="16" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -2496,12 +2502,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H31" s="16" t="inlineStr">
+      <c r="H31" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I31" s="16" t="inlineStr">
+      <c r="I31" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2516,20 +2522,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L31" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M31" s="16" t="inlineStr"/>
+      <c r="L31" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M31" s="21" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>4309802287</t>
         </is>
       </c>
-      <c r="B32" s="17" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2539,12 +2545,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D32" s="17" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E32" s="17" t="inlineStr">
+      <c r="E32" s="20" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -2559,12 +2565,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H32" s="17" t="inlineStr">
+      <c r="H32" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I32" s="17" t="inlineStr">
+      <c r="I32" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2579,20 +2585,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L32" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M32" s="17" t="inlineStr"/>
+      <c r="L32" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M32" s="20" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="21" t="inlineStr">
         <is>
           <t>4309694880</t>
         </is>
       </c>
-      <c r="B33" s="16" t="inlineStr">
+      <c r="B33" s="21" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2602,12 +2608,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D33" s="16" t="inlineStr">
+      <c r="D33" s="21" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr">
+      <c r="E33" s="21" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2622,12 +2628,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H33" s="16" t="inlineStr">
+      <c r="H33" s="21" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I33" s="16" t="inlineStr">
+      <c r="I33" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2642,20 +2648,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L33" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M33" s="16" t="inlineStr"/>
+      <c r="L33" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M33" s="21" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="17" t="inlineStr">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>4411274012</t>
         </is>
       </c>
-      <c r="B34" s="17" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2665,12 +2671,12 @@
           <t>Junior UI Developer</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>General Dynamics Information Technology</t>
         </is>
       </c>
-      <c r="E34" s="17" t="inlineStr">
+      <c r="E34" s="20" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -2685,12 +2691,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H34" s="17" t="inlineStr">
+      <c r="H34" s="20" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I34" s="17" t="inlineStr">
+      <c r="I34" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2705,20 +2711,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L34" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M34" s="17" t="inlineStr"/>
+      <c r="L34" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M34" s="20" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t>4264562292</t>
         </is>
       </c>
-      <c r="B35" s="16" t="inlineStr">
+      <c r="B35" s="21" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2728,12 +2734,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>Cymertek Corporation</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
+      <c r="E35" s="21" t="inlineStr">
         <is>
           <t>San Antonio, TX</t>
         </is>
@@ -2748,12 +2754,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H35" s="16" t="inlineStr">
+      <c r="H35" s="21" t="inlineStr">
         <is>
           <t>155</t>
         </is>
       </c>
-      <c r="I35" s="16" t="inlineStr">
+      <c r="I35" s="21" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2768,20 +2774,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L35" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M35" s="16" t="inlineStr"/>
+      <c r="L35" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M35" s="21" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="17" t="inlineStr">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>4417482675</t>
         </is>
       </c>
-      <c r="B36" s="17" t="inlineStr">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2791,12 +2797,12 @@
           <t>Software Developer I</t>
         </is>
       </c>
-      <c r="D36" s="17" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>El Paso Water</t>
         </is>
       </c>
-      <c r="E36" s="17" t="inlineStr">
+      <c r="E36" s="20" t="inlineStr">
         <is>
           <t>El Paso, TX</t>
         </is>
@@ -2811,12 +2817,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H36" s="17" t="inlineStr">
+      <c r="H36" s="20" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="I36" s="17" t="inlineStr">
+      <c r="I36" s="20" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2831,20 +2837,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L36" s="17" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M36" s="17" t="inlineStr"/>
+      <c r="L36" s="20" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M36" s="20" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t>4416508200</t>
         </is>
       </c>
-      <c r="B37" s="16" t="inlineStr">
+      <c r="B37" s="21" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2854,12 +2860,12 @@
           <t>Software Development Engineer in Test Intern (Global E-Commerce) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D37" s="16" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E37" s="16" t="inlineStr">
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -2874,12 +2880,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H37" s="16" t="inlineStr">
+      <c r="H37" s="21" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="I37" s="16" t="inlineStr">
+      <c r="I37" s="21" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -2894,12 +2900,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L37" s="16" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M37" s="16" t="inlineStr"/>
+      <c r="L37" s="21" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M37" s="21" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
@@ -3027,8 +3033,638 @@
       </c>
       <c r="M39" s="21" t="inlineStr"/>
     </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>4309808244</t>
+        </is>
+      </c>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E40" s="22" t="inlineStr">
+        <is>
+          <t>Massachusetts, United States</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H40" s="22" t="inlineStr">
+        <is>
+          <t>166</t>
+        </is>
+      </c>
+      <c r="I40" s="22" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, full stack, c++, Title match: Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L40" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M40" s="22" t="inlineStr"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>4362173625</t>
+        </is>
+      </c>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="D41" s="23" t="inlineStr">
+        <is>
+          <t>Empower Sleep</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H41" s="23" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I41" s="23" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>Skills: react, aws, api, git, full stack, backend, Title match: Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="K41" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L41" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M41" s="23" t="inlineStr"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>4309812093</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D42" s="22" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E42" s="22" t="inlineStr">
+        <is>
+          <t>Florida, United States</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H42" s="22" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="I42" s="22" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, full stack, c++, Title match: Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L42" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M42" s="22" t="inlineStr"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="23" t="inlineStr">
+        <is>
+          <t>4391759914</t>
+        </is>
+      </c>
+      <c r="B43" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>QA Engineering Internship</t>
+        </is>
+      </c>
+      <c r="D43" s="23" t="inlineStr">
+        <is>
+          <t>Chartbeat</t>
+        </is>
+      </c>
+      <c r="E43" s="23" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
+      </c>
+      <c r="G43" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H43" s="23" t="inlineStr">
+        <is>
+          <t>168</t>
+        </is>
+      </c>
+      <c r="I43" s="23" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J43" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, react, rest, api, git, Location: Austin, TX, Title match: QA Engineering Internship</t>
+        </is>
+      </c>
+      <c r="K43" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L43" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M43" s="23" t="inlineStr"/>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>4412855678</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>AI Integration Engineer</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>UST</t>
+        </is>
+      </c>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>Santa Clara, CA</t>
+        </is>
+      </c>
+      <c r="F44" s="18" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="G44" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H44" s="22" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I44" s="22" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, aws, rest, api, git, sql</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L44" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M44" s="22" t="inlineStr"/>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="23" t="inlineStr">
+        <is>
+          <t>4309805219</t>
+        </is>
+      </c>
+      <c r="B45" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D45" s="23" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E45" s="23" t="inlineStr">
+        <is>
+          <t>Washington, DC</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>76%</t>
+        </is>
+      </c>
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H45" s="23" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I45" s="23" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J45" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, full stack, c++, Location: Washington, DC, Title match: Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K45" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L45" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M45" s="23" t="inlineStr"/>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>4409726429</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Data Science Intern</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>Rundoo</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F46" s="18" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="G46" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H46" s="22" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I46" s="22" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, api, git, c, Title match: Data Science Intern</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L46" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M46" s="22" t="inlineStr"/>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t>4305671729</t>
+        </is>
+      </c>
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>DoD SkillBridge Internship/Fellowship Opportunity Application (U.S. Military Only)</t>
+        </is>
+      </c>
+      <c r="D47" s="23" t="inlineStr">
+        <is>
+          <t>Onsights</t>
+        </is>
+      </c>
+      <c r="E47" s="23" t="inlineStr">
+        <is>
+          <t>Washington, DC</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>68%</t>
+        </is>
+      </c>
+      <c r="G47" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H47" s="23" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="I47" s="23" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J47" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, react, sql, machine learning, c++, c, Location: Washington, DC, Title match: DoD SkillBridge Internship/Fellowship Opportunity Application (U.S. Military Only)</t>
+        </is>
+      </c>
+      <c r="K47" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L47" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M47" s="23" t="inlineStr"/>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t>4414096220</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Visualization Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D48" s="22" t="inlineStr">
+        <is>
+          <t>Leidos</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H48" s="22" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="I48" s="22" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, aws, rest, api, git, c++, Title match: Visualization Engineer Intern</t>
+        </is>
+      </c>
+      <c r="K48" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L48" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M48" s="22" t="inlineStr"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="23" t="inlineStr">
+        <is>
+          <t>4361076044</t>
+        </is>
+      </c>
+      <c r="B49" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>GenAI Engineering Intern  - SkillBridge (Remote)</t>
+        </is>
+      </c>
+      <c r="D49" s="23" t="inlineStr">
+        <is>
+          <t>CrowdStrike</t>
+        </is>
+      </c>
+      <c r="E49" s="23" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>48%</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H49" s="23" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I49" s="23" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J49" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, aws, rest, api, full stack, c, Title match: GenAI Engineering Intern  - SkillBridge (Remote)</t>
+        </is>
+      </c>
+      <c r="K49" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L49" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M49" s="23" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M39"/>
+  <autoFilter ref="A1:M49"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -3068,6 +3704,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-05-26
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -176,6 +176,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -554,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -640,12 +646,12 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>4406952064</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -655,12 +661,12 @@
           <t>DevSecOps Intern</t>
         </is>
       </c>
-      <c r="D2" s="20" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>Modern Technology Solutions, Inc. (MTSI)</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>Huntsville, AL</t>
         </is>
@@ -675,12 +681,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H2" s="20" t="inlineStr">
+      <c r="H2" s="22" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="I2" s="20" t="inlineStr">
+      <c r="I2" s="22" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -695,20 +701,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L2" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M2" s="20" t="inlineStr"/>
+      <c r="L2" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M2" s="22" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>4405630173</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -718,12 +724,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D3" s="21" t="inlineStr">
+      <c r="D3" s="23" t="inlineStr">
         <is>
           <t>DLRdmv®</t>
         </is>
       </c>
-      <c r="E3" s="21" t="inlineStr">
+      <c r="E3" s="23" t="inlineStr">
         <is>
           <t>Dallas, TX</t>
         </is>
@@ -738,12 +744,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H3" s="21" t="inlineStr">
+      <c r="H3" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I3" s="21" t="inlineStr">
+      <c r="I3" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -758,20 +764,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L3" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M3" s="21" t="inlineStr"/>
+      <c r="L3" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M3" s="23" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>4287414862</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -781,12 +787,12 @@
           <t>[Online Assessment]Software Development Engineer Intern (Network Automation)- 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>ByteDance</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -801,12 +807,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="20" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I4" s="20" t="inlineStr">
+      <c r="I4" s="22" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -821,20 +827,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L4" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M4" s="20" t="inlineStr"/>
+      <c r="L4" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M4" s="22" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>4309805269</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -844,12 +850,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="23" t="inlineStr">
         <is>
           <t>Delaware, United States</t>
         </is>
@@ -864,12 +870,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" s="21" t="inlineStr">
+      <c r="H5" s="23" t="inlineStr">
         <is>
           <t>81</t>
         </is>
       </c>
-      <c r="I5" s="21" t="inlineStr">
+      <c r="I5" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -884,20 +890,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L5" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M5" s="21" t="inlineStr"/>
+      <c r="L5" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M5" s="23" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>4371812987</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -907,12 +913,12 @@
           <t>Software Development Engineer Fall Intern - Military Veteran</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -927,12 +933,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H6" s="20" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr">
+      <c r="I6" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -947,20 +953,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L6" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M6" s="20" t="inlineStr"/>
+      <c r="L6" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M6" s="22" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>4274682122</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -970,12 +976,12 @@
           <t>Software Engineer Intern (Data Ecosystem) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D7" s="21" t="inlineStr">
+      <c r="D7" s="23" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E7" s="21" t="inlineStr">
+      <c r="E7" s="23" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -990,12 +996,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="21" t="inlineStr">
+      <c r="H7" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I7" s="21" t="inlineStr">
+      <c r="I7" s="23" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1010,20 +1016,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L7" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M7" s="21" t="inlineStr"/>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M7" s="23" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>4283848614</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1033,12 +1039,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Fall (BS/ MS)</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1053,12 +1059,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H8" s="20" t="inlineStr">
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I8" s="20" t="inlineStr">
+      <c r="I8" s="22" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1073,20 +1079,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L8" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M8" s="20" t="inlineStr"/>
+      <c r="L8" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M8" s="22" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>4411790844</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1096,12 +1102,12 @@
           <t>Software Engineer Intern (Infrastructure Automation) - Fall 2026</t>
         </is>
       </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="D9" s="23" t="inlineStr">
         <is>
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E9" s="21" t="inlineStr">
+      <c r="E9" s="23" t="inlineStr">
         <is>
           <t>Bellevue, WA</t>
         </is>
@@ -1116,12 +1122,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H9" s="21" t="inlineStr">
+      <c r="H9" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I9" s="21" t="inlineStr">
+      <c r="I9" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1136,20 +1142,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L9" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M9" s="21" t="inlineStr"/>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M9" s="23" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>4332425058</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1159,12 +1165,12 @@
           <t>Software Development Engineer Internship - Fall 2026 (US)</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1179,12 +1185,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H10" s="20" t="inlineStr">
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I10" s="20" t="inlineStr">
+      <c r="I10" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1199,20 +1205,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L10" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M10" s="20" t="inlineStr"/>
+      <c r="L10" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M10" s="22" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>4323643644</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1222,12 +1228,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D11" s="21" t="inlineStr">
+      <c r="D11" s="23" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E11" s="21" t="inlineStr">
+      <c r="E11" s="23" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1242,12 +1248,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H11" s="21" t="inlineStr">
+      <c r="H11" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I11" s="21" t="inlineStr">
+      <c r="I11" s="23" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1262,20 +1268,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L11" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M11" s="21" t="inlineStr"/>
+      <c r="L11" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M11" s="23" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>4320849104</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1285,12 +1291,12 @@
           <t>Software Engineer Intern (Commerce Ads) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E12" s="20" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1305,12 +1311,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H12" s="20" t="inlineStr">
+      <c r="H12" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I12" s="20" t="inlineStr">
+      <c r="I12" s="22" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1325,20 +1331,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L12" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M12" s="20" t="inlineStr"/>
+      <c r="L12" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M12" s="22" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>4401686051</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1348,12 +1354,12 @@
           <t>Front End Software Engineer</t>
         </is>
       </c>
-      <c r="D13" s="21" t="inlineStr">
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>Saronic Technologies</t>
         </is>
       </c>
-      <c r="E13" s="21" t="inlineStr">
+      <c r="E13" s="23" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
@@ -1368,12 +1374,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H13" s="21" t="inlineStr">
+      <c r="H13" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I13" s="21" t="inlineStr">
+      <c r="I13" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1388,20 +1394,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L13" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M13" s="21" t="inlineStr"/>
+      <c r="L13" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M13" s="23" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>4309696652</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1411,12 +1417,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="E14" s="22" t="inlineStr">
         <is>
           <t>Rhode Island, United States</t>
         </is>
@@ -1431,12 +1437,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H14" s="20" t="inlineStr">
+      <c r="H14" s="22" t="inlineStr">
         <is>
           <t>114</t>
         </is>
       </c>
-      <c r="I14" s="20" t="inlineStr">
+      <c r="I14" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1451,20 +1457,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L14" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M14" s="20" t="inlineStr"/>
+      <c r="L14" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M14" s="22" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>4309804319</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1474,12 +1480,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D15" s="21" t="inlineStr">
+      <c r="D15" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E15" s="21" t="inlineStr">
+      <c r="E15" s="23" t="inlineStr">
         <is>
           <t>Colorado, United States</t>
         </is>
@@ -1494,12 +1500,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H15" s="21" t="inlineStr">
+      <c r="H15" s="23" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="I15" s="21" t="inlineStr">
+      <c r="I15" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1514,20 +1520,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L15" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M15" s="21" t="inlineStr"/>
+      <c r="L15" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M15" s="23" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>4410271532</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1537,12 +1543,12 @@
           <t>Associate Developer</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>HealthStream</t>
         </is>
       </c>
-      <c r="E16" s="20" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>Nashville, TN</t>
         </is>
@@ -1557,12 +1563,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr">
+      <c r="H16" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I16" s="20" t="inlineStr">
+      <c r="I16" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1577,20 +1583,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L16" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M16" s="20" t="inlineStr"/>
+      <c r="L16" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M16" s="22" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>4304445726</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1600,12 +1606,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
+      <c r="E17" s="23" t="inlineStr">
         <is>
           <t>Oregon, United States</t>
         </is>
@@ -1620,12 +1626,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H17" s="21" t="inlineStr">
+      <c r="H17" s="23" t="inlineStr">
         <is>
           <t>115</t>
         </is>
       </c>
-      <c r="I17" s="21" t="inlineStr">
+      <c r="I17" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1640,20 +1646,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L17" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M17" s="21" t="inlineStr"/>
+      <c r="L17" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M17" s="23" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>4342036151</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1663,12 +1669,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D18" s="20" t="inlineStr">
+      <c r="D18" s="22" t="inlineStr">
         <is>
           <t>Modern Treasury</t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -1683,12 +1689,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H18" s="20" t="inlineStr">
+      <c r="H18" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I18" s="20" t="inlineStr">
+      <c r="I18" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1703,20 +1709,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L18" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M18" s="20" t="inlineStr"/>
+      <c r="L18" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M18" s="22" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>4304441843</t>
         </is>
       </c>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1726,12 +1732,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E19" s="23" t="inlineStr">
         <is>
           <t>Idaho, United States</t>
         </is>
@@ -1746,12 +1752,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H19" s="21" t="inlineStr">
+      <c r="H19" s="23" t="inlineStr">
         <is>
           <t>157</t>
         </is>
       </c>
-      <c r="I19" s="21" t="inlineStr">
+      <c r="I19" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1766,20 +1772,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L19" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M19" s="21" t="inlineStr"/>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M19" s="23" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>4408047047</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1789,12 +1795,12 @@
           <t>Computer Sciences - Graduates - AI Training - Las Vegas, US</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D20" s="22" t="inlineStr">
         <is>
           <t>Prolific</t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>Las Vegas, NV</t>
         </is>
@@ -1809,12 +1815,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H20" s="20" t="inlineStr">
+      <c r="H20" s="22" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="I20" s="20" t="inlineStr">
+      <c r="I20" s="22" t="inlineStr">
         <is>
           <t>Temporary</t>
         </is>
@@ -1829,20 +1835,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L20" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M20" s="20" t="inlineStr"/>
+      <c r="L20" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M20" s="22" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>4304444837</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1852,12 +1858,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D21" s="21" t="inlineStr">
+      <c r="D21" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E21" s="21" t="inlineStr">
+      <c r="E21" s="23" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -1872,12 +1878,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H21" s="21" t="inlineStr">
+      <c r="H21" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I21" s="21" t="inlineStr">
+      <c r="I21" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1892,20 +1898,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L21" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M21" s="21" t="inlineStr"/>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M21" s="23" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>4405641326</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1915,12 +1921,12 @@
           <t>Full-stack Engineer</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="D22" s="22" t="inlineStr">
         <is>
           <t>PartnerTap</t>
         </is>
       </c>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="E22" s="22" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1935,12 +1941,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H22" s="20" t="inlineStr">
+      <c r="H22" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I22" s="20" t="inlineStr">
+      <c r="I22" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1955,20 +1961,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L22" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M22" s="20" t="inlineStr"/>
+      <c r="L22" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M22" s="22" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>4341020900</t>
         </is>
       </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="B23" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1978,12 +1984,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D23" s="21" t="inlineStr">
+      <c r="D23" s="23" t="inlineStr">
         <is>
           <t>PlanIT Group, LLC</t>
         </is>
       </c>
-      <c r="E23" s="21" t="inlineStr">
+      <c r="E23" s="23" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -1998,12 +2004,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H23" s="21" t="inlineStr">
+      <c r="H23" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I23" s="21" t="inlineStr">
+      <c r="I23" s="23" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
@@ -2018,20 +2024,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L23" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M23" s="21" t="inlineStr"/>
+      <c r="L23" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M23" s="23" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>4304450637</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2041,12 +2047,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="D24" s="22" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="E24" s="22" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2061,12 +2067,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H24" s="20" t="inlineStr">
+      <c r="H24" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I24" s="20" t="inlineStr">
+      <c r="I24" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2081,20 +2087,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L24" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M24" s="20" t="inlineStr"/>
+      <c r="L24" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M24" s="22" t="inlineStr"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>4304451654</t>
         </is>
       </c>
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2104,12 +2110,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D25" s="21" t="inlineStr">
+      <c r="D25" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E25" s="21" t="inlineStr">
+      <c r="E25" s="23" t="inlineStr">
         <is>
           <t>Utah, United States</t>
         </is>
@@ -2124,12 +2130,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H25" s="21" t="inlineStr">
+      <c r="H25" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I25" s="21" t="inlineStr">
+      <c r="I25" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2144,20 +2150,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L25" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M25" s="21" t="inlineStr"/>
+      <c r="L25" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M25" s="23" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>4413745880</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2167,12 +2173,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D26" s="20" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
         <is>
           <t>Crate &amp; Barrel</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="E26" s="22" t="inlineStr">
         <is>
           <t>Northbrook, IL</t>
         </is>
@@ -2187,12 +2193,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H26" s="20" t="inlineStr">
+      <c r="H26" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I26" s="20" t="inlineStr">
+      <c r="I26" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2207,20 +2213,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L26" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M26" s="20" t="inlineStr"/>
+      <c r="L26" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M26" s="22" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="23" t="inlineStr">
         <is>
           <t>4304438841</t>
         </is>
       </c>
-      <c r="B27" s="21" t="inlineStr">
+      <c r="B27" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2230,12 +2236,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
+      <c r="D27" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
+      <c r="E27" s="23" t="inlineStr">
         <is>
           <t>Connecticut, United States</t>
         </is>
@@ -2250,12 +2256,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H27" s="21" t="inlineStr">
+      <c r="H27" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I27" s="21" t="inlineStr">
+      <c r="I27" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2270,20 +2276,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L27" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M27" s="21" t="inlineStr"/>
+      <c r="L27" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M27" s="23" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="20" t="inlineStr">
+      <c r="A28" s="22" t="inlineStr">
         <is>
           <t>4393215930</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2293,12 +2299,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D28" s="20" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>Transcend</t>
         </is>
       </c>
-      <c r="E28" s="20" t="inlineStr">
+      <c r="E28" s="22" t="inlineStr">
         <is>
           <t>California, United States</t>
         </is>
@@ -2313,12 +2319,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H28" s="20" t="inlineStr">
+      <c r="H28" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I28" s="20" t="inlineStr">
+      <c r="I28" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2333,20 +2339,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L28" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M28" s="20" t="inlineStr"/>
+      <c r="L28" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M28" s="22" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>4304445723</t>
         </is>
       </c>
-      <c r="B29" s="21" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2356,12 +2362,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D29" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E29" s="21" t="inlineStr">
+      <c r="E29" s="23" t="inlineStr">
         <is>
           <t>Illinois, United States</t>
         </is>
@@ -2376,12 +2382,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H29" s="21" t="inlineStr">
+      <c r="H29" s="23" t="inlineStr">
         <is>
           <t>198</t>
         </is>
       </c>
-      <c r="I29" s="21" t="inlineStr">
+      <c r="I29" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2396,20 +2402,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L29" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M29" s="21" t="inlineStr"/>
+      <c r="L29" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M29" s="23" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="20" t="inlineStr">
+      <c r="A30" s="22" t="inlineStr">
         <is>
           <t>4396380649</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B30" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2419,12 +2425,12 @@
           <t>Full-Stack Developer Intern, Music &amp; Audio</t>
         </is>
       </c>
-      <c r="D30" s="20" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>Melotech</t>
         </is>
       </c>
-      <c r="E30" s="20" t="inlineStr">
+      <c r="E30" s="22" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -2439,12 +2445,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H30" s="20" t="inlineStr">
+      <c r="H30" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I30" s="20" t="inlineStr">
+      <c r="I30" s="22" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -2459,20 +2465,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L30" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M30" s="20" t="inlineStr"/>
+      <c r="L30" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M30" s="22" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>4304454025</t>
         </is>
       </c>
-      <c r="B31" s="21" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2482,12 +2488,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D31" s="21" t="inlineStr">
+      <c r="D31" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E31" s="21" t="inlineStr">
+      <c r="E31" s="23" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -2502,12 +2508,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H31" s="21" t="inlineStr">
+      <c r="H31" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I31" s="21" t="inlineStr">
+      <c r="I31" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2522,20 +2528,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L31" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M31" s="21" t="inlineStr"/>
+      <c r="L31" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M31" s="23" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>4309802287</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B32" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2545,12 +2551,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D32" s="20" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E32" s="20" t="inlineStr">
+      <c r="E32" s="22" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -2565,12 +2571,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H32" s="20" t="inlineStr">
+      <c r="H32" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I32" s="20" t="inlineStr">
+      <c r="I32" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2585,20 +2591,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L32" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M32" s="20" t="inlineStr"/>
+      <c r="L32" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M32" s="22" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="21" t="inlineStr">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>4309694880</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2608,12 +2614,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D33" s="23" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E33" s="21" t="inlineStr">
+      <c r="E33" s="23" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2628,12 +2634,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H33" s="21" t="inlineStr">
+      <c r="H33" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I33" s="21" t="inlineStr">
+      <c r="I33" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2648,20 +2654,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L33" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M33" s="21" t="inlineStr"/>
+      <c r="L33" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M33" s="23" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="20" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>4411274012</t>
         </is>
       </c>
-      <c r="B34" s="20" t="inlineStr">
+      <c r="B34" s="22" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2671,12 +2677,12 @@
           <t>Junior UI Developer</t>
         </is>
       </c>
-      <c r="D34" s="20" t="inlineStr">
+      <c r="D34" s="22" t="inlineStr">
         <is>
           <t>General Dynamics Information Technology</t>
         </is>
       </c>
-      <c r="E34" s="20" t="inlineStr">
+      <c r="E34" s="22" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -2691,12 +2697,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H34" s="20" t="inlineStr">
+      <c r="H34" s="22" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I34" s="20" t="inlineStr">
+      <c r="I34" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2711,20 +2717,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L34" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M34" s="20" t="inlineStr"/>
+      <c r="L34" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M34" s="22" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="A35" s="23" t="inlineStr">
         <is>
           <t>4264562292</t>
         </is>
       </c>
-      <c r="B35" s="21" t="inlineStr">
+      <c r="B35" s="23" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2734,12 +2740,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D35" s="21" t="inlineStr">
+      <c r="D35" s="23" t="inlineStr">
         <is>
           <t>Cymertek Corporation</t>
         </is>
       </c>
-      <c r="E35" s="21" t="inlineStr">
+      <c r="E35" s="23" t="inlineStr">
         <is>
           <t>San Antonio, TX</t>
         </is>
@@ -2754,12 +2760,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H35" s="21" t="inlineStr">
+      <c r="H35" s="23" t="inlineStr">
         <is>
           <t>155</t>
         </is>
       </c>
-      <c r="I35" s="21" t="inlineStr">
+      <c r="I35" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2774,20 +2780,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L35" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M35" s="21" t="inlineStr"/>
+      <c r="L35" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M35" s="23" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="A36" s="22" t="inlineStr">
         <is>
           <t>4417482675</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B36" s="22" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2797,12 +2803,12 @@
           <t>Software Developer I</t>
         </is>
       </c>
-      <c r="D36" s="20" t="inlineStr">
+      <c r="D36" s="22" t="inlineStr">
         <is>
           <t>El Paso Water</t>
         </is>
       </c>
-      <c r="E36" s="20" t="inlineStr">
+      <c r="E36" s="22" t="inlineStr">
         <is>
           <t>El Paso, TX</t>
         </is>
@@ -2817,12 +2823,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H36" s="20" t="inlineStr">
+      <c r="H36" s="22" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="I36" s="20" t="inlineStr">
+      <c r="I36" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2837,20 +2843,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L36" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M36" s="20" t="inlineStr"/>
+      <c r="L36" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M36" s="22" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="21" t="inlineStr">
+      <c r="A37" s="23" t="inlineStr">
         <is>
           <t>4416508200</t>
         </is>
       </c>
-      <c r="B37" s="21" t="inlineStr">
+      <c r="B37" s="23" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2860,12 +2866,12 @@
           <t>Software Development Engineer in Test Intern (Global E-Commerce) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D37" s="21" t="inlineStr">
+      <c r="D37" s="23" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E37" s="21" t="inlineStr">
+      <c r="E37" s="23" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -2880,12 +2886,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H37" s="21" t="inlineStr">
+      <c r="H37" s="23" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="I37" s="21" t="inlineStr">
+      <c r="I37" s="23" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -2900,20 +2906,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L37" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M37" s="21" t="inlineStr"/>
+      <c r="L37" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M37" s="23" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="20" t="inlineStr">
+      <c r="A38" s="22" t="inlineStr">
         <is>
           <t>4309809191</t>
         </is>
       </c>
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B38" s="22" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -2923,12 +2929,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D38" s="20" t="inlineStr">
+      <c r="D38" s="22" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E38" s="20" t="inlineStr">
+      <c r="E38" s="22" t="inlineStr">
         <is>
           <t>Ohio, United States</t>
         </is>
@@ -2943,12 +2949,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H38" s="20" t="inlineStr">
+      <c r="H38" s="22" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="I38" s="20" t="inlineStr">
+      <c r="I38" s="22" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2963,20 +2969,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L38" s="20" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M38" s="20" t="inlineStr"/>
+      <c r="L38" s="22" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M38" s="22" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>3986118096</t>
         </is>
       </c>
-      <c r="B39" s="21" t="inlineStr">
+      <c r="B39" s="23" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -2986,12 +2992,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D39" s="21" t="inlineStr">
+      <c r="D39" s="23" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="E39" s="23" t="inlineStr">
         <is>
           <t>Irving, TX</t>
         </is>
@@ -3006,12 +3012,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H39" s="21" t="inlineStr">
+      <c r="H39" s="23" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I39" s="21" t="inlineStr">
+      <c r="I39" s="23" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3026,12 +3032,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L39" s="21" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M39" s="21" t="inlineStr"/>
+      <c r="L39" s="23" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M39" s="23" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="22" t="inlineStr">
@@ -3663,8 +3669,701 @@
       </c>
       <c r="M49" s="23" t="inlineStr"/>
     </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="24" t="inlineStr">
+        <is>
+          <t>4417553585</t>
+        </is>
+      </c>
+      <c r="B50" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Entry-Level Software Engineer | Remote</t>
+        </is>
+      </c>
+      <c r="D50" s="24" t="inlineStr">
+        <is>
+          <t>Crossing Hurdles</t>
+        </is>
+      </c>
+      <c r="E50" s="24" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H50" s="24" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I50" s="24" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>Skills: javascript, react, node, api, sql, backend, Title match: Entry-Level Software Engineer | Remote</t>
+        </is>
+      </c>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L50" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M50" s="24" t="inlineStr"/>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>4309699451</t>
+        </is>
+      </c>
+      <c r="B51" s="25" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D51" s="25" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E51" s="25" t="inlineStr">
+        <is>
+          <t>Washington, United States</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>76%</t>
+        </is>
+      </c>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H51" s="25" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="I51" s="25" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J51" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, full stack, c++, Location: Washington, United States, Title match: Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K51" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L51" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M51" s="25" t="inlineStr"/>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="24" t="inlineStr">
+        <is>
+          <t>4406945262</t>
+        </is>
+      </c>
+      <c r="B52" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>DevSecOps Intern</t>
+        </is>
+      </c>
+      <c r="D52" s="24" t="inlineStr">
+        <is>
+          <t>Modern Technology Solutions, Inc. (MTSI)</t>
+        </is>
+      </c>
+      <c r="E52" s="24" t="inlineStr">
+        <is>
+          <t>Niceville, FL</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H52" s="24" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="I52" s="24" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, rest, docker, git, c++, Title match: DevSecOps Intern</t>
+        </is>
+      </c>
+      <c r="K52" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L52" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M52" s="24" t="inlineStr"/>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="25" t="inlineStr">
+        <is>
+          <t>4407937810</t>
+        </is>
+      </c>
+      <c r="B53" s="25" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Temporary Intern - Agentic AI &amp; Neural-Symbolic Systems (Healthcare)</t>
+        </is>
+      </c>
+      <c r="D53" s="25" t="inlineStr">
+        <is>
+          <t>Cotiviti</t>
+        </is>
+      </c>
+      <c r="E53" s="25" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="G53" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H53" s="25" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I53" s="25" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J53" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, api, c, llm, Title match: Temporary Intern - Agentic AI &amp; Neural-Symbolic Systems (Healthcare)</t>
+        </is>
+      </c>
+      <c r="K53" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L53" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M53" s="25" t="inlineStr"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="24" t="inlineStr">
+        <is>
+          <t>4414089997</t>
+        </is>
+      </c>
+      <c r="B54" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Visualization Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D54" s="24" t="inlineStr">
+        <is>
+          <t>Leidos</t>
+        </is>
+      </c>
+      <c r="E54" s="24" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H54" s="24" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="I54" s="24" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, aws, rest, api, git, c++, Title match: Visualization Engineer Intern</t>
+        </is>
+      </c>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L54" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M54" s="24" t="inlineStr"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t>4387443129</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>2026 Interns</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="inlineStr">
+        <is>
+          <t>Givelify</t>
+        </is>
+      </c>
+      <c r="E55" s="25" t="inlineStr">
+        <is>
+          <t>Dallas, TX</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>48%</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H55" s="25" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I55" s="25" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J55" s="8" t="inlineStr">
+        <is>
+          <t>Skills: c, agile, Location: Dallas, TX, Title match: 2026 Interns</t>
+        </is>
+      </c>
+      <c r="K55" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L55" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M55" s="25" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="24" t="inlineStr">
+        <is>
+          <t>4337980765</t>
+        </is>
+      </c>
+      <c r="B56" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Submitting for a General Internship Application</t>
+        </is>
+      </c>
+      <c r="D56" s="24" t="inlineStr">
+        <is>
+          <t>Chainguard</t>
+        </is>
+      </c>
+      <c r="E56" s="24" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F56" s="18" t="inlineStr">
+        <is>
+          <t>32%</t>
+        </is>
+      </c>
+      <c r="G56" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H56" s="24" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I56" s="24" t="inlineStr">
+        <is>
+          <t>Volunteer</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Skills: api, c, express, Title match: Submitting for a General Internship Application</t>
+        </is>
+      </c>
+      <c r="K56" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L56" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M56" s="24" t="inlineStr"/>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>4417030460</t>
+        </is>
+      </c>
+      <c r="B57" s="25" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>AI Researcher Intern</t>
+        </is>
+      </c>
+      <c r="D57" s="25" t="inlineStr">
+        <is>
+          <t>BioSpace</t>
+        </is>
+      </c>
+      <c r="E57" s="25" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>48%</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H57" s="25" t="inlineStr">
+        <is>
+          <t>151</t>
+        </is>
+      </c>
+      <c r="I57" s="25" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J57" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, api, docker, c, express, llm, Title match: AI Researcher Intern</t>
+        </is>
+      </c>
+      <c r="K57" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L57" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M57" s="25" t="inlineStr"/>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="24" t="inlineStr">
+        <is>
+          <t>4406930916</t>
+        </is>
+      </c>
+      <c r="B58" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>DevSecOps Intern</t>
+        </is>
+      </c>
+      <c r="D58" s="24" t="inlineStr">
+        <is>
+          <t>Modern Technology Solutions, Inc. (MTSI)</t>
+        </is>
+      </c>
+      <c r="E58" s="24" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H58" s="24" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I58" s="24" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, rest, docker, git, c++, Title match: DevSecOps Intern</t>
+        </is>
+      </c>
+      <c r="K58" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L58" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M58" s="24" t="inlineStr"/>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="25" t="inlineStr">
+        <is>
+          <t>4385798937</t>
+        </is>
+      </c>
+      <c r="B59" s="25" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>Research Intern on Generative and Protective AI for Content Creation</t>
+        </is>
+      </c>
+      <c r="D59" s="25" t="inlineStr">
+        <is>
+          <t>SonyAI</t>
+        </is>
+      </c>
+      <c r="E59" s="25" t="inlineStr">
+        <is>
+          <t>New York, United States</t>
+        </is>
+      </c>
+      <c r="F59" s="18" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H59" s="25" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I59" s="25" t="inlineStr">
+        <is>
+          <t>Part-time</t>
+        </is>
+      </c>
+      <c r="J59" s="8" t="inlineStr">
+        <is>
+          <t>Skills: aws, pytorch, machine learning, c, algorithms, Title match: Research Intern on Generative and Protective AI for Content Creation</t>
+        </is>
+      </c>
+      <c r="K59" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L59" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M59" s="25" t="inlineStr"/>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="24" t="inlineStr">
+        <is>
+          <t>4414396950</t>
+        </is>
+      </c>
+      <c r="B60" s="24" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Power Platform Intern</t>
+        </is>
+      </c>
+      <c r="D60" s="24" t="inlineStr">
+        <is>
+          <t>Leidos</t>
+        </is>
+      </c>
+      <c r="E60" s="24" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H60" s="24" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="I60" s="24" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>Skills: aws, rest, html, css, git, sql, Title match: Power Platform Intern</t>
+        </is>
+      </c>
+      <c r="K60" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L60" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M60" s="24" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M49"/>
+  <autoFilter ref="A1:M60"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -3714,6 +4413,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-05-27
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -193,6 +193,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -560,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M60"/>
+  <dimension ref="A1:M81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -646,12 +652,12 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>4406952064</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -661,12 +667,12 @@
           <t>DevSecOps Intern</t>
         </is>
       </c>
-      <c r="D2" s="22" t="inlineStr">
+      <c r="D2" s="24" t="inlineStr">
         <is>
           <t>Modern Technology Solutions, Inc. (MTSI)</t>
         </is>
       </c>
-      <c r="E2" s="22" t="inlineStr">
+      <c r="E2" s="24" t="inlineStr">
         <is>
           <t>Huntsville, AL</t>
         </is>
@@ -681,12 +687,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H2" s="22" t="inlineStr">
+      <c r="H2" s="24" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="I2" s="22" t="inlineStr">
+      <c r="I2" s="24" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -701,20 +707,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L2" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M2" s="22" t="inlineStr"/>
+      <c r="L2" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M2" s="24" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>4405630173</t>
         </is>
       </c>
-      <c r="B3" s="23" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -724,12 +730,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D3" s="23" t="inlineStr">
+      <c r="D3" s="25" t="inlineStr">
         <is>
           <t>DLRdmv®</t>
         </is>
       </c>
-      <c r="E3" s="23" t="inlineStr">
+      <c r="E3" s="25" t="inlineStr">
         <is>
           <t>Dallas, TX</t>
         </is>
@@ -744,12 +750,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H3" s="23" t="inlineStr">
+      <c r="H3" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I3" s="23" t="inlineStr">
+      <c r="I3" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -764,20 +770,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L3" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M3" s="23" t="inlineStr"/>
+      <c r="L3" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M3" s="25" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>4287414862</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -787,12 +793,12 @@
           <t>[Online Assessment]Software Development Engineer Intern (Network Automation)- 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>ByteDance</t>
         </is>
       </c>
-      <c r="E4" s="22" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -807,12 +813,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="22" t="inlineStr">
+      <c r="H4" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I4" s="22" t="inlineStr">
+      <c r="I4" s="24" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -827,20 +833,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L4" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M4" s="22" t="inlineStr"/>
+      <c r="L4" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M4" s="24" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>4309805269</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -850,12 +856,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E5" s="23" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Delaware, United States</t>
         </is>
@@ -870,12 +876,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" s="23" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>81</t>
         </is>
       </c>
-      <c r="I5" s="23" t="inlineStr">
+      <c r="I5" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -890,20 +896,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L5" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M5" s="23" t="inlineStr"/>
+      <c r="L5" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M5" s="25" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>4371812987</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -913,12 +919,12 @@
           <t>Software Development Engineer Fall Intern - Military Veteran</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr">
+      <c r="D6" s="24" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E6" s="22" t="inlineStr">
+      <c r="E6" s="24" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -933,12 +939,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H6" s="22" t="inlineStr">
+      <c r="H6" s="24" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr">
+      <c r="I6" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -953,20 +959,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L6" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M6" s="22" t="inlineStr"/>
+      <c r="L6" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M6" s="24" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>4274682122</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -976,12 +982,12 @@
           <t>Software Engineer Intern (Data Ecosystem) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="25" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E7" s="23" t="inlineStr">
+      <c r="E7" s="25" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -996,12 +1002,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="23" t="inlineStr">
+      <c r="H7" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I7" s="23" t="inlineStr">
+      <c r="I7" s="25" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1016,20 +1022,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L7" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M7" s="23" t="inlineStr"/>
+      <c r="L7" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M7" s="25" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>4283848614</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1039,12 +1045,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Fall (BS/ MS)</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr">
+      <c r="D8" s="24" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr">
+      <c r="E8" s="24" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1059,12 +1065,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H8" s="22" t="inlineStr">
+      <c r="H8" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr">
+      <c r="I8" s="24" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1079,20 +1085,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L8" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M8" s="22" t="inlineStr"/>
+      <c r="L8" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M8" s="24" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>4411790844</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1102,12 +1108,12 @@
           <t>Software Engineer Intern (Infrastructure Automation) - Fall 2026</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="25" t="inlineStr">
         <is>
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E9" s="23" t="inlineStr">
+      <c r="E9" s="25" t="inlineStr">
         <is>
           <t>Bellevue, WA</t>
         </is>
@@ -1122,12 +1128,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H9" s="23" t="inlineStr">
+      <c r="H9" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I9" s="23" t="inlineStr">
+      <c r="I9" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1142,20 +1148,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L9" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M9" s="23" t="inlineStr"/>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M9" s="25" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>4332425058</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1165,12 +1171,12 @@
           <t>Software Development Engineer Internship - Fall 2026 (US)</t>
         </is>
       </c>
-      <c r="D10" s="22" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1185,12 +1191,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H10" s="22" t="inlineStr">
+      <c r="H10" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I10" s="22" t="inlineStr">
+      <c r="I10" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1205,20 +1211,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L10" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M10" s="22" t="inlineStr"/>
+      <c r="L10" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M10" s="24" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>4323643644</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1228,12 +1234,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D11" s="23" t="inlineStr">
+      <c r="D11" s="25" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E11" s="23" t="inlineStr">
+      <c r="E11" s="25" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1248,12 +1254,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H11" s="23" t="inlineStr">
+      <c r="H11" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I11" s="23" t="inlineStr">
+      <c r="I11" s="25" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1268,20 +1274,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L11" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M11" s="23" t="inlineStr"/>
+      <c r="L11" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M11" s="25" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>4320849104</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1291,12 +1297,12 @@
           <t>Software Engineer Intern (Commerce Ads) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D12" s="22" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
+      <c r="E12" s="24" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1311,12 +1317,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H12" s="22" t="inlineStr">
+      <c r="H12" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I12" s="22" t="inlineStr">
+      <c r="I12" s="24" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1331,20 +1337,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L12" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M12" s="22" t="inlineStr"/>
+      <c r="L12" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M12" s="24" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>4401686051</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1354,12 +1360,12 @@
           <t>Front End Software Engineer</t>
         </is>
       </c>
-      <c r="D13" s="23" t="inlineStr">
+      <c r="D13" s="25" t="inlineStr">
         <is>
           <t>Saronic Technologies</t>
         </is>
       </c>
-      <c r="E13" s="23" t="inlineStr">
+      <c r="E13" s="25" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
@@ -1374,12 +1380,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H13" s="23" t="inlineStr">
+      <c r="H13" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I13" s="23" t="inlineStr">
+      <c r="I13" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1394,20 +1400,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L13" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M13" s="23" t="inlineStr"/>
+      <c r="L13" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M13" s="25" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>4309696652</t>
         </is>
       </c>
-      <c r="B14" s="22" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1417,12 +1423,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D14" s="22" t="inlineStr">
+      <c r="D14" s="24" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E14" s="22" t="inlineStr">
+      <c r="E14" s="24" t="inlineStr">
         <is>
           <t>Rhode Island, United States</t>
         </is>
@@ -1437,12 +1443,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H14" s="22" t="inlineStr">
+      <c r="H14" s="24" t="inlineStr">
         <is>
           <t>114</t>
         </is>
       </c>
-      <c r="I14" s="22" t="inlineStr">
+      <c r="I14" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1457,20 +1463,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L14" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M14" s="22" t="inlineStr"/>
+      <c r="L14" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M14" s="24" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>4309804319</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1480,12 +1486,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D15" s="23" t="inlineStr">
+      <c r="D15" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E15" s="23" t="inlineStr">
+      <c r="E15" s="25" t="inlineStr">
         <is>
           <t>Colorado, United States</t>
         </is>
@@ -1500,12 +1506,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H15" s="23" t="inlineStr">
+      <c r="H15" s="25" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="I15" s="23" t="inlineStr">
+      <c r="I15" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1520,20 +1526,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L15" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M15" s="23" t="inlineStr"/>
+      <c r="L15" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M15" s="25" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>4410271532</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1543,12 +1549,12 @@
           <t>Associate Developer</t>
         </is>
       </c>
-      <c r="D16" s="22" t="inlineStr">
+      <c r="D16" s="24" t="inlineStr">
         <is>
           <t>HealthStream</t>
         </is>
       </c>
-      <c r="E16" s="22" t="inlineStr">
+      <c r="E16" s="24" t="inlineStr">
         <is>
           <t>Nashville, TN</t>
         </is>
@@ -1563,12 +1569,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H16" s="22" t="inlineStr">
+      <c r="H16" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I16" s="22" t="inlineStr">
+      <c r="I16" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1583,20 +1589,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L16" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M16" s="22" t="inlineStr"/>
+      <c r="L16" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M16" s="24" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>4304445726</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1606,12 +1612,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D17" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E17" s="23" t="inlineStr">
+      <c r="E17" s="25" t="inlineStr">
         <is>
           <t>Oregon, United States</t>
         </is>
@@ -1626,12 +1632,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H17" s="23" t="inlineStr">
+      <c r="H17" s="25" t="inlineStr">
         <is>
           <t>115</t>
         </is>
       </c>
-      <c r="I17" s="23" t="inlineStr">
+      <c r="I17" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1646,20 +1652,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L17" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M17" s="23" t="inlineStr"/>
+      <c r="L17" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M17" s="25" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>4342036151</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1669,12 +1675,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D18" s="22" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>Modern Treasury</t>
         </is>
       </c>
-      <c r="E18" s="22" t="inlineStr">
+      <c r="E18" s="24" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -1689,12 +1695,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H18" s="22" t="inlineStr">
+      <c r="H18" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I18" s="22" t="inlineStr">
+      <c r="I18" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1709,20 +1715,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L18" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M18" s="22" t="inlineStr"/>
+      <c r="L18" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M18" s="24" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>4304441843</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1732,12 +1738,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D19" s="23" t="inlineStr">
+      <c r="D19" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E19" s="23" t="inlineStr">
+      <c r="E19" s="25" t="inlineStr">
         <is>
           <t>Idaho, United States</t>
         </is>
@@ -1752,12 +1758,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H19" s="23" t="inlineStr">
+      <c r="H19" s="25" t="inlineStr">
         <is>
           <t>157</t>
         </is>
       </c>
-      <c r="I19" s="23" t="inlineStr">
+      <c r="I19" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1772,20 +1778,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L19" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M19" s="23" t="inlineStr"/>
+      <c r="L19" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M19" s="25" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>4408047047</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1795,12 +1801,12 @@
           <t>Computer Sciences - Graduates - AI Training - Las Vegas, US</t>
         </is>
       </c>
-      <c r="D20" s="22" t="inlineStr">
+      <c r="D20" s="24" t="inlineStr">
         <is>
           <t>Prolific</t>
         </is>
       </c>
-      <c r="E20" s="22" t="inlineStr">
+      <c r="E20" s="24" t="inlineStr">
         <is>
           <t>Las Vegas, NV</t>
         </is>
@@ -1815,12 +1821,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H20" s="22" t="inlineStr">
+      <c r="H20" s="24" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="I20" s="22" t="inlineStr">
+      <c r="I20" s="24" t="inlineStr">
         <is>
           <t>Temporary</t>
         </is>
@@ -1835,20 +1841,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L20" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M20" s="22" t="inlineStr"/>
+      <c r="L20" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M20" s="24" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>4304444837</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1858,12 +1864,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E21" s="23" t="inlineStr">
+      <c r="E21" s="25" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -1878,12 +1884,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H21" s="23" t="inlineStr">
+      <c r="H21" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I21" s="23" t="inlineStr">
+      <c r="I21" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1898,20 +1904,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L21" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M21" s="23" t="inlineStr"/>
+      <c r="L21" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M21" s="25" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>4405641326</t>
         </is>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1921,12 +1927,12 @@
           <t>Full-stack Engineer</t>
         </is>
       </c>
-      <c r="D22" s="22" t="inlineStr">
+      <c r="D22" s="24" t="inlineStr">
         <is>
           <t>PartnerTap</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
+      <c r="E22" s="24" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1941,12 +1947,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H22" s="22" t="inlineStr">
+      <c r="H22" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I22" s="22" t="inlineStr">
+      <c r="I22" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1961,20 +1967,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L22" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M22" s="22" t="inlineStr"/>
+      <c r="L22" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M22" s="24" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="23" t="inlineStr">
+      <c r="A23" s="25" t="inlineStr">
         <is>
           <t>4341020900</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1984,12 +1990,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D23" s="23" t="inlineStr">
+      <c r="D23" s="25" t="inlineStr">
         <is>
           <t>PlanIT Group, LLC</t>
         </is>
       </c>
-      <c r="E23" s="23" t="inlineStr">
+      <c r="E23" s="25" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -2004,12 +2010,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H23" s="23" t="inlineStr">
+      <c r="H23" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I23" s="23" t="inlineStr">
+      <c r="I23" s="25" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
@@ -2024,20 +2030,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L23" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M23" s="23" t="inlineStr"/>
+      <c r="L23" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M23" s="25" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="22" t="inlineStr">
+      <c r="A24" s="24" t="inlineStr">
         <is>
           <t>4304450637</t>
         </is>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2047,12 +2053,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D24" s="22" t="inlineStr">
+      <c r="D24" s="24" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr">
+      <c r="E24" s="24" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2067,12 +2073,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H24" s="22" t="inlineStr">
+      <c r="H24" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I24" s="22" t="inlineStr">
+      <c r="I24" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2087,20 +2093,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L24" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M24" s="22" t="inlineStr"/>
+      <c r="L24" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M24" s="24" t="inlineStr"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="23" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>4304451654</t>
         </is>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2110,12 +2116,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D25" s="23" t="inlineStr">
+      <c r="D25" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E25" s="23" t="inlineStr">
+      <c r="E25" s="25" t="inlineStr">
         <is>
           <t>Utah, United States</t>
         </is>
@@ -2130,12 +2136,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H25" s="23" t="inlineStr">
+      <c r="H25" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I25" s="23" t="inlineStr">
+      <c r="I25" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2150,20 +2156,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L25" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M25" s="23" t="inlineStr"/>
+      <c r="L25" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M25" s="25" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="22" t="inlineStr">
+      <c r="A26" s="24" t="inlineStr">
         <is>
           <t>4413745880</t>
         </is>
       </c>
-      <c r="B26" s="22" t="inlineStr">
+      <c r="B26" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2173,12 +2179,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D26" s="22" t="inlineStr">
+      <c r="D26" s="24" t="inlineStr">
         <is>
           <t>Crate &amp; Barrel</t>
         </is>
       </c>
-      <c r="E26" s="22" t="inlineStr">
+      <c r="E26" s="24" t="inlineStr">
         <is>
           <t>Northbrook, IL</t>
         </is>
@@ -2193,12 +2199,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H26" s="22" t="inlineStr">
+      <c r="H26" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I26" s="22" t="inlineStr">
+      <c r="I26" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2213,20 +2219,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L26" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M26" s="22" t="inlineStr"/>
+      <c r="L26" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M26" s="24" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="23" t="inlineStr">
+      <c r="A27" s="25" t="inlineStr">
         <is>
           <t>4304438841</t>
         </is>
       </c>
-      <c r="B27" s="23" t="inlineStr">
+      <c r="B27" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2236,12 +2242,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D27" s="23" t="inlineStr">
+      <c r="D27" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E27" s="23" t="inlineStr">
+      <c r="E27" s="25" t="inlineStr">
         <is>
           <t>Connecticut, United States</t>
         </is>
@@ -2256,12 +2262,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H27" s="23" t="inlineStr">
+      <c r="H27" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I27" s="23" t="inlineStr">
+      <c r="I27" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2276,20 +2282,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L27" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M27" s="23" t="inlineStr"/>
+      <c r="L27" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M27" s="25" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>4393215930</t>
         </is>
       </c>
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2299,12 +2305,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D28" s="22" t="inlineStr">
+      <c r="D28" s="24" t="inlineStr">
         <is>
           <t>Transcend</t>
         </is>
       </c>
-      <c r="E28" s="22" t="inlineStr">
+      <c r="E28" s="24" t="inlineStr">
         <is>
           <t>California, United States</t>
         </is>
@@ -2319,12 +2325,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H28" s="22" t="inlineStr">
+      <c r="H28" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I28" s="22" t="inlineStr">
+      <c r="I28" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2339,20 +2345,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L28" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M28" s="22" t="inlineStr"/>
+      <c r="L28" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M28" s="24" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="23" t="inlineStr">
+      <c r="A29" s="25" t="inlineStr">
         <is>
           <t>4304445723</t>
         </is>
       </c>
-      <c r="B29" s="23" t="inlineStr">
+      <c r="B29" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2362,12 +2368,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D29" s="23" t="inlineStr">
+      <c r="D29" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr">
+      <c r="E29" s="25" t="inlineStr">
         <is>
           <t>Illinois, United States</t>
         </is>
@@ -2382,12 +2388,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H29" s="23" t="inlineStr">
+      <c r="H29" s="25" t="inlineStr">
         <is>
           <t>198</t>
         </is>
       </c>
-      <c r="I29" s="23" t="inlineStr">
+      <c r="I29" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2402,20 +2408,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L29" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M29" s="23" t="inlineStr"/>
+      <c r="L29" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M29" s="25" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="22" t="inlineStr">
+      <c r="A30" s="24" t="inlineStr">
         <is>
           <t>4396380649</t>
         </is>
       </c>
-      <c r="B30" s="22" t="inlineStr">
+      <c r="B30" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2425,12 +2431,12 @@
           <t>Full-Stack Developer Intern, Music &amp; Audio</t>
         </is>
       </c>
-      <c r="D30" s="22" t="inlineStr">
+      <c r="D30" s="24" t="inlineStr">
         <is>
           <t>Melotech</t>
         </is>
       </c>
-      <c r="E30" s="22" t="inlineStr">
+      <c r="E30" s="24" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -2445,12 +2451,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H30" s="22" t="inlineStr">
+      <c r="H30" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I30" s="22" t="inlineStr">
+      <c r="I30" s="24" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -2465,20 +2471,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L30" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M30" s="22" t="inlineStr"/>
+      <c r="L30" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M30" s="24" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="23" t="inlineStr">
+      <c r="A31" s="25" t="inlineStr">
         <is>
           <t>4304454025</t>
         </is>
       </c>
-      <c r="B31" s="23" t="inlineStr">
+      <c r="B31" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2488,12 +2494,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D31" s="23" t="inlineStr">
+      <c r="D31" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E31" s="23" t="inlineStr">
+      <c r="E31" s="25" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -2508,12 +2514,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H31" s="23" t="inlineStr">
+      <c r="H31" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I31" s="23" t="inlineStr">
+      <c r="I31" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2528,20 +2534,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L31" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M31" s="23" t="inlineStr"/>
+      <c r="L31" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M31" s="25" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="22" t="inlineStr">
+      <c r="A32" s="24" t="inlineStr">
         <is>
           <t>4309802287</t>
         </is>
       </c>
-      <c r="B32" s="22" t="inlineStr">
+      <c r="B32" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2551,12 +2557,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D32" s="22" t="inlineStr">
+      <c r="D32" s="24" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E32" s="22" t="inlineStr">
+      <c r="E32" s="24" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -2571,12 +2577,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H32" s="22" t="inlineStr">
+      <c r="H32" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I32" s="22" t="inlineStr">
+      <c r="I32" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2591,20 +2597,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L32" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M32" s="22" t="inlineStr"/>
+      <c r="L32" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M32" s="24" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="23" t="inlineStr">
+      <c r="A33" s="25" t="inlineStr">
         <is>
           <t>4309694880</t>
         </is>
       </c>
-      <c r="B33" s="23" t="inlineStr">
+      <c r="B33" s="25" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2614,12 +2620,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D33" s="23" t="inlineStr">
+      <c r="D33" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E33" s="23" t="inlineStr">
+      <c r="E33" s="25" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2634,12 +2640,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H33" s="23" t="inlineStr">
+      <c r="H33" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I33" s="23" t="inlineStr">
+      <c r="I33" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2654,20 +2660,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L33" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M33" s="23" t="inlineStr"/>
+      <c r="L33" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M33" s="25" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="22" t="inlineStr">
+      <c r="A34" s="24" t="inlineStr">
         <is>
           <t>4411274012</t>
         </is>
       </c>
-      <c r="B34" s="22" t="inlineStr">
+      <c r="B34" s="24" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2677,12 +2683,12 @@
           <t>Junior UI Developer</t>
         </is>
       </c>
-      <c r="D34" s="22" t="inlineStr">
+      <c r="D34" s="24" t="inlineStr">
         <is>
           <t>General Dynamics Information Technology</t>
         </is>
       </c>
-      <c r="E34" s="22" t="inlineStr">
+      <c r="E34" s="24" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -2697,12 +2703,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H34" s="22" t="inlineStr">
+      <c r="H34" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I34" s="22" t="inlineStr">
+      <c r="I34" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2717,20 +2723,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L34" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M34" s="22" t="inlineStr"/>
+      <c r="L34" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M34" s="24" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="23" t="inlineStr">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>4264562292</t>
         </is>
       </c>
-      <c r="B35" s="23" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2740,12 +2746,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D35" s="23" t="inlineStr">
+      <c r="D35" s="25" t="inlineStr">
         <is>
           <t>Cymertek Corporation</t>
         </is>
       </c>
-      <c r="E35" s="23" t="inlineStr">
+      <c r="E35" s="25" t="inlineStr">
         <is>
           <t>San Antonio, TX</t>
         </is>
@@ -2760,12 +2766,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H35" s="23" t="inlineStr">
+      <c r="H35" s="25" t="inlineStr">
         <is>
           <t>155</t>
         </is>
       </c>
-      <c r="I35" s="23" t="inlineStr">
+      <c r="I35" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2780,20 +2786,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L35" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M35" s="23" t="inlineStr"/>
+      <c r="L35" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M35" s="25" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="22" t="inlineStr">
+      <c r="A36" s="24" t="inlineStr">
         <is>
           <t>4417482675</t>
         </is>
       </c>
-      <c r="B36" s="22" t="inlineStr">
+      <c r="B36" s="24" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2803,12 +2809,12 @@
           <t>Software Developer I</t>
         </is>
       </c>
-      <c r="D36" s="22" t="inlineStr">
+      <c r="D36" s="24" t="inlineStr">
         <is>
           <t>El Paso Water</t>
         </is>
       </c>
-      <c r="E36" s="22" t="inlineStr">
+      <c r="E36" s="24" t="inlineStr">
         <is>
           <t>El Paso, TX</t>
         </is>
@@ -2823,12 +2829,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H36" s="22" t="inlineStr">
+      <c r="H36" s="24" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="I36" s="22" t="inlineStr">
+      <c r="I36" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2843,20 +2849,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L36" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M36" s="22" t="inlineStr"/>
+      <c r="L36" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M36" s="24" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="23" t="inlineStr">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>4416508200</t>
         </is>
       </c>
-      <c r="B37" s="23" t="inlineStr">
+      <c r="B37" s="25" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2866,12 +2872,12 @@
           <t>Software Development Engineer in Test Intern (Global E-Commerce) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D37" s="23" t="inlineStr">
+      <c r="D37" s="25" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E37" s="23" t="inlineStr">
+      <c r="E37" s="25" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -2886,12 +2892,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H37" s="23" t="inlineStr">
+      <c r="H37" s="25" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="I37" s="23" t="inlineStr">
+      <c r="I37" s="25" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -2906,20 +2912,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L37" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M37" s="23" t="inlineStr"/>
+      <c r="L37" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M37" s="25" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="22" t="inlineStr">
+      <c r="A38" s="24" t="inlineStr">
         <is>
           <t>4309809191</t>
         </is>
       </c>
-      <c r="B38" s="22" t="inlineStr">
+      <c r="B38" s="24" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -2929,12 +2935,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D38" s="22" t="inlineStr">
+      <c r="D38" s="24" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E38" s="22" t="inlineStr">
+      <c r="E38" s="24" t="inlineStr">
         <is>
           <t>Ohio, United States</t>
         </is>
@@ -2949,12 +2955,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H38" s="22" t="inlineStr">
+      <c r="H38" s="24" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="I38" s="22" t="inlineStr">
+      <c r="I38" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2969,20 +2975,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L38" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M38" s="22" t="inlineStr"/>
+      <c r="L38" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M38" s="24" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="23" t="inlineStr">
+      <c r="A39" s="25" t="inlineStr">
         <is>
           <t>3986118096</t>
         </is>
       </c>
-      <c r="B39" s="23" t="inlineStr">
+      <c r="B39" s="25" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -2992,12 +2998,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D39" s="23" t="inlineStr">
+      <c r="D39" s="25" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="E39" s="23" t="inlineStr">
+      <c r="E39" s="25" t="inlineStr">
         <is>
           <t>Irving, TX</t>
         </is>
@@ -3012,12 +3018,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H39" s="23" t="inlineStr">
+      <c r="H39" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I39" s="23" t="inlineStr">
+      <c r="I39" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3032,20 +3038,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L39" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M39" s="23" t="inlineStr"/>
+      <c r="L39" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M39" s="25" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="22" t="inlineStr">
+      <c r="A40" s="24" t="inlineStr">
         <is>
           <t>4309808244</t>
         </is>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B40" s="24" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3055,12 +3061,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D40" s="22" t="inlineStr">
+      <c r="D40" s="24" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr">
+      <c r="E40" s="24" t="inlineStr">
         <is>
           <t>Massachusetts, United States</t>
         </is>
@@ -3075,12 +3081,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H40" s="22" t="inlineStr">
+      <c r="H40" s="24" t="inlineStr">
         <is>
           <t>166</t>
         </is>
       </c>
-      <c r="I40" s="22" t="inlineStr">
+      <c r="I40" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3095,20 +3101,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L40" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M40" s="22" t="inlineStr"/>
+      <c r="L40" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M40" s="24" t="inlineStr"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="23" t="inlineStr">
+      <c r="A41" s="25" t="inlineStr">
         <is>
           <t>4362173625</t>
         </is>
       </c>
-      <c r="B41" s="23" t="inlineStr">
+      <c r="B41" s="25" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3118,12 +3124,12 @@
           <t>Full Stack Engineer</t>
         </is>
       </c>
-      <c r="D41" s="23" t="inlineStr">
+      <c r="D41" s="25" t="inlineStr">
         <is>
           <t>Empower Sleep</t>
         </is>
       </c>
-      <c r="E41" s="23" t="inlineStr">
+      <c r="E41" s="25" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3138,12 +3144,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H41" s="23" t="inlineStr">
+      <c r="H41" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I41" s="23" t="inlineStr">
+      <c r="I41" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3158,20 +3164,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L41" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M41" s="23" t="inlineStr"/>
+      <c r="L41" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M41" s="25" t="inlineStr"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="22" t="inlineStr">
+      <c r="A42" s="24" t="inlineStr">
         <is>
           <t>4309812093</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="24" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3181,12 +3187,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D42" s="22" t="inlineStr">
+      <c r="D42" s="24" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr">
+      <c r="E42" s="24" t="inlineStr">
         <is>
           <t>Florida, United States</t>
         </is>
@@ -3201,12 +3207,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H42" s="22" t="inlineStr">
+      <c r="H42" s="24" t="inlineStr">
         <is>
           <t>158</t>
         </is>
       </c>
-      <c r="I42" s="22" t="inlineStr">
+      <c r="I42" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3221,20 +3227,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L42" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M42" s="22" t="inlineStr"/>
+      <c r="L42" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M42" s="24" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="23" t="inlineStr">
+      <c r="A43" s="25" t="inlineStr">
         <is>
           <t>4391759914</t>
         </is>
       </c>
-      <c r="B43" s="23" t="inlineStr">
+      <c r="B43" s="25" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3244,12 +3250,12 @@
           <t>QA Engineering Internship</t>
         </is>
       </c>
-      <c r="D43" s="23" t="inlineStr">
+      <c r="D43" s="25" t="inlineStr">
         <is>
           <t>Chartbeat</t>
         </is>
       </c>
-      <c r="E43" s="23" t="inlineStr">
+      <c r="E43" s="25" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
@@ -3264,12 +3270,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H43" s="23" t="inlineStr">
+      <c r="H43" s="25" t="inlineStr">
         <is>
           <t>168</t>
         </is>
       </c>
-      <c r="I43" s="23" t="inlineStr">
+      <c r="I43" s="25" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -3284,20 +3290,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L43" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M43" s="23" t="inlineStr"/>
+      <c r="L43" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M43" s="25" t="inlineStr"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="22" t="inlineStr">
+      <c r="A44" s="24" t="inlineStr">
         <is>
           <t>4412855678</t>
         </is>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B44" s="24" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3307,12 +3313,12 @@
           <t>AI Integration Engineer</t>
         </is>
       </c>
-      <c r="D44" s="22" t="inlineStr">
+      <c r="D44" s="24" t="inlineStr">
         <is>
           <t>UST</t>
         </is>
       </c>
-      <c r="E44" s="22" t="inlineStr">
+      <c r="E44" s="24" t="inlineStr">
         <is>
           <t>Santa Clara, CA</t>
         </is>
@@ -3327,12 +3333,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H44" s="22" t="inlineStr">
+      <c r="H44" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I44" s="22" t="inlineStr">
+      <c r="I44" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3347,20 +3353,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L44" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M44" s="22" t="inlineStr"/>
+      <c r="L44" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M44" s="24" t="inlineStr"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="23" t="inlineStr">
+      <c r="A45" s="25" t="inlineStr">
         <is>
           <t>4309805219</t>
         </is>
       </c>
-      <c r="B45" s="23" t="inlineStr">
+      <c r="B45" s="25" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3370,12 +3376,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D45" s="23" t="inlineStr">
+      <c r="D45" s="25" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E45" s="23" t="inlineStr">
+      <c r="E45" s="25" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -3390,12 +3396,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H45" s="23" t="inlineStr">
+      <c r="H45" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I45" s="23" t="inlineStr">
+      <c r="I45" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3410,20 +3416,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L45" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M45" s="23" t="inlineStr"/>
+      <c r="L45" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M45" s="25" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="22" t="inlineStr">
+      <c r="A46" s="24" t="inlineStr">
         <is>
           <t>4409726429</t>
         </is>
       </c>
-      <c r="B46" s="22" t="inlineStr">
+      <c r="B46" s="24" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3433,12 +3439,12 @@
           <t>Data Science Intern</t>
         </is>
       </c>
-      <c r="D46" s="22" t="inlineStr">
+      <c r="D46" s="24" t="inlineStr">
         <is>
           <t>Rundoo</t>
         </is>
       </c>
-      <c r="E46" s="22" t="inlineStr">
+      <c r="E46" s="24" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3453,12 +3459,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H46" s="22" t="inlineStr">
+      <c r="H46" s="24" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I46" s="22" t="inlineStr">
+      <c r="I46" s="24" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -3473,20 +3479,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L46" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M46" s="22" t="inlineStr"/>
+      <c r="L46" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M46" s="24" t="inlineStr"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="23" t="inlineStr">
+      <c r="A47" s="25" t="inlineStr">
         <is>
           <t>4305671729</t>
         </is>
       </c>
-      <c r="B47" s="23" t="inlineStr">
+      <c r="B47" s="25" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3496,12 +3502,12 @@
           <t>DoD SkillBridge Internship/Fellowship Opportunity Application (U.S. Military Only)</t>
         </is>
       </c>
-      <c r="D47" s="23" t="inlineStr">
+      <c r="D47" s="25" t="inlineStr">
         <is>
           <t>Onsights</t>
         </is>
       </c>
-      <c r="E47" s="23" t="inlineStr">
+      <c r="E47" s="25" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -3516,12 +3522,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H47" s="23" t="inlineStr">
+      <c r="H47" s="25" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="I47" s="23" t="inlineStr">
+      <c r="I47" s="25" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -3536,20 +3542,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L47" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M47" s="23" t="inlineStr"/>
+      <c r="L47" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M47" s="25" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="22" t="inlineStr">
+      <c r="A48" s="24" t="inlineStr">
         <is>
           <t>4414096220</t>
         </is>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B48" s="24" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3559,12 +3565,12 @@
           <t>Visualization Engineer Intern</t>
         </is>
       </c>
-      <c r="D48" s="22" t="inlineStr">
+      <c r="D48" s="24" t="inlineStr">
         <is>
           <t>Leidos</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr">
+      <c r="E48" s="24" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3579,12 +3585,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H48" s="22" t="inlineStr">
+      <c r="H48" s="24" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="I48" s="22" t="inlineStr">
+      <c r="I48" s="24" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3599,20 +3605,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L48" s="22" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M48" s="22" t="inlineStr"/>
+      <c r="L48" s="24" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M48" s="24" t="inlineStr"/>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="23" t="inlineStr">
+      <c r="A49" s="25" t="inlineStr">
         <is>
           <t>4361076044</t>
         </is>
       </c>
-      <c r="B49" s="23" t="inlineStr">
+      <c r="B49" s="25" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3622,12 +3628,12 @@
           <t>GenAI Engineering Intern  - SkillBridge (Remote)</t>
         </is>
       </c>
-      <c r="D49" s="23" t="inlineStr">
+      <c r="D49" s="25" t="inlineStr">
         <is>
           <t>CrowdStrike</t>
         </is>
       </c>
-      <c r="E49" s="23" t="inlineStr">
+      <c r="E49" s="25" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3642,12 +3648,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H49" s="23" t="inlineStr">
+      <c r="H49" s="25" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I49" s="23" t="inlineStr">
+      <c r="I49" s="25" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3662,12 +3668,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L49" s="23" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M49" s="23" t="inlineStr"/>
+      <c r="L49" s="25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M49" s="25" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="24" t="inlineStr">
@@ -4362,8 +4368,1331 @@
       </c>
       <c r="M60" s="24" t="inlineStr"/>
     </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="26" t="inlineStr">
+        <is>
+          <t>4413699205</t>
+        </is>
+      </c>
+      <c r="B61" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>Junior Software Engineer - Automation &amp; Integration</t>
+        </is>
+      </c>
+      <c r="D61" s="26" t="inlineStr">
+        <is>
+          <t>Fletcher Development LLC</t>
+        </is>
+      </c>
+      <c r="E61" s="26" t="inlineStr">
+        <is>
+          <t>Redding, CT</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>48%</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H61" s="26" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="I61" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J61" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, rest, api, git, sql, backend, Title match: Junior Software Engineer - Automation &amp; Integration</t>
+        </is>
+      </c>
+      <c r="K61" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L61" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M61" s="26" t="inlineStr"/>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="27" t="inlineStr">
+        <is>
+          <t>4416171988</t>
+        </is>
+      </c>
+      <c r="B62" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D62" s="27" t="inlineStr">
+        <is>
+          <t>Altec</t>
+        </is>
+      </c>
+      <c r="E62" s="27" t="inlineStr">
+        <is>
+          <t>Birmingham, AL</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="G62" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H62" s="27" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I62" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>Skills: api, sql, c, agile, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K62" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L62" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M62" s="27" t="inlineStr"/>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="26" t="inlineStr">
+        <is>
+          <t>4403444963</t>
+        </is>
+      </c>
+      <c r="B63" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>Junior Applications Developer (NY HELPS) #2026-252</t>
+        </is>
+      </c>
+      <c r="D63" s="26" t="inlineStr">
+        <is>
+          <t>Capital Region BOCES</t>
+        </is>
+      </c>
+      <c r="E63" s="26" t="inlineStr">
+        <is>
+          <t>Albany, NY</t>
+        </is>
+      </c>
+      <c r="F63" s="14" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="inlineStr">
+        <is>
+          <t>Very Low</t>
+        </is>
+      </c>
+      <c r="H63" s="26" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I63" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J63" s="8" t="inlineStr">
+        <is>
+          <t>Skills: c</t>
+        </is>
+      </c>
+      <c r="K63" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L63" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M63" s="26" t="inlineStr"/>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="27" t="inlineStr">
+        <is>
+          <t>4418506121</t>
+        </is>
+      </c>
+      <c r="B64" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Core System Junior Developer</t>
+        </is>
+      </c>
+      <c r="D64" s="27" t="inlineStr">
+        <is>
+          <t>Cyprus Federal Credit Union</t>
+        </is>
+      </c>
+      <c r="E64" s="27" t="inlineStr">
+        <is>
+          <t>West Jordan, UT</t>
+        </is>
+      </c>
+      <c r="F64" s="18" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="G64" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H64" s="27" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
+      </c>
+      <c r="I64" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, api, sql, c, Title match: Core System Junior Developer</t>
+        </is>
+      </c>
+      <c r="K64" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L64" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M64" s="27" t="inlineStr"/>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="26" t="inlineStr">
+        <is>
+          <t>4413905706</t>
+        </is>
+      </c>
+      <c r="B65" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="D65" s="26" t="inlineStr">
+        <is>
+          <t>Arnex Solutions LLC</t>
+        </is>
+      </c>
+      <c r="E65" s="26" t="inlineStr">
+        <is>
+          <t>Princeton, NJ</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="G65" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H65" s="26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="I65" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J65" s="8" t="inlineStr">
+        <is>
+          <t>Skills: javascript, html, css, sql, c, agile, Title match: Software Developer</t>
+        </is>
+      </c>
+      <c r="K65" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L65" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M65" s="26" t="inlineStr"/>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="27" t="inlineStr">
+        <is>
+          <t>4418963446</t>
+        </is>
+      </c>
+      <c r="B66" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Junior Software Engineer - Automation &amp; Integration</t>
+        </is>
+      </c>
+      <c r="D66" s="27" t="inlineStr">
+        <is>
+          <t>Vibrant Building Technologies</t>
+        </is>
+      </c>
+      <c r="E66" s="27" t="inlineStr">
+        <is>
+          <t>Ridgefield, CT</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>48%</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H66" s="27" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="I66" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, rest, api, git, sql, backend, Title match: Junior Software Engineer - Automation &amp; Integration</t>
+        </is>
+      </c>
+      <c r="K66" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L66" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M66" s="27" t="inlineStr"/>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="26" t="inlineStr">
+        <is>
+          <t>4413759052</t>
+        </is>
+      </c>
+      <c r="B67" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>Junior Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="D67" s="26" t="inlineStr">
+        <is>
+          <t>Allied World Reinsurance Company</t>
+        </is>
+      </c>
+      <c r="E67" s="26" t="inlineStr">
+        <is>
+          <t>Iselin, NJ</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H67" s="26" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I67" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J67" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, react, node, aws, api, Title match: Junior Full Stack Developer</t>
+        </is>
+      </c>
+      <c r="K67" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L67" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M67" s="26" t="inlineStr"/>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="27" t="inlineStr">
+        <is>
+          <t>4417542502</t>
+        </is>
+      </c>
+      <c r="B68" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Junior Developer</t>
+        </is>
+      </c>
+      <c r="D68" s="27" t="inlineStr">
+        <is>
+          <t>CloudMasonry</t>
+        </is>
+      </c>
+      <c r="E68" s="27" t="inlineStr">
+        <is>
+          <t>Indianapolis, IN</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H68" s="27" t="inlineStr">
+        <is>
+          <t>154</t>
+        </is>
+      </c>
+      <c r="I68" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, node, rest, api, html, Title match: Junior Developer</t>
+        </is>
+      </c>
+      <c r="K68" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L68" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M68" s="27" t="inlineStr"/>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="26" t="inlineStr">
+        <is>
+          <t>4374856035</t>
+        </is>
+      </c>
+      <c r="B69" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>Programmer II</t>
+        </is>
+      </c>
+      <c r="D69" s="26" t="inlineStr">
+        <is>
+          <t>Willis Knighton Health</t>
+        </is>
+      </c>
+      <c r="E69" s="26" t="inlineStr">
+        <is>
+          <t>Louisiana, United States</t>
+        </is>
+      </c>
+      <c r="F69" s="14" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="G69" s="15" t="inlineStr">
+        <is>
+          <t>Very Low</t>
+        </is>
+      </c>
+      <c r="H69" s="26" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="I69" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J69" s="8" t="inlineStr">
+        <is>
+          <t>Skills: c</t>
+        </is>
+      </c>
+      <c r="K69" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L69" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M69" s="26" t="inlineStr"/>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="27" t="inlineStr">
+        <is>
+          <t>4416302564</t>
+        </is>
+      </c>
+      <c r="B70" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer I</t>
+        </is>
+      </c>
+      <c r="D70" s="27" t="inlineStr">
+        <is>
+          <t>American Express</t>
+        </is>
+      </c>
+      <c r="E70" s="27" t="inlineStr">
+        <is>
+          <t>Sunrise, FL</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H70" s="27" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I70" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, react, aws, rest, api, docker, Title match: Software Engineer I</t>
+        </is>
+      </c>
+      <c r="K70" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L70" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M70" s="27" t="inlineStr"/>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="26" t="inlineStr">
+        <is>
+          <t>4417014137</t>
+        </is>
+      </c>
+      <c r="B71" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Junior Software Developer, Applications</t>
+        </is>
+      </c>
+      <c r="D71" s="26" t="inlineStr">
+        <is>
+          <t>ECS</t>
+        </is>
+      </c>
+      <c r="E71" s="26" t="inlineStr">
+        <is>
+          <t>O'Fallon, IL</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H71" s="26" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="I71" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J71" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, docker, git, sql, Title match: Junior Software Developer, Applications</t>
+        </is>
+      </c>
+      <c r="K71" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L71" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M71" s="26" t="inlineStr"/>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="27" t="inlineStr">
+        <is>
+          <t>4381211472</t>
+        </is>
+      </c>
+      <c r="B72" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Programmer</t>
+        </is>
+      </c>
+      <c r="D72" s="27" t="inlineStr">
+        <is>
+          <t>City of New York</t>
+        </is>
+      </c>
+      <c r="E72" s="27" t="inlineStr">
+        <is>
+          <t>Bronx, NY</t>
+        </is>
+      </c>
+      <c r="F72" s="14" t="inlineStr">
+        <is>
+          <t>24%</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="inlineStr">
+        <is>
+          <t>Very Low</t>
+        </is>
+      </c>
+      <c r="H72" s="27" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="I72" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>Skills: javascript, react, html, sql, c, agile</t>
+        </is>
+      </c>
+      <c r="K72" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L72" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M72" s="27" t="inlineStr"/>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="26" t="inlineStr">
+        <is>
+          <t>4168416236</t>
+        </is>
+      </c>
+      <c r="B73" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D73" s="26" t="inlineStr">
+        <is>
+          <t>Interclypse</t>
+        </is>
+      </c>
+      <c r="E73" s="26" t="inlineStr">
+        <is>
+          <t>San Antonio, TX</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H73" s="26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="I73" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J73" s="8" t="inlineStr">
+        <is>
+          <t>Skills: javascript, react, mongodb, sql, full stack, backend, Title match: Software Engineer</t>
+        </is>
+      </c>
+      <c r="K73" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L73" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M73" s="26" t="inlineStr"/>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="27" t="inlineStr">
+        <is>
+          <t>4403507357</t>
+        </is>
+      </c>
+      <c r="B74" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Software Developer:</t>
+        </is>
+      </c>
+      <c r="D74" s="27" t="inlineStr">
+        <is>
+          <t>IQuest Solutions Corporation</t>
+        </is>
+      </c>
+      <c r="E74" s="27" t="inlineStr">
+        <is>
+          <t>Plano, TX</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="G74" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H74" s="27" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="I74" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>Skills: aws, rest, api, c, Title match: Software Developer:</t>
+        </is>
+      </c>
+      <c r="K74" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L74" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M74" s="27" t="inlineStr"/>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="26" t="inlineStr">
+        <is>
+          <t>4309800238</t>
+        </is>
+      </c>
+      <c r="B75" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Backend Software Engineer</t>
+        </is>
+      </c>
+      <c r="D75" s="26" t="inlineStr">
+        <is>
+          <t>DataAnnotation</t>
+        </is>
+      </c>
+      <c r="E75" s="26" t="inlineStr">
+        <is>
+          <t>Texas, United States</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>76%</t>
+        </is>
+      </c>
+      <c r="G75" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H75" s="26" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I75" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J75" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, html, sql, backend, c++, Location: Texas, United States, Title match: Backend Software Engineer</t>
+        </is>
+      </c>
+      <c r="K75" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L75" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M75" s="26" t="inlineStr"/>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="27" t="inlineStr">
+        <is>
+          <t>4404109089</t>
+        </is>
+      </c>
+      <c r="B76" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Software Development Engineer I</t>
+        </is>
+      </c>
+      <c r="D76" s="27" t="inlineStr">
+        <is>
+          <t>GM Financial</t>
+        </is>
+      </c>
+      <c r="E76" s="27" t="inlineStr">
+        <is>
+          <t>Arlington, TX</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="G76" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H76" s="27" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I76" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>Skills: javascript, node, api, css, docker, git</t>
+        </is>
+      </c>
+      <c r="K76" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L76" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M76" s="27" t="inlineStr"/>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="26" t="inlineStr">
+        <is>
+          <t>3986116411</t>
+        </is>
+      </c>
+      <c r="B77" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D77" s="26" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="E77" s="26" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H77" s="26" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I77" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J77" s="8" t="inlineStr">
+        <is>
+          <t>Skills: rest, api, machine learning, c, Location: Austin, TX, Title match: Software Engineer</t>
+        </is>
+      </c>
+      <c r="K77" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L77" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M77" s="26" t="inlineStr"/>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="27" t="inlineStr">
+        <is>
+          <t>4418051524</t>
+        </is>
+      </c>
+      <c r="B78" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D78" s="27" t="inlineStr">
+        <is>
+          <t>Relativity</t>
+        </is>
+      </c>
+      <c r="E78" s="27" t="inlineStr">
+        <is>
+          <t>Texas, United States</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>64%</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H78" s="27" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I78" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, api, git, backend, c, llm, Location: Texas, United States, Title match: Software Engineer</t>
+        </is>
+      </c>
+      <c r="K78" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L78" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M78" s="27" t="inlineStr"/>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="26" t="inlineStr">
+        <is>
+          <t>4409856693</t>
+        </is>
+      </c>
+      <c r="B79" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>Software Engineer - Payments</t>
+        </is>
+      </c>
+      <c r="D79" s="26" t="inlineStr">
+        <is>
+          <t>Cloudbeds</t>
+        </is>
+      </c>
+      <c r="E79" s="26" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>76%</t>
+        </is>
+      </c>
+      <c r="G79" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H79" s="26" t="inlineStr">
+        <is>
+          <t>177</t>
+        </is>
+      </c>
+      <c r="I79" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J79" s="8" t="inlineStr">
+        <is>
+          <t>Skills: aws, api, docker, git, sql, machine learning, Location: Austin, TX, Title match: Software Engineer - Payments</t>
+        </is>
+      </c>
+      <c r="K79" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L79" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M79" s="26" t="inlineStr"/>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="27" t="inlineStr">
+        <is>
+          <t>3986111771</t>
+        </is>
+      </c>
+      <c r="B80" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D80" s="27" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="E80" s="27" t="inlineStr">
+        <is>
+          <t>Carrollton, TX</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="G80" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H80" s="27" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I80" s="27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>Skills: rest, api, machine learning, c, Title match: Software Engineer</t>
+        </is>
+      </c>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L80" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M80" s="27" t="inlineStr"/>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="26" t="inlineStr">
+        <is>
+          <t>4417160720</t>
+        </is>
+      </c>
+      <c r="B81" s="26" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Full-Stack AI Developer</t>
+        </is>
+      </c>
+      <c r="D81" s="26" t="inlineStr">
+        <is>
+          <t>AnswerMyQ</t>
+        </is>
+      </c>
+      <c r="E81" s="26" t="inlineStr">
+        <is>
+          <t>Austin, Texas Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H81" s="26" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I81" s="26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J81" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, react, aws, git, full-stack, backend, Location: Austin, Texas Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="K81" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L81" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M81" s="26" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M60"/>
+  <autoFilter ref="A1:M81"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -4424,6 +5753,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-05-28
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Matches'!$A$1:$M$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -199,6 +199,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -566,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M81"/>
+  <dimension ref="A1:M87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -652,12 +658,12 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>4406952064</t>
         </is>
       </c>
-      <c r="B2" s="24" t="inlineStr">
+      <c r="B2" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -667,12 +673,12 @@
           <t>DevSecOps Intern</t>
         </is>
       </c>
-      <c r="D2" s="24" t="inlineStr">
+      <c r="D2" s="27" t="inlineStr">
         <is>
           <t>Modern Technology Solutions, Inc. (MTSI)</t>
         </is>
       </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="E2" s="27" t="inlineStr">
         <is>
           <t>Huntsville, AL</t>
         </is>
@@ -687,12 +693,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H2" s="24" t="inlineStr">
+      <c r="H2" s="27" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="I2" s="24" t="inlineStr">
+      <c r="I2" s="27" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -707,20 +713,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L2" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M2" s="24" t="inlineStr"/>
+      <c r="L2" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M2" s="27" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>4405630173</t>
         </is>
       </c>
-      <c r="B3" s="25" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -730,12 +736,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D3" s="25" t="inlineStr">
+      <c r="D3" s="26" t="inlineStr">
         <is>
           <t>DLRdmv®</t>
         </is>
       </c>
-      <c r="E3" s="25" t="inlineStr">
+      <c r="E3" s="26" t="inlineStr">
         <is>
           <t>Dallas, TX</t>
         </is>
@@ -750,12 +756,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H3" s="25" t="inlineStr">
+      <c r="H3" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I3" s="25" t="inlineStr">
+      <c r="I3" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -770,20 +776,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L3" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M3" s="25" t="inlineStr"/>
+      <c r="L3" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M3" s="26" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>4287414862</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -793,12 +799,12 @@
           <t>[Online Assessment]Software Development Engineer Intern (Network Automation)- 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="27" t="inlineStr">
         <is>
           <t>ByteDance</t>
         </is>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="27" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -813,12 +819,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="H4" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I4" s="24" t="inlineStr">
+      <c r="I4" s="27" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -833,20 +839,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L4" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M4" s="24" t="inlineStr"/>
+      <c r="L4" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M4" s="27" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>4309805269</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -856,12 +862,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Delaware, United States</t>
         </is>
@@ -876,12 +882,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>81</t>
         </is>
       </c>
-      <c r="I5" s="25" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -896,20 +902,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L5" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M5" s="25" t="inlineStr"/>
+      <c r="L5" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M5" s="26" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>4371812987</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -919,12 +925,12 @@
           <t>Software Development Engineer Fall Intern - Military Veteran</t>
         </is>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="27" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -939,12 +945,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="H6" s="27" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="I6" s="24" t="inlineStr">
+      <c r="I6" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -959,20 +965,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L6" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M6" s="24" t="inlineStr"/>
+      <c r="L6" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M6" s="27" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>4274682122</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -982,12 +988,12 @@
           <t>Software Engineer Intern (Data Ecosystem) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D7" s="25" t="inlineStr">
+      <c r="D7" s="26" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E7" s="25" t="inlineStr">
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1002,12 +1008,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="25" t="inlineStr">
+      <c r="H7" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I7" s="25" t="inlineStr">
+      <c r="I7" s="26" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1022,20 +1028,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L7" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M7" s="25" t="inlineStr"/>
+      <c r="L7" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M7" s="26" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>4283848614</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1045,12 +1051,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Fall (BS/ MS)</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="27" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E8" s="24" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1065,12 +1071,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H8" s="24" t="inlineStr">
+      <c r="H8" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I8" s="24" t="inlineStr">
+      <c r="I8" s="27" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1085,20 +1091,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L8" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M8" s="24" t="inlineStr"/>
+      <c r="L8" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M8" s="27" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>4411790844</t>
         </is>
       </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1108,12 +1114,12 @@
           <t>Software Engineer Intern (Infrastructure Automation) - Fall 2026</t>
         </is>
       </c>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="D9" s="26" t="inlineStr">
         <is>
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E9" s="25" t="inlineStr">
+      <c r="E9" s="26" t="inlineStr">
         <is>
           <t>Bellevue, WA</t>
         </is>
@@ -1128,12 +1134,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H9" s="25" t="inlineStr">
+      <c r="H9" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I9" s="25" t="inlineStr">
+      <c r="I9" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1148,20 +1154,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L9" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M9" s="25" t="inlineStr"/>
+      <c r="L9" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M9" s="26" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>4332425058</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1171,12 +1177,12 @@
           <t>Software Development Engineer Internship - Fall 2026 (US)</t>
         </is>
       </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="D10" s="27" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1191,12 +1197,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H10" s="24" t="inlineStr">
+      <c r="H10" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I10" s="24" t="inlineStr">
+      <c r="I10" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1211,20 +1217,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L10" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M10" s="24" t="inlineStr"/>
+      <c r="L10" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M10" s="27" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>4323643644</t>
         </is>
       </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1234,12 +1240,12 @@
           <t>[Online Assessment] Software Engineer Intern (Recommendation Infrastructure) - 2026 Summer (BS/ MS)</t>
         </is>
       </c>
-      <c r="D11" s="25" t="inlineStr">
+      <c r="D11" s="26" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E11" s="25" t="inlineStr">
+      <c r="E11" s="26" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1254,12 +1260,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H11" s="25" t="inlineStr">
+      <c r="H11" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I11" s="25" t="inlineStr">
+      <c r="I11" s="26" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1274,20 +1280,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L11" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M11" s="25" t="inlineStr"/>
+      <c r="L11" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M11" s="26" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>4320849104</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1297,12 +1303,12 @@
           <t>Software Engineer Intern (Commerce Ads) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D12" s="24" t="inlineStr">
+      <c r="D12" s="27" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E12" s="24" t="inlineStr">
+      <c r="E12" s="27" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1317,12 +1323,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H12" s="24" t="inlineStr">
+      <c r="H12" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I12" s="24" t="inlineStr">
+      <c r="I12" s="27" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -1337,20 +1343,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L12" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M12" s="24" t="inlineStr"/>
+      <c r="L12" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M12" s="27" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="25" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>4401686051</t>
         </is>
       </c>
-      <c r="B13" s="25" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1360,12 +1366,12 @@
           <t>Front End Software Engineer</t>
         </is>
       </c>
-      <c r="D13" s="25" t="inlineStr">
+      <c r="D13" s="26" t="inlineStr">
         <is>
           <t>Saronic Technologies</t>
         </is>
       </c>
-      <c r="E13" s="25" t="inlineStr">
+      <c r="E13" s="26" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
@@ -1380,12 +1386,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H13" s="25" t="inlineStr">
+      <c r="H13" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I13" s="25" t="inlineStr">
+      <c r="I13" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1400,20 +1406,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L13" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M13" s="25" t="inlineStr"/>
+      <c r="L13" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M13" s="26" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>4309696652</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1423,12 +1429,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D14" s="24" t="inlineStr">
+      <c r="D14" s="27" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E14" s="24" t="inlineStr">
+      <c r="E14" s="27" t="inlineStr">
         <is>
           <t>Rhode Island, United States</t>
         </is>
@@ -1443,12 +1449,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H14" s="24" t="inlineStr">
+      <c r="H14" s="27" t="inlineStr">
         <is>
           <t>114</t>
         </is>
       </c>
-      <c r="I14" s="24" t="inlineStr">
+      <c r="I14" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1463,20 +1469,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L14" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M14" s="24" t="inlineStr"/>
+      <c r="L14" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M14" s="27" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>4309804319</t>
         </is>
       </c>
-      <c r="B15" s="25" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1486,12 +1492,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D15" s="25" t="inlineStr">
+      <c r="D15" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E15" s="25" t="inlineStr">
+      <c r="E15" s="26" t="inlineStr">
         <is>
           <t>Colorado, United States</t>
         </is>
@@ -1506,12 +1512,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H15" s="25" t="inlineStr">
+      <c r="H15" s="26" t="inlineStr">
         <is>
           <t>91</t>
         </is>
       </c>
-      <c r="I15" s="25" t="inlineStr">
+      <c r="I15" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1526,20 +1532,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L15" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M15" s="25" t="inlineStr"/>
+      <c r="L15" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M15" s="26" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>4410271532</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1549,12 +1555,12 @@
           <t>Associate Developer</t>
         </is>
       </c>
-      <c r="D16" s="24" t="inlineStr">
+      <c r="D16" s="27" t="inlineStr">
         <is>
           <t>HealthStream</t>
         </is>
       </c>
-      <c r="E16" s="24" t="inlineStr">
+      <c r="E16" s="27" t="inlineStr">
         <is>
           <t>Nashville, TN</t>
         </is>
@@ -1569,12 +1575,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H16" s="24" t="inlineStr">
+      <c r="H16" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I16" s="24" t="inlineStr">
+      <c r="I16" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1589,20 +1595,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L16" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M16" s="24" t="inlineStr"/>
+      <c r="L16" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M16" s="27" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="25" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>4304445726</t>
         </is>
       </c>
-      <c r="B17" s="25" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1612,12 +1618,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D17" s="25" t="inlineStr">
+      <c r="D17" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E17" s="25" t="inlineStr">
+      <c r="E17" s="26" t="inlineStr">
         <is>
           <t>Oregon, United States</t>
         </is>
@@ -1632,12 +1638,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H17" s="25" t="inlineStr">
+      <c r="H17" s="26" t="inlineStr">
         <is>
           <t>115</t>
         </is>
       </c>
-      <c r="I17" s="25" t="inlineStr">
+      <c r="I17" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1652,20 +1658,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L17" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M17" s="25" t="inlineStr"/>
+      <c r="L17" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M17" s="26" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>4342036151</t>
         </is>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1675,12 +1681,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D18" s="24" t="inlineStr">
+      <c r="D18" s="27" t="inlineStr">
         <is>
           <t>Modern Treasury</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="27" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -1695,12 +1701,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H18" s="24" t="inlineStr">
+      <c r="H18" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I18" s="24" t="inlineStr">
+      <c r="I18" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1715,20 +1721,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L18" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M18" s="24" t="inlineStr"/>
+      <c r="L18" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M18" s="27" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>4304441843</t>
         </is>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1738,12 +1744,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D19" s="25" t="inlineStr">
+      <c r="D19" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E19" s="25" t="inlineStr">
+      <c r="E19" s="26" t="inlineStr">
         <is>
           <t>Idaho, United States</t>
         </is>
@@ -1758,12 +1764,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H19" s="25" t="inlineStr">
+      <c r="H19" s="26" t="inlineStr">
         <is>
           <t>157</t>
         </is>
       </c>
-      <c r="I19" s="25" t="inlineStr">
+      <c r="I19" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1778,20 +1784,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L19" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M19" s="25" t="inlineStr"/>
+      <c r="L19" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M19" s="26" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>4408047047</t>
         </is>
       </c>
-      <c r="B20" s="24" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1801,12 +1807,12 @@
           <t>Computer Sciences - Graduates - AI Training - Las Vegas, US</t>
         </is>
       </c>
-      <c r="D20" s="24" t="inlineStr">
+      <c r="D20" s="27" t="inlineStr">
         <is>
           <t>Prolific</t>
         </is>
       </c>
-      <c r="E20" s="24" t="inlineStr">
+      <c r="E20" s="27" t="inlineStr">
         <is>
           <t>Las Vegas, NV</t>
         </is>
@@ -1821,12 +1827,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H20" s="24" t="inlineStr">
+      <c r="H20" s="27" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="I20" s="24" t="inlineStr">
+      <c r="I20" s="27" t="inlineStr">
         <is>
           <t>Temporary</t>
         </is>
@@ -1841,20 +1847,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L20" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M20" s="24" t="inlineStr"/>
+      <c r="L20" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M20" s="27" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>4304444837</t>
         </is>
       </c>
-      <c r="B21" s="25" t="inlineStr">
+      <c r="B21" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1864,12 +1870,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D21" s="25" t="inlineStr">
+      <c r="D21" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E21" s="25" t="inlineStr">
+      <c r="E21" s="26" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -1884,12 +1890,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H21" s="25" t="inlineStr">
+      <c r="H21" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I21" s="25" t="inlineStr">
+      <c r="I21" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1904,20 +1910,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L21" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M21" s="25" t="inlineStr"/>
+      <c r="L21" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M21" s="26" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="27" t="inlineStr">
         <is>
           <t>4405641326</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1927,12 +1933,12 @@
           <t>Full-stack Engineer</t>
         </is>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D22" s="27" t="inlineStr">
         <is>
           <t>PartnerTap</t>
         </is>
       </c>
-      <c r="E22" s="24" t="inlineStr">
+      <c r="E22" s="27" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1947,12 +1953,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H22" s="24" t="inlineStr">
+      <c r="H22" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I22" s="24" t="inlineStr">
+      <c r="I22" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -1967,20 +1973,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L22" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M22" s="24" t="inlineStr"/>
+      <c r="L22" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M22" s="27" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>4341020900</t>
         </is>
       </c>
-      <c r="B23" s="25" t="inlineStr">
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1990,12 +1996,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D23" s="25" t="inlineStr">
+      <c r="D23" s="26" t="inlineStr">
         <is>
           <t>PlanIT Group, LLC</t>
         </is>
       </c>
-      <c r="E23" s="25" t="inlineStr">
+      <c r="E23" s="26" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -2010,12 +2016,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H23" s="25" t="inlineStr">
+      <c r="H23" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I23" s="25" t="inlineStr">
+      <c r="I23" s="26" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
@@ -2030,20 +2036,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L23" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M23" s="25" t="inlineStr"/>
+      <c r="L23" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M23" s="26" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="27" t="inlineStr">
         <is>
           <t>4304450637</t>
         </is>
       </c>
-      <c r="B24" s="24" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2053,12 +2059,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D24" s="24" t="inlineStr">
+      <c r="D24" s="27" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E24" s="24" t="inlineStr">
+      <c r="E24" s="27" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2073,12 +2079,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H24" s="24" t="inlineStr">
+      <c r="H24" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I24" s="24" t="inlineStr">
+      <c r="I24" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2093,20 +2099,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L24" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M24" s="24" t="inlineStr"/>
+      <c r="L24" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M24" s="27" t="inlineStr"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>4304451654</t>
         </is>
       </c>
-      <c r="B25" s="25" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2116,12 +2122,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D25" s="25" t="inlineStr">
+      <c r="D25" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E25" s="25" t="inlineStr">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>Utah, United States</t>
         </is>
@@ -2136,12 +2142,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H25" s="25" t="inlineStr">
+      <c r="H25" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I25" s="25" t="inlineStr">
+      <c r="I25" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2156,20 +2162,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L25" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M25" s="25" t="inlineStr"/>
+      <c r="L25" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M25" s="26" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="24" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>4413745880</t>
         </is>
       </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2179,12 +2185,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D26" s="24" t="inlineStr">
+      <c r="D26" s="27" t="inlineStr">
         <is>
           <t>Crate &amp; Barrel</t>
         </is>
       </c>
-      <c r="E26" s="24" t="inlineStr">
+      <c r="E26" s="27" t="inlineStr">
         <is>
           <t>Northbrook, IL</t>
         </is>
@@ -2199,12 +2205,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H26" s="24" t="inlineStr">
+      <c r="H26" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I26" s="24" t="inlineStr">
+      <c r="I26" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2219,20 +2225,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L26" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M26" s="24" t="inlineStr"/>
+      <c r="L26" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M26" s="27" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="25" t="inlineStr">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>4304438841</t>
         </is>
       </c>
-      <c r="B27" s="25" t="inlineStr">
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2242,12 +2248,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D27" s="25" t="inlineStr">
+      <c r="D27" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E27" s="25" t="inlineStr">
+      <c r="E27" s="26" t="inlineStr">
         <is>
           <t>Connecticut, United States</t>
         </is>
@@ -2262,12 +2268,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H27" s="25" t="inlineStr">
+      <c r="H27" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I27" s="25" t="inlineStr">
+      <c r="I27" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2282,20 +2288,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L27" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M27" s="25" t="inlineStr"/>
+      <c r="L27" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M27" s="26" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="24" t="inlineStr">
+      <c r="A28" s="27" t="inlineStr">
         <is>
           <t>4393215930</t>
         </is>
       </c>
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2305,12 +2311,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D28" s="24" t="inlineStr">
+      <c r="D28" s="27" t="inlineStr">
         <is>
           <t>Transcend</t>
         </is>
       </c>
-      <c r="E28" s="24" t="inlineStr">
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>California, United States</t>
         </is>
@@ -2325,12 +2331,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H28" s="24" t="inlineStr">
+      <c r="H28" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I28" s="24" t="inlineStr">
+      <c r="I28" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2345,20 +2351,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L28" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M28" s="24" t="inlineStr"/>
+      <c r="L28" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M28" s="27" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="25" t="inlineStr">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>4304445723</t>
         </is>
       </c>
-      <c r="B29" s="25" t="inlineStr">
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2368,12 +2374,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D29" s="25" t="inlineStr">
+      <c r="D29" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E29" s="25" t="inlineStr">
+      <c r="E29" s="26" t="inlineStr">
         <is>
           <t>Illinois, United States</t>
         </is>
@@ -2388,12 +2394,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H29" s="25" t="inlineStr">
+      <c r="H29" s="26" t="inlineStr">
         <is>
           <t>198</t>
         </is>
       </c>
-      <c r="I29" s="25" t="inlineStr">
+      <c r="I29" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2408,20 +2414,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L29" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M29" s="25" t="inlineStr"/>
+      <c r="L29" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M29" s="26" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="24" t="inlineStr">
+      <c r="A30" s="27" t="inlineStr">
         <is>
           <t>4396380649</t>
         </is>
       </c>
-      <c r="B30" s="24" t="inlineStr">
+      <c r="B30" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2431,12 +2437,12 @@
           <t>Full-Stack Developer Intern, Music &amp; Audio</t>
         </is>
       </c>
-      <c r="D30" s="24" t="inlineStr">
+      <c r="D30" s="27" t="inlineStr">
         <is>
           <t>Melotech</t>
         </is>
       </c>
-      <c r="E30" s="24" t="inlineStr">
+      <c r="E30" s="27" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
@@ -2451,12 +2457,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H30" s="24" t="inlineStr">
+      <c r="H30" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I30" s="24" t="inlineStr">
+      <c r="I30" s="27" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -2471,20 +2477,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L30" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M30" s="24" t="inlineStr"/>
+      <c r="L30" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M30" s="27" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="25" t="inlineStr">
+      <c r="A31" s="26" t="inlineStr">
         <is>
           <t>4304454025</t>
         </is>
       </c>
-      <c r="B31" s="25" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2494,12 +2500,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D31" s="25" t="inlineStr">
+      <c r="D31" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E31" s="25" t="inlineStr">
+      <c r="E31" s="26" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -2514,12 +2520,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H31" s="25" t="inlineStr">
+      <c r="H31" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I31" s="25" t="inlineStr">
+      <c r="I31" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2534,20 +2540,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L31" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M31" s="25" t="inlineStr"/>
+      <c r="L31" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M31" s="26" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="24" t="inlineStr">
+      <c r="A32" s="27" t="inlineStr">
         <is>
           <t>4309802287</t>
         </is>
       </c>
-      <c r="B32" s="24" t="inlineStr">
+      <c r="B32" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2557,12 +2563,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D32" s="24" t="inlineStr">
+      <c r="D32" s="27" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E32" s="24" t="inlineStr">
+      <c r="E32" s="27" t="inlineStr">
         <is>
           <t>New Jersey, United States</t>
         </is>
@@ -2577,12 +2583,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H32" s="24" t="inlineStr">
+      <c r="H32" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I32" s="24" t="inlineStr">
+      <c r="I32" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2597,20 +2603,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L32" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M32" s="24" t="inlineStr"/>
+      <c r="L32" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M32" s="27" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="25" t="inlineStr">
+      <c r="A33" s="26" t="inlineStr">
         <is>
           <t>4309694880</t>
         </is>
       </c>
-      <c r="B33" s="25" t="inlineStr">
+      <c r="B33" s="26" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2620,12 +2626,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D33" s="25" t="inlineStr">
+      <c r="D33" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E33" s="25" t="inlineStr">
+      <c r="E33" s="26" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -2640,12 +2646,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H33" s="25" t="inlineStr">
+      <c r="H33" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I33" s="25" t="inlineStr">
+      <c r="I33" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2660,20 +2666,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L33" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M33" s="25" t="inlineStr"/>
+      <c r="L33" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M33" s="26" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
+      <c r="A34" s="27" t="inlineStr">
         <is>
           <t>4411274012</t>
         </is>
       </c>
-      <c r="B34" s="24" t="inlineStr">
+      <c r="B34" s="27" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2683,12 +2689,12 @@
           <t>Junior UI Developer</t>
         </is>
       </c>
-      <c r="D34" s="24" t="inlineStr">
+      <c r="D34" s="27" t="inlineStr">
         <is>
           <t>General Dynamics Information Technology</t>
         </is>
       </c>
-      <c r="E34" s="24" t="inlineStr">
+      <c r="E34" s="27" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -2703,12 +2709,12 @@
           <t>Very Low</t>
         </is>
       </c>
-      <c r="H34" s="24" t="inlineStr">
+      <c r="H34" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I34" s="24" t="inlineStr">
+      <c r="I34" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2723,20 +2729,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L34" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M34" s="24" t="inlineStr"/>
+      <c r="L34" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M34" s="27" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="25" t="inlineStr">
+      <c r="A35" s="26" t="inlineStr">
         <is>
           <t>4264562292</t>
         </is>
       </c>
-      <c r="B35" s="25" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2746,12 +2752,12 @@
           <t>Software Developer</t>
         </is>
       </c>
-      <c r="D35" s="25" t="inlineStr">
+      <c r="D35" s="26" t="inlineStr">
         <is>
           <t>Cymertek Corporation</t>
         </is>
       </c>
-      <c r="E35" s="25" t="inlineStr">
+      <c r="E35" s="26" t="inlineStr">
         <is>
           <t>San Antonio, TX</t>
         </is>
@@ -2766,12 +2772,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H35" s="25" t="inlineStr">
+      <c r="H35" s="26" t="inlineStr">
         <is>
           <t>155</t>
         </is>
       </c>
-      <c r="I35" s="25" t="inlineStr">
+      <c r="I35" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2786,20 +2792,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L35" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M35" s="25" t="inlineStr"/>
+      <c r="L35" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M35" s="26" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
+      <c r="A36" s="27" t="inlineStr">
         <is>
           <t>4417482675</t>
         </is>
       </c>
-      <c r="B36" s="24" t="inlineStr">
+      <c r="B36" s="27" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2809,12 +2815,12 @@
           <t>Software Developer I</t>
         </is>
       </c>
-      <c r="D36" s="24" t="inlineStr">
+      <c r="D36" s="27" t="inlineStr">
         <is>
           <t>El Paso Water</t>
         </is>
       </c>
-      <c r="E36" s="24" t="inlineStr">
+      <c r="E36" s="27" t="inlineStr">
         <is>
           <t>El Paso, TX</t>
         </is>
@@ -2829,12 +2835,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H36" s="24" t="inlineStr">
+      <c r="H36" s="27" t="inlineStr">
         <is>
           <t>61</t>
         </is>
       </c>
-      <c r="I36" s="24" t="inlineStr">
+      <c r="I36" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2849,20 +2855,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L36" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M36" s="24" t="inlineStr"/>
+      <c r="L36" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M36" s="27" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="25" t="inlineStr">
+      <c r="A37" s="26" t="inlineStr">
         <is>
           <t>4416508200</t>
         </is>
       </c>
-      <c r="B37" s="25" t="inlineStr">
+      <c r="B37" s="26" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -2872,12 +2878,12 @@
           <t>Software Development Engineer in Test Intern (Global E-Commerce) - 2026 Summer (BS/MS)</t>
         </is>
       </c>
-      <c r="D37" s="25" t="inlineStr">
+      <c r="D37" s="26" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="E37" s="25" t="inlineStr">
+      <c r="E37" s="26" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -2892,12 +2898,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H37" s="25" t="inlineStr">
+      <c r="H37" s="26" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="I37" s="25" t="inlineStr">
+      <c r="I37" s="26" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -2912,20 +2918,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L37" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M37" s="25" t="inlineStr"/>
+      <c r="L37" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M37" s="26" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="24" t="inlineStr">
+      <c r="A38" s="27" t="inlineStr">
         <is>
           <t>4309809191</t>
         </is>
       </c>
-      <c r="B38" s="24" t="inlineStr">
+      <c r="B38" s="27" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -2935,12 +2941,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D38" s="24" t="inlineStr">
+      <c r="D38" s="27" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E38" s="24" t="inlineStr">
+      <c r="E38" s="27" t="inlineStr">
         <is>
           <t>Ohio, United States</t>
         </is>
@@ -2955,12 +2961,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H38" s="24" t="inlineStr">
+      <c r="H38" s="27" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="I38" s="24" t="inlineStr">
+      <c r="I38" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -2975,20 +2981,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L38" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M38" s="24" t="inlineStr"/>
+      <c r="L38" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M38" s="27" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="25" t="inlineStr">
+      <c r="A39" s="26" t="inlineStr">
         <is>
           <t>3986118096</t>
         </is>
       </c>
-      <c r="B39" s="25" t="inlineStr">
+      <c r="B39" s="26" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -2998,12 +3004,12 @@
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="D39" s="25" t="inlineStr">
+      <c r="D39" s="26" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="E39" s="25" t="inlineStr">
+      <c r="E39" s="26" t="inlineStr">
         <is>
           <t>Irving, TX</t>
         </is>
@@ -3018,12 +3024,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H39" s="25" t="inlineStr">
+      <c r="H39" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I39" s="25" t="inlineStr">
+      <c r="I39" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3038,20 +3044,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L39" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M39" s="25" t="inlineStr"/>
+      <c r="L39" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M39" s="26" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="24" t="inlineStr">
+      <c r="A40" s="27" t="inlineStr">
         <is>
           <t>4309808244</t>
         </is>
       </c>
-      <c r="B40" s="24" t="inlineStr">
+      <c r="B40" s="27" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3061,12 +3067,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D40" s="24" t="inlineStr">
+      <c r="D40" s="27" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E40" s="24" t="inlineStr">
+      <c r="E40" s="27" t="inlineStr">
         <is>
           <t>Massachusetts, United States</t>
         </is>
@@ -3081,12 +3087,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H40" s="24" t="inlineStr">
+      <c r="H40" s="27" t="inlineStr">
         <is>
           <t>166</t>
         </is>
       </c>
-      <c r="I40" s="24" t="inlineStr">
+      <c r="I40" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3101,20 +3107,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L40" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M40" s="24" t="inlineStr"/>
+      <c r="L40" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M40" s="27" t="inlineStr"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="25" t="inlineStr">
+      <c r="A41" s="26" t="inlineStr">
         <is>
           <t>4362173625</t>
         </is>
       </c>
-      <c r="B41" s="25" t="inlineStr">
+      <c r="B41" s="26" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3124,12 +3130,12 @@
           <t>Full Stack Engineer</t>
         </is>
       </c>
-      <c r="D41" s="25" t="inlineStr">
+      <c r="D41" s="26" t="inlineStr">
         <is>
           <t>Empower Sleep</t>
         </is>
       </c>
-      <c r="E41" s="25" t="inlineStr">
+      <c r="E41" s="26" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3144,12 +3150,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H41" s="25" t="inlineStr">
+      <c r="H41" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I41" s="25" t="inlineStr">
+      <c r="I41" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3164,20 +3170,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L41" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M41" s="25" t="inlineStr"/>
+      <c r="L41" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M41" s="26" t="inlineStr"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="24" t="inlineStr">
+      <c r="A42" s="27" t="inlineStr">
         <is>
           <t>4309812093</t>
         </is>
       </c>
-      <c r="B42" s="24" t="inlineStr">
+      <c r="B42" s="27" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3187,12 +3193,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D42" s="24" t="inlineStr">
+      <c r="D42" s="27" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E42" s="24" t="inlineStr">
+      <c r="E42" s="27" t="inlineStr">
         <is>
           <t>Florida, United States</t>
         </is>
@@ -3207,12 +3213,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H42" s="24" t="inlineStr">
+      <c r="H42" s="27" t="inlineStr">
         <is>
           <t>158</t>
         </is>
       </c>
-      <c r="I42" s="24" t="inlineStr">
+      <c r="I42" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3227,20 +3233,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L42" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M42" s="24" t="inlineStr"/>
+      <c r="L42" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M42" s="27" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="25" t="inlineStr">
+      <c r="A43" s="26" t="inlineStr">
         <is>
           <t>4391759914</t>
         </is>
       </c>
-      <c r="B43" s="25" t="inlineStr">
+      <c r="B43" s="26" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3250,12 +3256,12 @@
           <t>QA Engineering Internship</t>
         </is>
       </c>
-      <c r="D43" s="25" t="inlineStr">
+      <c r="D43" s="26" t="inlineStr">
         <is>
           <t>Chartbeat</t>
         </is>
       </c>
-      <c r="E43" s="25" t="inlineStr">
+      <c r="E43" s="26" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
@@ -3270,12 +3276,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H43" s="25" t="inlineStr">
+      <c r="H43" s="26" t="inlineStr">
         <is>
           <t>168</t>
         </is>
       </c>
-      <c r="I43" s="25" t="inlineStr">
+      <c r="I43" s="26" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -3290,20 +3296,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L43" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M43" s="25" t="inlineStr"/>
+      <c r="L43" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M43" s="26" t="inlineStr"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="24" t="inlineStr">
+      <c r="A44" s="27" t="inlineStr">
         <is>
           <t>4412855678</t>
         </is>
       </c>
-      <c r="B44" s="24" t="inlineStr">
+      <c r="B44" s="27" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3313,12 +3319,12 @@
           <t>AI Integration Engineer</t>
         </is>
       </c>
-      <c r="D44" s="24" t="inlineStr">
+      <c r="D44" s="27" t="inlineStr">
         <is>
           <t>UST</t>
         </is>
       </c>
-      <c r="E44" s="24" t="inlineStr">
+      <c r="E44" s="27" t="inlineStr">
         <is>
           <t>Santa Clara, CA</t>
         </is>
@@ -3333,12 +3339,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H44" s="24" t="inlineStr">
+      <c r="H44" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I44" s="24" t="inlineStr">
+      <c r="I44" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3353,20 +3359,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L44" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M44" s="24" t="inlineStr"/>
+      <c r="L44" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M44" s="27" t="inlineStr"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="25" t="inlineStr">
+      <c r="A45" s="26" t="inlineStr">
         <is>
           <t>4309805219</t>
         </is>
       </c>
-      <c r="B45" s="25" t="inlineStr">
+      <c r="B45" s="26" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3376,12 +3382,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D45" s="25" t="inlineStr">
+      <c r="D45" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E45" s="25" t="inlineStr">
+      <c r="E45" s="26" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -3396,12 +3402,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H45" s="25" t="inlineStr">
+      <c r="H45" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I45" s="25" t="inlineStr">
+      <c r="I45" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3416,20 +3422,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L45" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M45" s="25" t="inlineStr"/>
+      <c r="L45" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M45" s="26" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="24" t="inlineStr">
+      <c r="A46" s="27" t="inlineStr">
         <is>
           <t>4409726429</t>
         </is>
       </c>
-      <c r="B46" s="24" t="inlineStr">
+      <c r="B46" s="27" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3439,12 +3445,12 @@
           <t>Data Science Intern</t>
         </is>
       </c>
-      <c r="D46" s="24" t="inlineStr">
+      <c r="D46" s="27" t="inlineStr">
         <is>
           <t>Rundoo</t>
         </is>
       </c>
-      <c r="E46" s="24" t="inlineStr">
+      <c r="E46" s="27" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3459,12 +3465,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H46" s="24" t="inlineStr">
+      <c r="H46" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I46" s="24" t="inlineStr">
+      <c r="I46" s="27" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -3479,20 +3485,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L46" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M46" s="24" t="inlineStr"/>
+      <c r="L46" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M46" s="27" t="inlineStr"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="25" t="inlineStr">
+      <c r="A47" s="26" t="inlineStr">
         <is>
           <t>4305671729</t>
         </is>
       </c>
-      <c r="B47" s="25" t="inlineStr">
+      <c r="B47" s="26" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3502,12 +3508,12 @@
           <t>DoD SkillBridge Internship/Fellowship Opportunity Application (U.S. Military Only)</t>
         </is>
       </c>
-      <c r="D47" s="25" t="inlineStr">
+      <c r="D47" s="26" t="inlineStr">
         <is>
           <t>Onsights</t>
         </is>
       </c>
-      <c r="E47" s="25" t="inlineStr">
+      <c r="E47" s="26" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -3522,12 +3528,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H47" s="25" t="inlineStr">
+      <c r="H47" s="26" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="I47" s="25" t="inlineStr">
+      <c r="I47" s="26" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -3542,20 +3548,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L47" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M47" s="25" t="inlineStr"/>
+      <c r="L47" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M47" s="26" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="24" t="inlineStr">
+      <c r="A48" s="27" t="inlineStr">
         <is>
           <t>4414096220</t>
         </is>
       </c>
-      <c r="B48" s="24" t="inlineStr">
+      <c r="B48" s="27" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3565,12 +3571,12 @@
           <t>Visualization Engineer Intern</t>
         </is>
       </c>
-      <c r="D48" s="24" t="inlineStr">
+      <c r="D48" s="27" t="inlineStr">
         <is>
           <t>Leidos</t>
         </is>
       </c>
-      <c r="E48" s="24" t="inlineStr">
+      <c r="E48" s="27" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3585,12 +3591,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H48" s="24" t="inlineStr">
+      <c r="H48" s="27" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="I48" s="24" t="inlineStr">
+      <c r="I48" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3605,20 +3611,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L48" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M48" s="24" t="inlineStr"/>
+      <c r="L48" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M48" s="27" t="inlineStr"/>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="25" t="inlineStr">
+      <c r="A49" s="26" t="inlineStr">
         <is>
           <t>4361076044</t>
         </is>
       </c>
-      <c r="B49" s="25" t="inlineStr">
+      <c r="B49" s="26" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -3628,12 +3634,12 @@
           <t>GenAI Engineering Intern  - SkillBridge (Remote)</t>
         </is>
       </c>
-      <c r="D49" s="25" t="inlineStr">
+      <c r="D49" s="26" t="inlineStr">
         <is>
           <t>CrowdStrike</t>
         </is>
       </c>
-      <c r="E49" s="25" t="inlineStr">
+      <c r="E49" s="26" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3648,12 +3654,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H49" s="25" t="inlineStr">
+      <c r="H49" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I49" s="25" t="inlineStr">
+      <c r="I49" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3668,20 +3674,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L49" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M49" s="25" t="inlineStr"/>
+      <c r="L49" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M49" s="26" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="24" t="inlineStr">
+      <c r="A50" s="27" t="inlineStr">
         <is>
           <t>4417553585</t>
         </is>
       </c>
-      <c r="B50" s="24" t="inlineStr">
+      <c r="B50" s="27" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -3691,12 +3697,12 @@
           <t>Entry-Level Software Engineer | Remote</t>
         </is>
       </c>
-      <c r="D50" s="24" t="inlineStr">
+      <c r="D50" s="27" t="inlineStr">
         <is>
           <t>Crossing Hurdles</t>
         </is>
       </c>
-      <c r="E50" s="24" t="inlineStr">
+      <c r="E50" s="27" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3711,12 +3717,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H50" s="24" t="inlineStr">
+      <c r="H50" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I50" s="24" t="inlineStr">
+      <c r="I50" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3731,20 +3737,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L50" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M50" s="24" t="inlineStr"/>
+      <c r="L50" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M50" s="27" t="inlineStr"/>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="25" t="inlineStr">
+      <c r="A51" s="26" t="inlineStr">
         <is>
           <t>4309699451</t>
         </is>
       </c>
-      <c r="B51" s="25" t="inlineStr">
+      <c r="B51" s="26" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -3754,12 +3760,12 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="D51" s="25" t="inlineStr">
+      <c r="D51" s="26" t="inlineStr">
         <is>
           <t>DataAnnotation</t>
         </is>
       </c>
-      <c r="E51" s="25" t="inlineStr">
+      <c r="E51" s="26" t="inlineStr">
         <is>
           <t>Washington, United States</t>
         </is>
@@ -3774,12 +3780,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H51" s="25" t="inlineStr">
+      <c r="H51" s="26" t="inlineStr">
         <is>
           <t>109</t>
         </is>
       </c>
-      <c r="I51" s="25" t="inlineStr">
+      <c r="I51" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3794,20 +3800,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L51" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M51" s="25" t="inlineStr"/>
+      <c r="L51" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M51" s="26" t="inlineStr"/>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="24" t="inlineStr">
+      <c r="A52" s="27" t="inlineStr">
         <is>
           <t>4406945262</t>
         </is>
       </c>
-      <c r="B52" s="24" t="inlineStr">
+      <c r="B52" s="27" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -3817,12 +3823,12 @@
           <t>DevSecOps Intern</t>
         </is>
       </c>
-      <c r="D52" s="24" t="inlineStr">
+      <c r="D52" s="27" t="inlineStr">
         <is>
           <t>Modern Technology Solutions, Inc. (MTSI)</t>
         </is>
       </c>
-      <c r="E52" s="24" t="inlineStr">
+      <c r="E52" s="27" t="inlineStr">
         <is>
           <t>Niceville, FL</t>
         </is>
@@ -3837,12 +3843,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H52" s="24" t="inlineStr">
+      <c r="H52" s="27" t="inlineStr">
         <is>
           <t>72</t>
         </is>
       </c>
-      <c r="I52" s="24" t="inlineStr">
+      <c r="I52" s="27" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -3857,20 +3863,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L52" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M52" s="24" t="inlineStr"/>
+      <c r="L52" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M52" s="27" t="inlineStr"/>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="25" t="inlineStr">
+      <c r="A53" s="26" t="inlineStr">
         <is>
           <t>4407937810</t>
         </is>
       </c>
-      <c r="B53" s="25" t="inlineStr">
+      <c r="B53" s="26" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -3880,12 +3886,12 @@
           <t>Temporary Intern - Agentic AI &amp; Neural-Symbolic Systems (Healthcare)</t>
         </is>
       </c>
-      <c r="D53" s="25" t="inlineStr">
+      <c r="D53" s="26" t="inlineStr">
         <is>
           <t>Cotiviti</t>
         </is>
       </c>
-      <c r="E53" s="25" t="inlineStr">
+      <c r="E53" s="26" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3900,12 +3906,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H53" s="25" t="inlineStr">
+      <c r="H53" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I53" s="25" t="inlineStr">
+      <c r="I53" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3920,20 +3926,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L53" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M53" s="25" t="inlineStr"/>
+      <c r="L53" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M53" s="26" t="inlineStr"/>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="24" t="inlineStr">
+      <c r="A54" s="27" t="inlineStr">
         <is>
           <t>4414089997</t>
         </is>
       </c>
-      <c r="B54" s="24" t="inlineStr">
+      <c r="B54" s="27" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -3943,12 +3949,12 @@
           <t>Visualization Engineer Intern</t>
         </is>
       </c>
-      <c r="D54" s="24" t="inlineStr">
+      <c r="D54" s="27" t="inlineStr">
         <is>
           <t>Leidos</t>
         </is>
       </c>
-      <c r="E54" s="24" t="inlineStr">
+      <c r="E54" s="27" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -3963,12 +3969,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H54" s="24" t="inlineStr">
+      <c r="H54" s="27" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="I54" s="24" t="inlineStr">
+      <c r="I54" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -3983,20 +3989,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L54" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M54" s="24" t="inlineStr"/>
+      <c r="L54" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M54" s="27" t="inlineStr"/>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="25" t="inlineStr">
+      <c r="A55" s="26" t="inlineStr">
         <is>
           <t>4387443129</t>
         </is>
       </c>
-      <c r="B55" s="25" t="inlineStr">
+      <c r="B55" s="26" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -4006,12 +4012,12 @@
           <t>2026 Interns</t>
         </is>
       </c>
-      <c r="D55" s="25" t="inlineStr">
+      <c r="D55" s="26" t="inlineStr">
         <is>
           <t>Givelify</t>
         </is>
       </c>
-      <c r="E55" s="25" t="inlineStr">
+      <c r="E55" s="26" t="inlineStr">
         <is>
           <t>Dallas, TX</t>
         </is>
@@ -4026,12 +4032,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H55" s="25" t="inlineStr">
+      <c r="H55" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I55" s="25" t="inlineStr">
+      <c r="I55" s="26" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -4046,20 +4052,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L55" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M55" s="25" t="inlineStr"/>
+      <c r="L55" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M55" s="26" t="inlineStr"/>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="24" t="inlineStr">
+      <c r="A56" s="27" t="inlineStr">
         <is>
           <t>4337980765</t>
         </is>
       </c>
-      <c r="B56" s="24" t="inlineStr">
+      <c r="B56" s="27" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -4069,12 +4075,12 @@
           <t>Submitting for a General Internship Application</t>
         </is>
       </c>
-      <c r="D56" s="24" t="inlineStr">
+      <c r="D56" s="27" t="inlineStr">
         <is>
           <t>Chainguard</t>
         </is>
       </c>
-      <c r="E56" s="24" t="inlineStr">
+      <c r="E56" s="27" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -4089,12 +4095,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H56" s="24" t="inlineStr">
+      <c r="H56" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I56" s="24" t="inlineStr">
+      <c r="I56" s="27" t="inlineStr">
         <is>
           <t>Volunteer</t>
         </is>
@@ -4109,20 +4115,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L56" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M56" s="24" t="inlineStr"/>
+      <c r="L56" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M56" s="27" t="inlineStr"/>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="25" t="inlineStr">
+      <c r="A57" s="26" t="inlineStr">
         <is>
           <t>4417030460</t>
         </is>
       </c>
-      <c r="B57" s="25" t="inlineStr">
+      <c r="B57" s="26" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -4132,12 +4138,12 @@
           <t>AI Researcher Intern</t>
         </is>
       </c>
-      <c r="D57" s="25" t="inlineStr">
+      <c r="D57" s="26" t="inlineStr">
         <is>
           <t>BioSpace</t>
         </is>
       </c>
-      <c r="E57" s="25" t="inlineStr">
+      <c r="E57" s="26" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -4152,12 +4158,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H57" s="25" t="inlineStr">
+      <c r="H57" s="26" t="inlineStr">
         <is>
           <t>151</t>
         </is>
       </c>
-      <c r="I57" s="25" t="inlineStr">
+      <c r="I57" s="26" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -4172,20 +4178,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L57" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M57" s="25" t="inlineStr"/>
+      <c r="L57" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M57" s="26" t="inlineStr"/>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="24" t="inlineStr">
+      <c r="A58" s="27" t="inlineStr">
         <is>
           <t>4406930916</t>
         </is>
       </c>
-      <c r="B58" s="24" t="inlineStr">
+      <c r="B58" s="27" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -4195,12 +4201,12 @@
           <t>DevSecOps Intern</t>
         </is>
       </c>
-      <c r="D58" s="24" t="inlineStr">
+      <c r="D58" s="27" t="inlineStr">
         <is>
           <t>Modern Technology Solutions, Inc. (MTSI)</t>
         </is>
       </c>
-      <c r="E58" s="24" t="inlineStr">
+      <c r="E58" s="27" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -4215,12 +4221,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H58" s="24" t="inlineStr">
+      <c r="H58" s="27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I58" s="24" t="inlineStr">
+      <c r="I58" s="27" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -4235,20 +4241,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L58" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M58" s="24" t="inlineStr"/>
+      <c r="L58" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M58" s="27" t="inlineStr"/>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="25" t="inlineStr">
+      <c r="A59" s="26" t="inlineStr">
         <is>
           <t>4385798937</t>
         </is>
       </c>
-      <c r="B59" s="25" t="inlineStr">
+      <c r="B59" s="26" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -4258,12 +4264,12 @@
           <t>Research Intern on Generative and Protective AI for Content Creation</t>
         </is>
       </c>
-      <c r="D59" s="25" t="inlineStr">
+      <c r="D59" s="26" t="inlineStr">
         <is>
           <t>SonyAI</t>
         </is>
       </c>
-      <c r="E59" s="25" t="inlineStr">
+      <c r="E59" s="26" t="inlineStr">
         <is>
           <t>New York, United States</t>
         </is>
@@ -4278,12 +4284,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="H59" s="25" t="inlineStr">
+      <c r="H59" s="26" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="I59" s="25" t="inlineStr">
+      <c r="I59" s="26" t="inlineStr">
         <is>
           <t>Part-time</t>
         </is>
@@ -4298,20 +4304,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L59" s="25" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M59" s="25" t="inlineStr"/>
+      <c r="L59" s="26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M59" s="26" t="inlineStr"/>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="24" t="inlineStr">
+      <c r="A60" s="27" t="inlineStr">
         <is>
           <t>4414396950</t>
         </is>
       </c>
-      <c r="B60" s="24" t="inlineStr">
+      <c r="B60" s="27" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
@@ -4321,12 +4327,12 @@
           <t>Power Platform Intern</t>
         </is>
       </c>
-      <c r="D60" s="24" t="inlineStr">
+      <c r="D60" s="27" t="inlineStr">
         <is>
           <t>Leidos</t>
         </is>
       </c>
-      <c r="E60" s="24" t="inlineStr">
+      <c r="E60" s="27" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
@@ -4341,12 +4347,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H60" s="24" t="inlineStr">
+      <c r="H60" s="27" t="inlineStr">
         <is>
           <t>135</t>
         </is>
       </c>
-      <c r="I60" s="24" t="inlineStr">
+      <c r="I60" s="27" t="inlineStr">
         <is>
           <t>Full-time</t>
         </is>
@@ -4361,12 +4367,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="L60" s="24" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="M60" s="24" t="inlineStr"/>
+      <c r="L60" s="27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M60" s="27" t="inlineStr"/>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="26" t="inlineStr">
@@ -5691,8 +5697,386 @@
       </c>
       <c r="M81" s="26" t="inlineStr"/>
     </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="28" t="inlineStr">
+        <is>
+          <t>4418507307</t>
+        </is>
+      </c>
+      <c r="B82" s="28" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Entry Level Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D82" s="28" t="inlineStr">
+        <is>
+          <t>CORMAC</t>
+        </is>
+      </c>
+      <c r="E82" s="28" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="G82" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H82" s="28" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="I82" s="28" t="inlineStr">
+        <is>
+          <t>Volunteer</t>
+        </is>
+      </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>Skills: javascript, git, c, express, agile, Title match: Entry Level Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="K82" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L82" s="28" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M82" s="28" t="inlineStr"/>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="29" t="inlineStr">
+        <is>
+          <t>4413360938</t>
+        </is>
+      </c>
+      <c r="B83" s="29" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Software Engineer Internship (Remote)</t>
+        </is>
+      </c>
+      <c r="D83" s="29" t="inlineStr">
+        <is>
+          <t>Orange Trail</t>
+        </is>
+      </c>
+      <c r="E83" s="29" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>48%</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H83" s="29" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I83" s="29" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J83" s="8" t="inlineStr">
+        <is>
+          <t>Skills: javascript, html, css, backend, c, llm, Title match: Software Engineer Internship (Remote)</t>
+        </is>
+      </c>
+      <c r="K83" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L83" s="29" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M83" s="29" t="inlineStr"/>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="28" t="inlineStr">
+        <is>
+          <t>4348111641</t>
+        </is>
+      </c>
+      <c r="B84" s="28" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D84" s="28" t="inlineStr">
+        <is>
+          <t>Simular</t>
+        </is>
+      </c>
+      <c r="E84" s="28" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>48%</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H84" s="28" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I84" s="28" t="inlineStr">
+        <is>
+          <t>Volunteer</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, javascript, rest, backend, frontend, c, Title match: Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="K84" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L84" s="28" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M84" s="28" t="inlineStr"/>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="29" t="inlineStr">
+        <is>
+          <t>4411853543</t>
+        </is>
+      </c>
+      <c r="B85" s="29" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Intern, Software Engineer</t>
+        </is>
+      </c>
+      <c r="D85" s="29" t="inlineStr">
+        <is>
+          <t>Accelerate Learning</t>
+        </is>
+      </c>
+      <c r="E85" s="29" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H85" s="29" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I85" s="29" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="J85" s="8" t="inlineStr">
+        <is>
+          <t>Skills: react, node, aws, rest, api, git, Title match: Intern, Software Engineer</t>
+        </is>
+      </c>
+      <c r="K85" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L85" s="29" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M85" s="29" t="inlineStr"/>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="28" t="inlineStr">
+        <is>
+          <t>4408586245</t>
+        </is>
+      </c>
+      <c r="B86" s="28" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Junior Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D86" s="28" t="inlineStr">
+        <is>
+          <t>Cantaloupe Inc</t>
+        </is>
+      </c>
+      <c r="E86" s="28" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H86" s="28" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I86" s="28" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>Skills: javascript, aws, rest, html, css, git, Title match: Junior Software Engineer Intern</t>
+        </is>
+      </c>
+      <c r="K86" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L86" s="28" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M86" s="28" t="inlineStr"/>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="29" t="inlineStr">
+        <is>
+          <t>4364536992</t>
+        </is>
+      </c>
+      <c r="B87" s="29" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Summer Internship - Measurement, Research and Development - Academic Measurement</t>
+        </is>
+      </c>
+      <c r="D87" s="29" t="inlineStr">
+        <is>
+          <t>ChatGPT Jobs</t>
+        </is>
+      </c>
+      <c r="E87" s="29" t="inlineStr">
+        <is>
+          <t>Iowa City, IA</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="G87" s="19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H87" s="29" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="I87" s="29" t="inlineStr">
+        <is>
+          <t>Volunteer</t>
+        </is>
+      </c>
+      <c r="J87" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, rest, git, pytorch, machine learning, c, Title match: Summer Internship - Measurement, Research and Development - Academic Measurement</t>
+        </is>
+      </c>
+      <c r="K87" s="11" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L87" s="29" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M87" s="29" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M81"/>
+  <autoFilter ref="A1:M87"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -5774,6 +6158,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-07-07
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$L$9</definedName>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-07-08
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$L$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -153,6 +153,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -519,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1062,8 +1068,124 @@
       </c>
       <c r="L9" s="7" t="inlineStr"/>
     </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>gh:togetherai:5157380007</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Frontier Agents Intern (Fall 2026)</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Together AI</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>51%</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Gh</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, pytorch, nlp, machine learning, deep learning, algorithms, Internship title, Posted &lt;7d ago, Flags: PhD-oriented role</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>gh:togetherai:5157559007</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Systems Research Engineer Intern - GPU Programming (Fall 2026)</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Together AI</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>51%</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Gh</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Skills: algorithms, artificial intelligence, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="L11" s="15" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L9"/>
+  <autoFilter ref="A1:L11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -1073,6 +1195,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-07-09
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$L$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -158,6 +158,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -525,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -605,12 +608,12 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>ashby:baseten:58d7d8e6-86ee-43a1-baec-3dddcb661d51</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -620,12 +623,12 @@
           <t>Base Labs Fellowship</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="14" t="inlineStr">
         <is>
           <t>Baseten</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>San Francisco (Remote)</t>
         </is>
@@ -640,7 +643,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="14" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -655,20 +658,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="14" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="L2" s="14" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>ashby:notion:297b4ece-765f-4eea-b1b8-46057cb6501f</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -678,12 +681,12 @@
           <t>Software Engineer, Early Career</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>San Francisco, California</t>
         </is>
@@ -698,7 +701,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="15" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -713,20 +716,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="K3" s="15" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="L3" s="15" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>ashby:notion:5b15697c-fa91-4511-9482-c98a6ff29f90</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -736,12 +739,12 @@
           <t>Software Engineer Intern (Fall 2026)</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -756,7 +759,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -771,20 +774,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="14" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="L4" s="14" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>ashby:notion:7e6dc7fe-7ddd-42c1-8928-13f7bddb9ec9</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -794,12 +797,12 @@
           <t>Software Engineer, New Grad (AI)</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -814,7 +817,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -829,20 +832,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="K5" s="15" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="15" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>ashby:notion:85947779-6b87-466a-98bc-30a640448c28</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -852,12 +855,12 @@
           <t>Software Engineer, Early Career (AI)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -872,7 +875,7 @@
           <t>Strong Fit</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -887,20 +890,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="14" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="L6" s="14" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>ashby:notion:a6311f97-4850-4674-a5f3-d9fe5f6f2555</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -910,12 +913,12 @@
           <t>Software Engineer, New Grad</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -930,7 +933,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -945,20 +948,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="K7" s="15" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="15" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>ashby:ramp:67fadb77-43d8-4449-954b-d4cf2c6d3b8b</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -968,12 +971,12 @@
           <t xml:space="preserve">Software Engineer Internship, Android </t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Ramp</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>New York, NY (HQ) (Remote)</t>
         </is>
@@ -988,7 +991,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="14" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -1003,20 +1006,20 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K8" s="14" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="L8" s="14" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>gh:scaleai:4703343005</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -1026,12 +1029,12 @@
           <t>AI Builder Intern</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Scale AI</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>San Francisco, CA; New York, NY</t>
         </is>
@@ -1046,7 +1049,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
@@ -1061,12 +1064,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K9" s="15" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="15" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
@@ -1184,8 +1187,66 @@
       </c>
       <c r="L11" s="15" t="inlineStr"/>
     </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>gh:scaleai:4660340005</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Machine Learning Fellow - Human Frontier Collective (US)</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Scale AI</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>55%</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Good Fit</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>Gh</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, docker, aws, tensorflow, pytorch, langchain, Fellowship title, Posted &lt;7d ago, Flags: PhD-oriented role</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="L12" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L12"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -1197,6 +1258,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-07-10
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -608,12 +608,12 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>ashby:baseten:58d7d8e6-86ee-43a1-baec-3dddcb661d51</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -623,12 +623,12 @@
           <t>Base Labs Fellowship</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="16" t="inlineStr">
         <is>
           <t>Baseten</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>San Francisco (Remote)</t>
         </is>
@@ -643,7 +643,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H2" s="14" t="inlineStr">
+      <c r="H2" s="16" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -658,12 +658,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K2" s="14" t="inlineStr">
+      <c r="K2" s="16" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L2" s="14" t="inlineStr"/>
+      <c r="L2" s="16" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="15" t="inlineStr">
@@ -724,12 +724,12 @@
       <c r="L3" s="15" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>ashby:notion:5b15697c-fa91-4511-9482-c98a6ff29f90</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -739,12 +739,12 @@
           <t>Software Engineer Intern (Fall 2026)</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -759,7 +759,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -774,12 +774,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K4" s="14" t="inlineStr">
+      <c r="K4" s="16" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L4" s="14" t="inlineStr"/>
+      <c r="L4" s="16" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="15" t="inlineStr">
@@ -840,12 +840,12 @@
       <c r="L5" s="15" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>ashby:notion:85947779-6b87-466a-98bc-30a640448c28</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -855,12 +855,12 @@
           <t>Software Engineer, Early Career (AI)</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -875,7 +875,7 @@
           <t>Strong Fit</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="16" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -890,12 +890,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K6" s="14" t="inlineStr">
+      <c r="K6" s="16" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L6" s="14" t="inlineStr"/>
+      <c r="L6" s="16" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
@@ -956,12 +956,12 @@
       <c r="L7" s="15" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>ashby:ramp:67fadb77-43d8-4449-954b-d4cf2c6d3b8b</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
@@ -971,12 +971,12 @@
           <t xml:space="preserve">Software Engineer Internship, Android </t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Ramp</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>New York, NY (HQ) (Remote)</t>
         </is>
@@ -991,7 +991,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -1006,12 +1006,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K8" s="14" t="inlineStr">
+      <c r="K8" s="16" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L8" s="14" t="inlineStr"/>
+      <c r="L8" s="16" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="15" t="inlineStr">
@@ -1072,12 +1072,12 @@
       <c r="L9" s="15" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>gh:togetherai:5157380007</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
@@ -1087,12 +1087,12 @@
           <t>Frontier Agents Intern (Fall 2026)</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>Together AI</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>San Francisco</t>
         </is>
@@ -1107,7 +1107,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H10" s="14" t="inlineStr">
+      <c r="H10" s="16" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
@@ -1122,12 +1122,12 @@
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K10" s="14" t="inlineStr">
+      <c r="K10" s="16" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L10" s="14" t="inlineStr"/>
+      <c r="L10" s="16" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="15" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-07-11
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startups" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Startups" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$L$18</definedName>

</xml_diff>

<commit_message>
Add outreach drafts, company website column, and region-filtered Startups tab
- LinkedIn Note Draft / Email Draft columns: personalized outreach text
  generated per posting (picks the most relevant project highlight based
  on matched skills). No LinkedIn scraping, no auto-sending — these are
  just drafts sitting in a cell for Giri to copy and send himself.
- WSU Alumni Search / Recruiter Search columns: pre-built LinkedIn people-
  search links per company, opened logged-in as Giri. Same reasoning —
  automating the actual search/send would violate LinkedIn's ToS.
- Company Website column: direct link to each company's homepage.
- Startups tab is now narrowed further to companies located in Seattle,
  the SF Bay Area, Texas, Arizona, or remote (on top of the existing
  startup:true tag) via STARTUP_TAB_LOCATION_RE.
- Rebuilt jobs.xlsx fresh again since the column layout changed (17 cols,
  same pattern as the last two structural changes).
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Startups" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startups" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$L$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Startups'!$A$1:$L$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$Q$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Startups'!$A$1:$Q$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -126,13 +126,13 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -141,13 +141,13 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -521,21 +521,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -561,46 +566,71 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Company Website</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Match %</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Fit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Why It Matched</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>WSU Alumni Search</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Recruiter Search</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>LinkedIn Note Draft</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Email Draft</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ashby:baseten:58d7d8e6-86ee-43a1-baec-3dddcb661d51</t>
@@ -621,44 +651,76 @@
           <t>Baseten</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>San Francisco (Remote)</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>54%</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Skills: machine learning, statistics, Fellowship title, Location: San Francisco (Remote), Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Baseten is hiring for Base Labs Fellowship. I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Base Labs Fellowship role at Baseten
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Base Labs Fellowship opening at Baseten and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
-    <row r="3" ht="18" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>ashby:notion:a6311f97-4850-4674-a5f3-d9fe5f6f2555</t>
@@ -679,44 +741,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>64%</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Skills: python, javascript, typescript, react, node, node.js, New-grad title, Location: San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer, New Grad. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer, New Grad role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer, New Grad opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="Q3" s="7" t="inlineStr"/>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ashby:notion:5b15697c-fa91-4511-9482-c98a6ff29f90</t>
@@ -737,44 +831,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>68%</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Skills: python, typescript, react, node, node.js, embeddings, Internship title, Location: San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer Intern (Fall 2026). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer Intern (Fall 2026) role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer Intern (Fall 2026) opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
-    <row r="5" ht="18" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>ashby:notion:7e6dc7fe-7ddd-42c1-8928-13f7bddb9ec9</t>
@@ -795,44 +921,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>52%</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>Skills: python, typescript, react, node, node.js, embeddings, New-grad title, Location: San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="J5" s="11" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer, New Grad (AI). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer, New Grad (AI) role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer, New Grad (AI) opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="Q5" s="7" t="inlineStr"/>
     </row>
-    <row r="6" ht="18" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>ashby:notion:85947779-6b87-466a-98bc-30a640448c28</t>
@@ -853,44 +1011,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>73%</t>
         </is>
       </c>
-      <c r="G6" s="13" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>Strong Fit</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Skills: typescript, react, node, node.js, embeddings, data structures, New-grad title, Location: San Francisco, California (Remote), Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer, Early Career (AI). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer, Early Career (AI) role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer, Early Career (AI) opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
     </row>
-    <row r="7" ht="18" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>ashby:notion:297b4ece-765f-4eea-b1b8-46057cb6501f</t>
@@ -911,44 +1101,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>San Francisco, California</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>53%</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>Skills: typescript, react, node, node.js, backend, data structures, New-grad title, Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J7" s="11" t="inlineStr">
+      <c r="K7" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer, Early Career. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer, Early Career role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer, Early Career opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="Q7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="18" customHeight="1">
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>ashby:ramp:67fadb77-43d8-4449-954b-d4cf2c6d3b8b</t>
@@ -969,44 +1191,76 @@
           <t>Ramp</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>New York, NY (HQ) (Remote)</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>65%</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Skills: python, typescript, react, flask, sql, backend, Internship title, Location: New York, NY (HQ) (Remote)</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Ramp is hiring for Software Engineer Internship, Android . I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer Internship, Android  role at Ramp
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer Internship, Android  opening at Ramp and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
     </row>
-    <row r="9" ht="18" customHeight="1">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>gh:togetherai:5157380007</t>
@@ -1027,44 +1281,76 @@
           <t>Together AI</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>51%</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>Skills: python, pytorch, nlp, machine learning, deep learning, algorithms, Internship title, Posted &lt;7d ago, Flags: PhD-oriented role</t>
         </is>
       </c>
-      <c r="J9" s="11" t="inlineStr">
+      <c r="K9" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Together AI is hiring for Frontier Agents Intern (Fall 2026). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Frontier Agents Intern (Fall 2026) role at Together AI
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Frontier Agents Intern (Fall 2026) opening at Together AI and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="Q9" s="7" t="inlineStr"/>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>gh:togetherai:5157559007</t>
@@ -1085,44 +1371,76 @@
           <t>Together AI</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>51%</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Skills: algorithms, artificial intelligence, Internship title, Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Together AI is hiring for Systems Research Engineer Intern - GPU Programming (Fall 2026). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Systems Research Engineer Intern - GPU Programming (Fall 2026) role at Together AI
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Systems Research Engineer Intern - GPU Programming (Fall 2026) opening at Together AI and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
     </row>
-    <row r="11" ht="18" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>gh:scaleai:4703343005</t>
@@ -1143,44 +1461,76 @@
           <t>Scale AI</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>San Francisco, CA; New York, NY</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>72%</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>Strong Fit</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>Skills: python, javascript, react, api, github, llm, Internship title, Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J11" s="11" t="inlineStr">
+      <c r="K11" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Scale AI is hiring for AI Builder Intern. I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the AI Builder Intern role at Scale AI
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the AI Builder Intern opening at Scale AI and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="Q11" s="7" t="inlineStr"/>
     </row>
-    <row r="12" ht="18" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>gh:scaleai:4660340005</t>
@@ -1201,44 +1551,76 @@
           <t>Scale AI</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="G12" s="10" t="inlineStr">
         <is>
           <t>55%</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Skills: python, docker, aws, tensorflow, pytorch, langchain, Fellowship title, Posted &lt;7d ago, Flags: PhD-oriented role</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Scale AI is hiring for Machine Learning Fellow - Human Frontier Collective (US). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Machine Learning Fellow - Human Frontier Collective (US) role at Scale AI
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Machine Learning Fellow - Human Frontier Collective (US) opening at Scale AI and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>lever:palantir:f17e98d0-046a-4e6e-9d65-ed0b12dd0ff7</t>
@@ -1259,44 +1641,76 @@
           <t>Palantir</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Washington, D.C.</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="G13" s="10" t="inlineStr">
         <is>
           <t>62%</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>Lever</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>Skills: typescript, react, github, backend, frontend, Internship title, Location: Washington, D.C.</t>
         </is>
       </c>
-      <c r="J13" s="11" t="inlineStr">
+      <c r="K13" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr">
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Palantir is hiring for Software Engineer, Internship - Defense Tech. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer, Internship - Defense Tech role at Palantir
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer, Internship - Defense Tech opening at Palantir and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr"/>
+      <c r="Q13" s="7" t="inlineStr"/>
     </row>
-    <row r="14" ht="18" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>gh:cloudflare:8031027</t>
@@ -1317,44 +1731,76 @@
           <t>Cloudflare</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>In-Office</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>54%</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>Skills: python, sql, data analysis, excel, kpi, Internship title</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Cloudflare is hiring for Network Strategy Intern (Fall 2026). I've built a couple of data-heavy projects, including an automated stock signal analyzer — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Network Strategy Intern (Fall 2026) role at Cloudflare
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Network Strategy Intern (Fall 2026) opening at Cloudflare and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've built a couple of data-focused projects — an automated stock analysis tool applying technical indicators to live market data, and an interactive trail-mapping app processing 200+ real-world datasets with Pandas.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
     </row>
-    <row r="15" ht="18" customHeight="1">
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>gh:cloudflare:8013562</t>
@@ -1375,44 +1821,76 @@
           <t>Cloudflare</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>In-Office</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>54%</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>Skills: python, sql, data analysis, excel, kpi, Internship title</t>
         </is>
       </c>
-      <c r="J15" s="11" t="inlineStr">
+      <c r="K15" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Cloudflare is hiring for Network Strategy Intern (Fall 2026). I've built a couple of data-heavy projects, including an automated stock signal analyzer — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Network Strategy Intern (Fall 2026) role at Cloudflare
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Network Strategy Intern (Fall 2026) opening at Cloudflare and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've built a couple of data-focused projects — an automated stock analysis tool applying technical indicators to live market data, and an interactive trail-mapping app processing 200+ real-world datasets with Pandas.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="Q15" s="7" t="inlineStr"/>
     </row>
-    <row r="16" ht="18" customHeight="1">
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>gh:cloudflare:8041135</t>
@@ -1433,44 +1911,76 @@
           <t>Cloudflare</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>In-Office</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="G16" s="10" t="inlineStr">
         <is>
           <t>57%</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>Skills: python, javascript, rest, git, Internship title, Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Cloudflare is hiring for Technical Support Engineer Intern (Fall 2026). I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Technical Support Engineer Intern (Fall 2026) role at Cloudflare
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Technical Support Engineer Intern (Fall 2026) opening at Cloudflare and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>gh:imc:4907430101</t>
@@ -1491,44 +2001,76 @@
           <t>IMC Trading</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Chicago, United States</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>51%</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I17" s="8" t="inlineStr">
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>Skills: python, tensorflow, pytorch, machine learning, deep learning, algorithms, Internship title, Posted &lt;7d ago, Flags: PhD-oriented role</t>
         </is>
       </c>
-      <c r="J17" s="11" t="inlineStr">
+      <c r="K17" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw IMC Trading is hiring for Machine Learning Research Intern - Summer 2027 - Chicago. I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Machine Learning Research Intern - Summer 2027 - Chicago role at IMC Trading
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Machine Learning Research Intern - Summer 2027 - Chicago opening at IMC Trading and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr"/>
+      <c r="Q17" s="7" t="inlineStr"/>
     </row>
-    <row r="18" ht="18" customHeight="1">
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>gh:imc:4907399101</t>
@@ -1549,63 +2091,146 @@
           <t>IMC Trading</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Chicago, United States</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>54%</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>Skills: python, c++, statistics, Internship title, Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw IMC Trading is hiring for Quantitative Research Intern (BS/MS) - Summer 2027. I've built a couple of data-heavy projects, including an automated stock signal analyzer — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Quantitative Research Intern (BS/MS) - Summer 2027 role at IMC Trading
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Quantitative Research Intern (BS/MS) - Summer 2027 opening at IMC Trading and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've built a couple of data-focused projects — an automated stock analysis tool applying technical indicators to live market data, and an interactive trail-mapping app processing 200+ real-world datasets with Pandas.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L18"/>
+  <autoFilter ref="A1:Q18"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1617,21 +2242,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1657,46 +2287,71 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Company Website</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Match %</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Fit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Why It Matched</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>WSU Alumni Search</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Recruiter Search</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>LinkedIn Note Draft</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Email Draft</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ashby:baseten:58d7d8e6-86ee-43a1-baec-3dddcb661d51</t>
@@ -1717,44 +2372,76 @@
           <t>Baseten</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>San Francisco (Remote)</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>54%</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Skills: machine learning, statistics, Fellowship title, Location: San Francisco (Remote), Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Baseten is hiring for Base Labs Fellowship. I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Base Labs Fellowship role at Baseten
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Base Labs Fellowship opening at Baseten and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
-    <row r="3" ht="18" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>ashby:notion:a6311f97-4850-4674-a5f3-d9fe5f6f2555</t>
@@ -1775,44 +2462,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>64%</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Skills: python, javascript, typescript, react, node, node.js, New-grad title, Location: San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer, New Grad. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer, New Grad role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer, New Grad opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="Q3" s="7" t="inlineStr"/>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ashby:notion:5b15697c-fa91-4511-9482-c98a6ff29f90</t>
@@ -1833,44 +2552,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>68%</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Skills: python, typescript, react, node, node.js, embeddings, Internship title, Location: San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer Intern (Fall 2026). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer Intern (Fall 2026) role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer Intern (Fall 2026) opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
-    <row r="5" ht="18" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>ashby:notion:7e6dc7fe-7ddd-42c1-8928-13f7bddb9ec9</t>
@@ -1891,44 +2642,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>52%</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>Skills: python, typescript, react, node, node.js, embeddings, New-grad title, Location: San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="J5" s="11" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer, New Grad (AI). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer, New Grad (AI) role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer, New Grad (AI) opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="Q5" s="7" t="inlineStr"/>
     </row>
-    <row r="6" ht="18" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>ashby:notion:85947779-6b87-466a-98bc-30a640448c28</t>
@@ -1949,44 +2732,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>73%</t>
         </is>
       </c>
-      <c r="G6" s="13" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>Strong Fit</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Skills: typescript, react, node, node.js, embeddings, data structures, New-grad title, Location: San Francisco, California (Remote), Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer, Early Career (AI). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer, Early Career (AI) role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer, Early Career (AI) opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
     </row>
-    <row r="7" ht="18" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>ashby:notion:297b4ece-765f-4eea-b1b8-46057cb6501f</t>
@@ -2007,44 +2822,76 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>San Francisco, California</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>53%</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>Skills: typescript, react, node, node.js, backend, data structures, New-grad title, Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J7" s="11" t="inlineStr">
+      <c r="K7" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Notion is hiring for Software Engineer, Early Career. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer, Early Career role at Notion
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer, Early Career opening at Notion and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="Q7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="18" customHeight="1">
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>ashby:ramp:67fadb77-43d8-4449-954b-d4cf2c6d3b8b</t>
@@ -2065,44 +2912,76 @@
           <t>Ramp</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>New York, NY (HQ) (Remote)</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>65%</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Skills: python, typescript, react, flask, sql, backend, Internship title, Location: New York, NY (HQ) (Remote)</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Ramp is hiring for Software Engineer Internship, Android . I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer Internship, Android  role at Ramp
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer Internship, Android  opening at Ramp and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
     </row>
-    <row r="9" ht="18" customHeight="1">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>gh:togetherai:5157380007</t>
@@ -2123,44 +3002,76 @@
           <t>Together AI</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>51%</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>Skills: python, pytorch, nlp, machine learning, deep learning, algorithms, Internship title, Posted &lt;7d ago, Flags: PhD-oriented role</t>
         </is>
       </c>
-      <c r="J9" s="11" t="inlineStr">
+      <c r="K9" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Together AI is hiring for Frontier Agents Intern (Fall 2026). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Frontier Agents Intern (Fall 2026) role at Together AI
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Frontier Agents Intern (Fall 2026) opening at Together AI and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="Q9" s="7" t="inlineStr"/>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>gh:togetherai:5157559007</t>
@@ -2181,44 +3092,76 @@
           <t>Together AI</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>51%</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Skills: algorithms, artificial intelligence, Internship title, Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Together AI is hiring for Systems Research Engineer Intern - GPU Programming (Fall 2026). I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Systems Research Engineer Intern - GPU Programming (Fall 2026) role at Together AI
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Systems Research Engineer Intern - GPU Programming (Fall 2026) opening at Together AI and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
     </row>
-    <row r="11" ht="18" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>gh:scaleai:4703343005</t>
@@ -2239,115 +3182,118 @@
           <t>Scale AI</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>San Francisco, CA; New York, NY</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>72%</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>Strong Fit</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>Skills: python, javascript, react, api, github, llm, Internship title, Posted &lt;7d ago</t>
         </is>
       </c>
-      <c r="J11" s="11" t="inlineStr">
+      <c r="K11" s="9" t="inlineStr">
         <is>
           <t>Apply →</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>WSU Alumni →</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Recruiters →</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Scale AI is hiring for AI Builder Intern. I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the AI Builder Intern role at Scale AI
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the AI Builder Intern opening at Scale AI and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr">
         <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>gh:scaleai:4660340005</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Machine Learning Fellow - Human Frontier Collective (US)</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Scale AI</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>55%</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>Good Fit</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Gh</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>Skills: python, docker, aws, tensorflow, pytorch, langchain, Fellowship title, Posted &lt;7d ago, Flags: PhD-oriented role</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>Apply →</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="Q11" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L12"/>
+  <autoFilter ref="A1:Q11"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 9 Texas/Arizona companies for future Startups-tab coverage
Investigated why Seattle/TX/AZ weren't showing on the Startups tab:
- Seattle: all 12 Seattle-area companies currently have zero open
  internships — normal day-to-day fluctuation, not a bug.
- TX/AZ: the company list had zero actual TX/AZ presence before this.
  Added Carvana (Tempe, AZ) and Axon (Scottsdale, AZ) — both public, so
  main tab only — plus CS Disco and Bazaarvoice (Austin, TX, also
  public/mature). Added Homeward, ShiftKey, AlertMedia, Convey, and
  Shipwell (all Austin/Dallas, TX, genuinely private/startup-stage) which
  will land on the Startups tab once they have internships open.

None of the 9 currently have open internships (confirmed: 147
internship-tagged postings found, same as before the addition), so
today's sheet is unchanged — this closes structural coverage for later.
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Startups" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startups" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$Q$18</definedName>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-07-12
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startups" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Internship Matches" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Startups" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internship Matches'!$A$1:$Q$113</definedName>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-07-13
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internships" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startups" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Internships" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Jobs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Startups" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internships'!$A$1:$P$60</definedName>

</xml_diff>

<commit_message>
🤖 Daily job update — 2026-07-14
</commit_message>
<xml_diff>
--- a/jobs.xlsx
+++ b/jobs.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Startups" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internships'!$A$1:$P$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internships'!$A$1:$P$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Jobs'!$A$1:$P$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Startups'!$A$1:$P$11</definedName>
   </definedNames>
@@ -117,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -157,6 +157,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -526,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P65"/>
+  <dimension ref="A1:P77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -715,12 +721,12 @@
       <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>ashby:notion:5b15697c-fa91-4511-9482-c98a6ff29f90</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -730,7 +736,7 @@
           <t>Software Engineer Intern (Fall 2026)</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
@@ -740,7 +746,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="14" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -755,7 +761,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -792,12 +798,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P3" s="7" t="inlineStr"/>
+      <c r="O3" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P3" s="14" t="inlineStr"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -885,12 +891,12 @@
       <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>gh:scaleai:4703343005</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -900,7 +906,7 @@
           <t>AI Builder Intern</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Scale AI</t>
         </is>
@@ -910,7 +916,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>San Francisco, CA; New York, NY</t>
         </is>
@@ -925,7 +931,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
@@ -962,12 +968,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O5" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P5" s="7" t="inlineStr"/>
+      <c r="O5" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P5" s="14" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1055,12 +1061,12 @@
       <c r="P6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>lever:palantir:f17e98d0-046a-4e6e-9d65-ed0b12dd0ff7</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -1070,7 +1076,7 @@
           <t>Software Engineer, Internship - Defense Tech</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Palantir</t>
         </is>
@@ -1080,7 +1086,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>Washington, D.C.</t>
         </is>
@@ -1095,7 +1101,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="14" t="inlineStr">
         <is>
           <t>Lever</t>
         </is>
@@ -1132,12 +1138,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P7" s="7" t="inlineStr"/>
+      <c r="O7" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P7" s="14" t="inlineStr"/>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1225,12 +1231,12 @@
       <c r="P8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>gh:cloudflare:8013562</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -1240,7 +1246,7 @@
           <t>Network Strategy Intern (Fall 2026)</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Cloudflare</t>
         </is>
@@ -1250,7 +1256,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>In-Office</t>
         </is>
@@ -1265,7 +1271,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
@@ -1302,12 +1308,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P9" s="7" t="inlineStr"/>
+      <c r="O9" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P9" s="14" t="inlineStr"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1395,12 +1401,12 @@
       <c r="P10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>simplify:e5045382-ee6d-4bcb-a35a-9d5d2d395276</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -1410,13 +1416,13 @@
           <t>AI Automation Intern</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>Advantmed</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr"/>
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>Remote in USA</t>
         </is>
@@ -1431,7 +1437,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -1468,12 +1474,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P11" s="7" t="inlineStr"/>
+      <c r="O11" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P11" s="14" t="inlineStr"/>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1557,12 +1563,12 @@
       <c r="P12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>simplify:7cbf5e66-95b6-4b66-b41f-fa9cdeadcadc</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -1572,7 +1578,7 @@
           <t>Software Engineer Intern - Commerce Ads - 2026 Summer</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
@@ -1582,7 +1588,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1597,7 +1603,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -1634,12 +1640,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P13" s="7" t="inlineStr"/>
+      <c r="O13" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P13" s="14" t="inlineStr"/>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1727,12 +1733,12 @@
       <c r="P14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>simplify:f9c3682d-25e0-42b3-aeb8-ae98854876fe</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -1742,7 +1748,7 @@
           <t>Software Engineer Intern - Payment Network - Global Payment</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>ByteDance</t>
         </is>
@@ -1752,7 +1758,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -1767,7 +1773,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -1804,12 +1810,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O15" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P15" s="7" t="inlineStr"/>
+      <c r="O15" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P15" s="14" t="inlineStr"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1897,12 +1903,12 @@
       <c r="P16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>simplify:7107711b-0874-460d-932c-0c0d7b729f42</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -1912,7 +1918,7 @@
           <t>Year at Palantir Intern - Forward Deployed Software Engineer</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Palantir</t>
         </is>
@@ -1922,7 +1928,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -1937,7 +1943,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -1974,12 +1980,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O17" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P17" s="7" t="inlineStr"/>
+      <c r="O17" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P17" s="14" t="inlineStr"/>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -2067,12 +2073,12 @@
       <c r="P18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>simplify:6c56bd42-aaca-45b8-b770-128f543898e0</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -2082,7 +2088,7 @@
           <t>Applied Scientist AI/ML Intern</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>Wealth.com</t>
         </is>
@@ -2092,7 +2098,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F19" s="14" t="inlineStr">
         <is>
           <t>Remote in USA</t>
         </is>
@@ -2107,7 +2113,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="I19" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -2144,12 +2150,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O19" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P19" s="7" t="inlineStr"/>
+      <c r="O19" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P19" s="14" t="inlineStr"/>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -2237,12 +2243,12 @@
       <c r="P20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>simplify:8d981cf1-c610-41cc-84d1-800ea078fd37</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -2252,7 +2258,7 @@
           <t>Software Development Engineer Intern - Network Automation</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>ByteDance</t>
         </is>
@@ -2262,7 +2268,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="14" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -2277,7 +2283,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I21" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -2314,12 +2320,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O21" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P21" s="7" t="inlineStr"/>
+      <c r="O21" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P21" s="14" t="inlineStr"/>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -2407,12 +2413,12 @@
       <c r="P22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>simplify:6bc3983c-65aa-4d29-9a3b-a08c3230a75a</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -2422,7 +2428,7 @@
           <t>Machine Learning Engineer Intern - E-Commerce Knowledge Graph - Computer Vision/Multimodal/Natural Language Processing</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>ByteDance</t>
         </is>
@@ -2432,7 +2438,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F23" s="14" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -2447,7 +2453,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I23" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -2484,12 +2490,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P23" s="7" t="inlineStr"/>
+      <c r="O23" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P23" s="14" t="inlineStr"/>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -2577,12 +2583,12 @@
       <c r="P24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>simplify:0d8819e9-06a6-4bf6-9c18-a00012e17263</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -2592,7 +2598,7 @@
           <t>Full Stack Software Engineer Intern</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>Rippling</t>
         </is>
@@ -2602,7 +2608,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>Seattle, WA; SF; NYC</t>
         </is>
@@ -2617,7 +2623,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I25" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -2654,12 +2660,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O25" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P25" s="7" t="inlineStr"/>
+      <c r="O25" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P25" s="14" t="inlineStr"/>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2747,12 +2753,12 @@
       <c r="P26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="60" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>simplify:3fa70c31-5b5a-41e7-8aa4-3e415e17364f</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -2762,7 +2768,7 @@
           <t>Data Science Intern</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>iSpot.tv</t>
         </is>
@@ -2772,7 +2778,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>Bellevue, WA</t>
         </is>
@@ -2787,7 +2793,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I27" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -2824,12 +2830,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O27" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P27" s="7" t="inlineStr"/>
+      <c r="O27" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P27" s="14" t="inlineStr"/>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2917,12 +2923,12 @@
       <c r="P28" s="2" t="inlineStr"/>
     </row>
     <row r="29" ht="60" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>simplify:94896995-4fb6-4ac7-8f06-5ef16ac5ad82</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -2932,7 +2938,7 @@
           <t>Data Scientist Intern</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
@@ -2942,7 +2948,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>Seattle, WA</t>
         </is>
@@ -2957,7 +2963,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I29" s="7" t="inlineStr">
+      <c r="I29" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -2994,12 +3000,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O29" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P29" s="7" t="inlineStr"/>
+      <c r="O29" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P29" s="14" t="inlineStr"/>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -3087,12 +3093,12 @@
       <c r="P30" s="2" t="inlineStr"/>
     </row>
     <row r="31" ht="60" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>simplify:fe77f108-84fc-48fd-bc64-dfd8921d203f</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -3102,7 +3108,7 @@
           <t>Forward Deployed Software Engineer Intern - Defense Tech</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="14" t="inlineStr">
         <is>
           <t>Palantir</t>
         </is>
@@ -3112,7 +3118,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="F31" s="14" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -3127,7 +3133,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
+      <c r="I31" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -3164,12 +3170,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O31" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P31" s="7" t="inlineStr"/>
+      <c r="O31" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P31" s="14" t="inlineStr"/>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -3257,12 +3263,12 @@
       <c r="P32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="60" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>simplify:36e30f4d-f208-49e7-b220-df4872f5af7b</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -3272,7 +3278,7 @@
           <t>Software Development Intern</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>iHerb</t>
         </is>
@@ -3282,7 +3288,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>Remote in USA</t>
         </is>
@@ -3297,7 +3303,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="I33" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -3334,12 +3340,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O33" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P33" s="7" t="inlineStr"/>
+      <c r="O33" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P33" s="14" t="inlineStr"/>
     </row>
     <row r="34" ht="60" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -3423,12 +3429,12 @@
       <c r="P34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="60" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>simplify:3b16aba4-17cf-4636-b0fa-03bc53122db2</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -3438,13 +3444,13 @@
           <t>Full Stack Developer Intern</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>VetsEZ</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr"/>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr"/>
+      <c r="F35" s="14" t="inlineStr">
         <is>
           <t>Remote in US</t>
         </is>
@@ -3459,7 +3465,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I35" s="7" t="inlineStr">
+      <c r="I35" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -3496,12 +3502,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O35" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P35" s="7" t="inlineStr"/>
+      <c r="O35" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P35" s="14" t="inlineStr"/>
     </row>
     <row r="36" ht="60" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -3589,12 +3595,12 @@
       <c r="P36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>simplify:4a30dd71-73a0-48c8-9e4a-9422a6952920</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -3604,7 +3610,7 @@
           <t>Software Engineer Intern - Defense Tech</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="14" t="inlineStr">
         <is>
           <t>Palantir</t>
         </is>
@@ -3614,7 +3620,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="F37" s="14" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -3629,7 +3635,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="I37" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -3666,12 +3672,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O37" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P37" s="7" t="inlineStr"/>
+      <c r="O37" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P37" s="14" t="inlineStr"/>
     </row>
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -3759,12 +3765,12 @@
       <c r="P38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="60" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>simplify:2c1046a7-cf40-410a-bf96-843e6e4db629</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -3774,7 +3780,7 @@
           <t>Software Engineer Intern - Production Infrastructure</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D39" s="14" t="inlineStr">
         <is>
           <t>Palantir</t>
         </is>
@@ -3784,7 +3790,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F39" s="14" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -3799,7 +3805,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="I39" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -3836,12 +3842,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O39" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P39" s="7" t="inlineStr"/>
+      <c r="O39" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P39" s="14" t="inlineStr"/>
     </row>
     <row r="40" ht="60" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -3929,12 +3935,12 @@
       <c r="P40" s="2" t="inlineStr"/>
     </row>
     <row r="41" ht="60" customHeight="1">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>simplify:a6f6dea0-a60c-411e-b4f6-09d69755164b</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -3944,7 +3950,7 @@
           <t>Data Analyst Intern</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="14" t="inlineStr">
         <is>
           <t>ConnectPrep</t>
         </is>
@@ -3954,7 +3960,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="F41" s="14" t="inlineStr">
         <is>
           <t>Washington, DC; Remote in USA</t>
         </is>
@@ -3969,7 +3975,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I41" s="7" t="inlineStr">
+      <c r="I41" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -4006,12 +4012,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O41" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P41" s="7" t="inlineStr"/>
+      <c r="O41" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P41" s="14" t="inlineStr"/>
     </row>
     <row r="42" ht="60" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -4099,12 +4105,12 @@
       <c r="P42" s="2" t="inlineStr"/>
     </row>
     <row r="43" ht="60" customHeight="1">
-      <c r="A43" s="7" t="inlineStr">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>simplify:28286b52-4c99-4d00-a870-d919c13d68c6</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -4114,7 +4120,7 @@
           <t>Software Engineer Intern</t>
         </is>
       </c>
-      <c r="D43" s="7" t="inlineStr">
+      <c r="D43" s="14" t="inlineStr">
         <is>
           <t>Citadel</t>
         </is>
@@ -4124,7 +4130,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
+      <c r="F43" s="14" t="inlineStr">
         <is>
           <t>Greenwich, CT; Houston, TX; Miami, FL; NYC</t>
         </is>
@@ -4139,7 +4145,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I43" s="7" t="inlineStr">
+      <c r="I43" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -4176,12 +4182,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O43" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P43" s="7" t="inlineStr"/>
+      <c r="O43" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P43" s="14" t="inlineStr"/>
     </row>
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -4269,12 +4275,12 @@
       <c r="P44" s="2" t="inlineStr"/>
     </row>
     <row r="45" ht="60" customHeight="1">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>simplify:1f3b2933-fe37-4e8a-b727-eb9166e6df99</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -4284,7 +4290,7 @@
           <t>Appian Intern</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>Horizon Industries</t>
         </is>
@@ -4294,7 +4300,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F45" s="14" t="inlineStr">
         <is>
           <t>Washington, DC</t>
         </is>
@@ -4309,7 +4315,7 @@
           <t>Strong Fit</t>
         </is>
       </c>
-      <c r="I45" s="7" t="inlineStr">
+      <c r="I45" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -4346,12 +4352,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O45" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P45" s="7" t="inlineStr"/>
+      <c r="O45" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P45" s="14" t="inlineStr"/>
     </row>
     <row r="46" ht="60" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -4439,12 +4445,12 @@
       <c r="P46" s="2" t="inlineStr"/>
     </row>
     <row r="47" ht="60" customHeight="1">
-      <c r="A47" s="7" t="inlineStr">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>simplify:fe925a08-6009-425a-b112-6e80d0c715d0</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -4454,7 +4460,7 @@
           <t>Uptime Management Center Intern</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D47" s="14" t="inlineStr">
         <is>
           <t>EquipmentShare</t>
         </is>
@@ -4464,7 +4470,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F47" s="14" t="inlineStr">
         <is>
           <t>Columbia, MO</t>
         </is>
@@ -4479,7 +4485,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I47" s="7" t="inlineStr">
+      <c r="I47" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -4516,12 +4522,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O47" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P47" s="7" t="inlineStr"/>
+      <c r="O47" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P47" s="14" t="inlineStr"/>
     </row>
     <row r="48" ht="60" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -4609,12 +4615,12 @@
       <c r="P48" s="2" t="inlineStr"/>
     </row>
     <row r="49" ht="60" customHeight="1">
-      <c r="A49" s="7" t="inlineStr">
+      <c r="A49" s="14" t="inlineStr">
         <is>
           <t>simplify:268262ab-3056-48bd-a78d-3fe70d2fb886</t>
         </is>
       </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="B49" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -4624,7 +4630,7 @@
           <t>AI Transformation / Forward Deployed Engineer Intern - Forward Deployed Engineer</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="14" t="inlineStr">
         <is>
           <t>Datasite</t>
         </is>
@@ -4634,7 +4640,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
+      <c r="F49" s="14" t="inlineStr">
         <is>
           <t>NYC</t>
         </is>
@@ -4649,7 +4655,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I49" s="7" t="inlineStr">
+      <c r="I49" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -4686,12 +4692,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O49" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P49" s="7" t="inlineStr"/>
+      <c r="O49" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P49" s="14" t="inlineStr"/>
     </row>
     <row r="50" ht="60" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -4779,12 +4785,12 @@
       <c r="P50" s="2" t="inlineStr"/>
     </row>
     <row r="51" ht="60" customHeight="1">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>simplify:8990370a-d091-498f-98bb-082a18262cfa</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -4794,7 +4800,7 @@
           <t>Data Engineering Intern</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="14" t="inlineStr">
         <is>
           <t>Hone Health</t>
         </is>
@@ -4804,7 +4810,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
+      <c r="F51" s="14" t="inlineStr">
         <is>
           <t>Remote in USA</t>
         </is>
@@ -4819,7 +4825,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I51" s="7" t="inlineStr">
+      <c r="I51" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -4856,12 +4862,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O51" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P51" s="7" t="inlineStr"/>
+      <c r="O51" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P51" s="14" t="inlineStr"/>
     </row>
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
@@ -4949,12 +4955,12 @@
       <c r="P52" s="2" t="inlineStr"/>
     </row>
     <row r="53" ht="60" customHeight="1">
-      <c r="A53" s="7" t="inlineStr">
+      <c r="A53" s="14" t="inlineStr">
         <is>
           <t>simplify:51146492-0c25-4e83-b0f2-9bd98505db21</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -4964,7 +4970,7 @@
           <t>Data Scientist Intern</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="14" t="inlineStr">
         <is>
           <t>Uber Freight</t>
         </is>
@@ -4974,7 +4980,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
+      <c r="F53" s="14" t="inlineStr">
         <is>
           <t>Chicago, IL</t>
         </is>
@@ -4989,7 +4995,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I53" s="7" t="inlineStr">
+      <c r="I53" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -5026,12 +5032,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O53" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P53" s="7" t="inlineStr"/>
+      <c r="O53" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P53" s="14" t="inlineStr"/>
     </row>
     <row r="54" ht="60" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -5119,12 +5125,12 @@
       <c r="P54" s="2" t="inlineStr"/>
     </row>
     <row r="55" ht="60" customHeight="1">
-      <c r="A55" s="7" t="inlineStr">
+      <c r="A55" s="14" t="inlineStr">
         <is>
           <t>simplify:f0aadc2c-2a47-404c-bc18-f3863ab3e456</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -5134,7 +5140,7 @@
           <t>Software Engineer Intern</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="14" t="inlineStr">
         <is>
           <t>Pylon</t>
         </is>
@@ -5144,7 +5150,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
+      <c r="F55" s="14" t="inlineStr">
         <is>
           <t>SF</t>
         </is>
@@ -5159,7 +5165,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I55" s="7" t="inlineStr">
+      <c r="I55" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -5196,12 +5202,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O55" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P55" s="7" t="inlineStr"/>
+      <c r="O55" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P55" s="14" t="inlineStr"/>
     </row>
     <row r="56" ht="60" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -5289,12 +5295,12 @@
       <c r="P56" s="2" t="inlineStr"/>
     </row>
     <row r="57" ht="60" customHeight="1">
-      <c r="A57" s="7" t="inlineStr">
+      <c r="A57" s="14" t="inlineStr">
         <is>
           <t>simplify:f5df0ff3-923c-48b4-abf3-9c10848eb7ed</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -5304,7 +5310,7 @@
           <t>Software Engineer Intern - Energy Engineering</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>Tesla</t>
         </is>
@@ -5314,7 +5320,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
+      <c r="F57" s="14" t="inlineStr">
         <is>
           <t>Palo Alto, CA</t>
         </is>
@@ -5329,7 +5335,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I57" s="7" t="inlineStr">
+      <c r="I57" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -5366,12 +5372,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O57" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P57" s="7" t="inlineStr"/>
+      <c r="O57" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P57" s="14" t="inlineStr"/>
     </row>
     <row r="58" ht="60" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
@@ -5459,12 +5465,12 @@
       <c r="P58" s="2" t="inlineStr"/>
     </row>
     <row r="59" ht="60" customHeight="1">
-      <c r="A59" s="7" t="inlineStr">
+      <c r="A59" s="14" t="inlineStr">
         <is>
           <t>simplify:03e2c12e-866f-454c-b240-466b9ae8ed18</t>
         </is>
       </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="B59" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -5474,7 +5480,7 @@
           <t>Undergraduate Intern</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D59" s="14" t="inlineStr">
         <is>
           <t>Fidelity Investments</t>
         </is>
@@ -5484,7 +5490,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F59" s="7" t="inlineStr">
+      <c r="F59" s="14" t="inlineStr">
         <is>
           <t>Westlake, TX</t>
         </is>
@@ -5499,7 +5505,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I59" s="7" t="inlineStr">
+      <c r="I59" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -5536,12 +5542,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O59" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P59" s="7" t="inlineStr"/>
+      <c r="O59" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P59" s="14" t="inlineStr"/>
     </row>
     <row r="60" ht="60" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -5629,12 +5635,12 @@
       <c r="P60" s="2" t="inlineStr"/>
     </row>
     <row r="61" ht="60" customHeight="1">
-      <c r="A61" s="7" t="inlineStr">
+      <c r="A61" s="14" t="inlineStr">
         <is>
           <t>uw:post-615259</t>
         </is>
       </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -5644,13 +5650,13 @@
           <t>UX Design Intern</t>
         </is>
       </c>
-      <c r="D61" s="7" t="inlineStr">
+      <c r="D61" s="14" t="inlineStr">
         <is>
           <t>YIRENTAL</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr"/>
-      <c r="F61" s="7" t="inlineStr">
+      <c r="E61" s="14" t="inlineStr"/>
+      <c r="F61" s="14" t="inlineStr">
         <is>
           <t>Washington</t>
         </is>
@@ -5665,7 +5671,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I61" s="7" t="inlineStr">
+      <c r="I61" s="14" t="inlineStr">
         <is>
           <t>Uw</t>
         </is>
@@ -5702,12 +5708,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O61" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P61" s="7" t="inlineStr"/>
+      <c r="O61" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P61" s="14" t="inlineStr"/>
     </row>
     <row r="62" ht="60" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
@@ -5791,12 +5797,12 @@
       <c r="P62" s="2" t="inlineStr"/>
     </row>
     <row r="63" ht="60" customHeight="1">
-      <c r="A63" s="7" t="inlineStr">
+      <c r="A63" s="14" t="inlineStr">
         <is>
           <t>uw:post-612599</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -5806,13 +5812,13 @@
           <t>IT Support Intern Helpdesk &amp; End User Support</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
+      <c r="D63" s="14" t="inlineStr">
         <is>
           <t>Trimlite</t>
         </is>
       </c>
-      <c r="E63" s="7" t="inlineStr"/>
-      <c r="F63" s="7" t="inlineStr">
+      <c r="E63" s="14" t="inlineStr"/>
+      <c r="F63" s="14" t="inlineStr">
         <is>
           <t>Washington</t>
         </is>
@@ -5827,7 +5833,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I63" s="7" t="inlineStr">
+      <c r="I63" s="14" t="inlineStr">
         <is>
           <t>Uw</t>
         </is>
@@ -5864,12 +5870,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O63" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P63" s="7" t="inlineStr"/>
+      <c r="O63" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P63" s="14" t="inlineStr"/>
     </row>
     <row r="64" ht="60" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -6033,8 +6039,1028 @@
       </c>
       <c r="P65" s="14" t="inlineStr"/>
     </row>
+    <row r="66" ht="60" customHeight="1">
+      <c r="A66" s="15" t="inlineStr">
+        <is>
+          <t>simplify:30a79016-bc6f-4525-a5fe-a459b18de455</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern - C++</t>
+        </is>
+      </c>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>Akuna Capital University</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F66" s="15" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>63%</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I66" s="15" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Skills: rest, api, full stack, backend, frontend, c++, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L66" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M66" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Akuna Capital University is hiring for Software Engineer Intern - C++. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N66" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer Intern - C++ role at Akuna Capital University
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer Intern - C++ opening at Akuna Capital University and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O66" s="15" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P66" s="15" t="inlineStr"/>
+    </row>
+    <row r="67" ht="60" customHeight="1">
+      <c r="A67" s="16" t="inlineStr">
+        <is>
+          <t>simplify:bc91fbea-a1d8-4e14-8446-6d0df9d7a3f3</t>
+        </is>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>Quantitative Development &amp; Strategy Intern</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Akuna Capital University</t>
+        </is>
+      </c>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I67" s="16" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J67" s="8" t="inlineStr">
+        <is>
+          <t>Skills: rest, api, full stack, backend, frontend, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K67" s="9" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L67" s="9" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M67" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Akuna Capital University is hiring for Quantitative Development &amp; Strategy Intern. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N67" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Quantitative Development &amp; Strategy Intern role at Akuna Capital University
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Quantitative Development &amp; Strategy Intern opening at Akuna Capital University and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O67" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P67" s="16" t="inlineStr"/>
+    </row>
+    <row r="68" ht="60" customHeight="1">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>simplify:18e99160-24c6-4a84-bc61-bec64dd7decb</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern - Full Stack Web</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>Akuna Capital University</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F68" s="15" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I68" s="15" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Skills: rest, api, full stack, backend, frontend, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L68" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Akuna Capital University is hiring for Software Engineer Intern - Full Stack Web. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N68" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer Intern - Full Stack Web role at Akuna Capital University
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer Intern - Full Stack Web opening at Akuna Capital University and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O68" s="15" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P68" s="15" t="inlineStr"/>
+    </row>
+    <row r="69" ht="60" customHeight="1">
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>simplify:13b103af-8b5c-4685-9b00-18ce29399f40</t>
+        </is>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern - Python</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Akuna Capital University</t>
+        </is>
+      </c>
+      <c r="E69" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>63%</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I69" s="16" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J69" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, rest, api, full stack, backend, frontend, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K69" s="9" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L69" s="9" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M69" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Akuna Capital University is hiring for Software Engineer Intern - Python. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N69" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer Intern - Python role at Akuna Capital University
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer Intern - Python opening at Akuna Capital University and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O69" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P69" s="16" t="inlineStr"/>
+    </row>
+    <row r="70" ht="60" customHeight="1">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>simplify:d1bb038f-04a0-4995-9bcc-ff779f3a2054</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Software Developer Intern</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>DRW</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F70" s="15" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I70" s="15" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>Skills: rest, api, full stack, backend, frontend, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L70" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw DRW is hiring for Software Developer Intern. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N70" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Developer Intern role at DRW
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Developer Intern opening at DRW and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O70" s="15" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P70" s="15" t="inlineStr"/>
+    </row>
+    <row r="71" ht="60" customHeight="1">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>simplify:87235779-9531-4bf2-b265-6cc448aa0f35</t>
+        </is>
+      </c>
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern - C++ or Python</t>
+        </is>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>Hudson River Trading</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>Austin, TX; Chicago, IL; NYC</t>
+        </is>
+      </c>
+      <c r="G71" s="10" t="inlineStr">
+        <is>
+          <t>66%</t>
+        </is>
+      </c>
+      <c r="H71" s="11" t="inlineStr">
+        <is>
+          <t>Good Fit</t>
+        </is>
+      </c>
+      <c r="I71" s="16" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J71" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, rest, api, full stack, backend, frontend, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K71" s="9" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L71" s="9" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M71" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Hudson River Trading is hiring for Software Engineer Intern - C++ or Python. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N71" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer Intern - C++ or Python role at Hudson River Trading
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer Intern - C++ or Python opening at Hudson River Trading and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O71" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P71" s="16" t="inlineStr"/>
+    </row>
+    <row r="72" ht="60" customHeight="1">
+      <c r="A72" s="15" t="inlineStr">
+        <is>
+          <t>simplify:df655811-97ff-42e6-951f-e7e0a02c6beb</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>AI Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>Nextiva</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>Scottsdale, AZ</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I72" s="15" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>Skills: python, machine learning, data analysis, artificial intelligence, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L72" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M72" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Nextiva is hiring for AI Engineer Intern. I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N72" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the AI Engineer Intern role at Nextiva
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the AI Engineer Intern opening at Nextiva and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O72" s="15" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P72" s="15" t="inlineStr"/>
+    </row>
+    <row r="73" ht="60" customHeight="1">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>simplify:1c39cba6-ebfc-4c07-b06a-3ab376302145</t>
+        </is>
+      </c>
+      <c r="B73" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>Energy Data Analysis Intern</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>National Laboratory of the Rockies</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
+        <is>
+          <t>Golden, CO</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I73" s="16" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J73" s="8" t="inlineStr">
+        <is>
+          <t>Skills: python, machine learning, data analysis, artificial intelligence, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K73" s="9" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L73" s="9" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M73" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw National Laboratory of the Rockies is hiring for Energy Data Analysis Intern. I recently built APEX, an ML-driven trading signal system with a self-retraining model — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N73" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Energy Data Analysis Intern role at National Laboratory of the Rockies
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Energy Data Analysis Intern opening at National Laboratory of the Rockies and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+Most recently I built APEX, a full-stack system that combines a technical-analysis signal engine with a RandomForest model that retrains itself on live trading outcomes — deployed end-to-end on AWS.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O73" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P73" s="16" t="inlineStr"/>
+    </row>
+    <row r="74" ht="60" customHeight="1">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>simplify:45903a19-328a-4e71-802e-c33fbc45d459</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Associate Product Manager Intern - Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I74" s="15" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>Skills: data analytics, business analyst, product management, product manager, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K74" s="4" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L74" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M74" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Salesforce is hiring for Associate Product Manager Intern - Associate Product Manager. I've built a couple of data-heavy projects, including an automated stock signal analyzer — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N74" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Associate Product Manager Intern - Associate Product Manager role at Salesforce
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Associate Product Manager Intern - Associate Product Manager opening at Salesforce and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've built a couple of data-focused projects — an automated stock analysis tool applying technical indicators to live market data, and an interactive trail-mapping app processing 200+ real-world datasets with Pandas.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O74" s="15" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P74" s="15" t="inlineStr"/>
+    </row>
+    <row r="75" ht="60" customHeight="1">
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t>simplify:224ca026-078b-4524-bf33-5a214373c094</t>
+        </is>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Associate Product Manager Intern - Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>57%</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I75" s="16" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J75" s="8" t="inlineStr">
+        <is>
+          <t>Skills: data analytics, business analyst, product management, product manager, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K75" s="9" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L75" s="9" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M75" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Salesforce is hiring for Associate Product Manager Intern - Associate Product Manager. I've built a couple of data-heavy projects, including an automated stock signal analyzer — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N75" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Associate Product Manager Intern - Associate Product Manager role at Salesforce
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Associate Product Manager Intern - Associate Product Manager opening at Salesforce and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've built a couple of data-focused projects — an automated stock analysis tool applying technical indicators to live market data, and an interactive trail-mapping app processing 200+ real-world datasets with Pandas.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O75" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P75" s="16" t="inlineStr"/>
+    </row>
+    <row r="76" ht="60" customHeight="1">
+      <c r="A76" s="15" t="inlineStr">
+        <is>
+          <t>simplify:12c71417-7d4c-4820-a1dc-e69c433eb686</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Teleoperation Software Engineering Internship</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>Persona AI</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>Houston, TX; Pensacola, FL</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I76" s="15" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>Skills: rest, api, full stack, backend, frontend, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L76" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M76" s="3" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Persona AI is hiring for Teleoperation Software Engineering Internship. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N76" s="3" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Teleoperation Software Engineering Internship role at Persona AI
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Teleoperation Software Engineering Internship opening at Persona AI and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O76" s="15" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P76" s="15" t="inlineStr"/>
+    </row>
+    <row r="77" ht="60" customHeight="1">
+      <c r="A77" s="16" t="inlineStr">
+        <is>
+          <t>simplify:17b55e16-4b9d-4870-ba60-51a53eaf71c5</t>
+        </is>
+      </c>
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Software Engineer Intern - C# .NET Desktop</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>Akuna Capital University</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="inlineStr">
+        <is>
+          <t>Website →</t>
+        </is>
+      </c>
+      <c r="F77" s="16" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>Possible Fit</t>
+        </is>
+      </c>
+      <c r="I77" s="16" t="inlineStr">
+        <is>
+          <t>Simplify</t>
+        </is>
+      </c>
+      <c r="J77" s="8" t="inlineStr">
+        <is>
+          <t>Skills: rest, api, full stack, backend, frontend, Internship title, Posted &lt;7d ago</t>
+        </is>
+      </c>
+      <c r="K77" s="9" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+      <c r="L77" s="9" t="inlineStr">
+        <is>
+          <t>LinkedIn Search →</t>
+        </is>
+      </c>
+      <c r="M77" s="8" t="inlineStr">
+        <is>
+          <t>Hi! I'm a CS student at Washington State University and saw Akuna Capital University is hiring for Software Engineer Intern - C# .NET Desktop. I've shipped a few full-stack apps (Flask/React, deployed on AWS) including an AI travel planner — would love to connect and hear more about the team.</t>
+        </is>
+      </c>
+      <c r="N77" s="8" t="inlineStr">
+        <is>
+          <t>Subject: Interested in the Software Engineer Intern - C# .NET Desktop role at Akuna Capital University
+Hi,
+My name is Giri Vignesh, and I'm a Computer Science student at Washington State University (graduating May 2027). I came across the Software Engineer Intern - C# .NET Desktop opening at Akuna Capital University and wanted to reach out directly — I'm genuinely interested in the role and think my background lines up well.
+I've shipped several full-stack projects — including TravelBuddy, an AI-powered travel planner with a Flask backend and React frontend deployed on AWS, and a hackathon project integrating the Anthropic Claude API built in 24 hours.
+I'd love to learn more about the team and what you're looking for — happy to send my resume or hop on a quick call if you're open to it.
+Thanks so much for your time,
+Giri Vignesh
+(425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
+        </is>
+      </c>
+      <c r="O77" s="16" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P77" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P65"/>
+  <autoFilter ref="A1:P77"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId2"/>
@@ -6219,6 +7245,42 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId181"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId182"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L73" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L74" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L75" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L76" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L77" r:id="rId219"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6419,12 +7481,12 @@
       <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>ashby:notion:85947779-6b87-466a-98bc-30a640448c28</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -6434,7 +7496,7 @@
           <t>Software Engineer, Early Career (AI)</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
@@ -6444,7 +7506,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="14" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -6459,7 +7521,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -6496,12 +7558,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P3" s="7" t="inlineStr"/>
+      <c r="O3" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P3" s="14" t="inlineStr"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -6883,12 +7945,12 @@
       <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>ashby:notion:a6311f97-4850-4674-a5f3-d9fe5f6f2555</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -6898,7 +7960,7 @@
           <t>Software Engineer, New Grad</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
@@ -6908,7 +7970,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="14" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -6923,7 +7985,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -6960,12 +8022,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P3" s="7" t="inlineStr"/>
+      <c r="O3" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P3" s="14" t="inlineStr"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -7053,12 +8115,12 @@
       <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>ashby:notion:85947779-6b87-466a-98bc-30a640448c28</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -7068,7 +8130,7 @@
           <t>Software Engineer, Early Career (AI)</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Notion</t>
         </is>
@@ -7078,7 +8140,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>San Francisco, California (Remote)</t>
         </is>
@@ -7093,7 +8155,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>Ashby</t>
         </is>
@@ -7130,12 +8192,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O5" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P5" s="7" t="inlineStr"/>
+      <c r="O5" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P5" s="14" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -7223,12 +8285,12 @@
       <c r="P6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>gh:scaleai:4703343005</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -7238,7 +8300,7 @@
           <t>AI Builder Intern</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Scale AI</t>
         </is>
@@ -7248,7 +8310,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>San Francisco, CA; New York, NY</t>
         </is>
@@ -7263,7 +8325,7 @@
           <t>Good Fit</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="14" t="inlineStr">
         <is>
           <t>Gh</t>
         </is>
@@ -7300,12 +8362,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P7" s="7" t="inlineStr"/>
+      <c r="O7" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P7" s="14" t="inlineStr"/>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -7393,12 +8455,12 @@
       <c r="P8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>simplify:c0a71d19-4941-44c1-9408-7c39f29dfb85</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
@@ -7408,7 +8470,7 @@
           <t>Software Engineer Intern - Agent Platform - AI</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Exowatt</t>
         </is>
@@ -7418,7 +8480,7 @@
           <t>Website →</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
@@ -7433,7 +8495,7 @@
           <t>Possible Fit</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>Simplify</t>
         </is>
@@ -7470,12 +8532,12 @@
 (425) 362-2938 | girivignesh5@gmail.com | github.com/gvignesh286</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr">
-        <is>
-          <t>Not Applied</t>
-        </is>
-      </c>
-      <c r="P9" s="7" t="inlineStr"/>
+      <c r="O9" s="14" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="P9" s="14" t="inlineStr"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">

</xml_diff>